<commit_message>
Implantación sistema salud + poder + escalado UI
</commit_message>
<xml_diff>
--- a/public/resources/cartas.xlsx
+++ b/public/resources/cartas.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FAC5932-C31F-4B15-9901-C3B4A7AAFD8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EE1870F-4241-43AD-B147-C8D28C003057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="297">
   <si>
     <t>Nombre</t>
   </si>
@@ -830,6 +830,87 @@
   </si>
   <si>
     <t>La Bat-Familia;Aves de Presa</t>
+  </si>
+  <si>
+    <t>skill_class</t>
+  </si>
+  <si>
+    <t>skill_name</t>
+  </si>
+  <si>
+    <t>skill_info</t>
+  </si>
+  <si>
+    <t>skill_power</t>
+  </si>
+  <si>
+    <t>buff</t>
+  </si>
+  <si>
+    <t>debuff</t>
+  </si>
+  <si>
+    <t>heal</t>
+  </si>
+  <si>
+    <t>revive</t>
+  </si>
+  <si>
+    <t>shield</t>
+  </si>
+  <si>
+    <t>skill_trigger</t>
+  </si>
+  <si>
+    <t>Poder+</t>
+  </si>
+  <si>
+    <t>Poder-</t>
+  </si>
+  <si>
+    <t>Curar+</t>
+  </si>
+  <si>
+    <t>Revivir</t>
+  </si>
+  <si>
+    <t>Escudo</t>
+  </si>
+  <si>
+    <t>Aumenta el poder de todos las cartas aliadas en juego.</t>
+  </si>
+  <si>
+    <t>Reduce el poder de todas las cartas enemigas en juego.</t>
+  </si>
+  <si>
+    <t>Cura 500 puntos de salud una carta aliada</t>
+  </si>
+  <si>
+    <t>Revive una carta de tu elección del cementerio y la devuelve al mazo.</t>
+  </si>
+  <si>
+    <t>Aplica un escudo en esta carta, o en una carta aliada.</t>
+  </si>
+  <si>
+    <t>auto</t>
+  </si>
+  <si>
+    <t>usar</t>
+  </si>
+  <si>
+    <t>aoe</t>
+  </si>
+  <si>
+    <t>poder/2</t>
+  </si>
+  <si>
+    <t>Ataque múltiple</t>
+  </si>
+  <si>
+    <t>Ataca a todas las cartas enemigas enemigos de forma simultanea.</t>
+  </si>
+  <si>
+    <t>Salud</t>
   </si>
 </sst>
 </file>
@@ -920,7 +1001,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -951,6 +1032,7 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1232,20 +1314,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:N111"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="2" max="2" width="6.85546875" customWidth="1"/>
-    <col min="3" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="105.85546875" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" customWidth="1"/>
-    <col min="7" max="7" width="42.42578125" customWidth="1"/>
-    <col min="8" max="8" width="71.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="38.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="105.85546875" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" customWidth="1"/>
+    <col min="8" max="8" width="42.42578125" customWidth="1"/>
+    <col min="9" max="9" width="71.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="63.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" customWidth="1"/>
+    <col min="13" max="13" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1253,29 +1339,43 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="I1" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J1" s="11" t="s">
+        <v>271</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>272</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>270</v>
+      </c>
+      <c r="M1" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="N1" s="12" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -1283,22 +1383,40 @@
         <v>1</v>
       </c>
       <c r="C2" s="3">
+        <v>6000</v>
+      </c>
+      <c r="D2" s="3">
         <v>5000</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G2" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="10" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J2" t="s">
+        <v>280</v>
+      </c>
+      <c r="K2" t="s">
+        <v>285</v>
+      </c>
+      <c r="L2" t="s">
+        <v>274</v>
+      </c>
+      <c r="M2">
+        <v>500</v>
+      </c>
+      <c r="N2" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
@@ -1306,22 +1424,40 @@
         <v>1</v>
       </c>
       <c r="C3" s="3">
-        <v>4500</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="6" t="s">
+        <v>5500</v>
+      </c>
+      <c r="D3" s="3">
+        <v>4500</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G3" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="10" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J3" t="s">
+        <v>281</v>
+      </c>
+      <c r="K3" t="s">
+        <v>286</v>
+      </c>
+      <c r="L3" t="s">
+        <v>275</v>
+      </c>
+      <c r="M3">
+        <v>500</v>
+      </c>
+      <c r="N3" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -1329,22 +1465,40 @@
         <v>1</v>
       </c>
       <c r="C4" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D4" s="3">
         <v>4000</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" s="10" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J4" t="s">
+        <v>282</v>
+      </c>
+      <c r="K4" t="s">
+        <v>287</v>
+      </c>
+      <c r="L4" t="s">
+        <v>276</v>
+      </c>
+      <c r="M4">
+        <v>500</v>
+      </c>
+      <c r="N4" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>18</v>
       </c>
@@ -1352,22 +1506,40 @@
         <v>1</v>
       </c>
       <c r="C5" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D5" s="3" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D5" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G5" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" s="10" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J5" t="s">
+        <v>283</v>
+      </c>
+      <c r="K5" t="s">
+        <v>288</v>
+      </c>
+      <c r="L5" t="s">
+        <v>277</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="N5" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>22</v>
       </c>
@@ -1375,22 +1547,40 @@
         <v>1</v>
       </c>
       <c r="C6" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D6" s="3">
         <v>4000</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G6" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="10" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J6" t="s">
+        <v>284</v>
+      </c>
+      <c r="K6" t="s">
+        <v>289</v>
+      </c>
+      <c r="L6" t="s">
+        <v>278</v>
+      </c>
+      <c r="M6">
+        <v>1000</v>
+      </c>
+      <c r="N6" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>26</v>
       </c>
@@ -1398,22 +1588,40 @@
         <v>1</v>
       </c>
       <c r="C7" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D7" s="3">
         <v>4000</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G7" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" s="10" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J7" t="s">
+        <v>294</v>
+      </c>
+      <c r="K7" t="s">
+        <v>295</v>
+      </c>
+      <c r="L7" t="s">
+        <v>292</v>
+      </c>
+      <c r="M7" t="s">
+        <v>293</v>
+      </c>
+      <c r="N7" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
@@ -1421,22 +1629,25 @@
         <v>1</v>
       </c>
       <c r="C8" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D8" s="3" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D8" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G8" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>32</v>
       </c>
@@ -1444,22 +1655,25 @@
         <v>1</v>
       </c>
       <c r="C9" s="3">
-        <v>4500</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="6" t="s">
+        <v>5500</v>
+      </c>
+      <c r="D9" s="3">
+        <v>4500</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G9" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H9" s="10" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>34</v>
       </c>
@@ -1467,25 +1681,28 @@
         <v>1</v>
       </c>
       <c r="C10" s="3">
-        <v>4500</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="6" t="s">
+        <v>5500</v>
+      </c>
+      <c r="D10" s="3">
+        <v>4500</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F10" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G10" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H10" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>37</v>
       </c>
@@ -1493,20 +1710,23 @@
         <v>1</v>
       </c>
       <c r="C11" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D11" s="3">
         <v>3000</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G11" s="10"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="G11" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11" s="10"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>39</v>
       </c>
@@ -1514,22 +1734,25 @@
         <v>1</v>
       </c>
       <c r="C12" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D12" s="3">
         <v>3000</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G12" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12" s="10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>42</v>
       </c>
@@ -1537,20 +1760,23 @@
         <v>1</v>
       </c>
       <c r="C13" s="3">
-        <v>4500</v>
-      </c>
-      <c r="D13" s="3" t="s">
+        <v>5500</v>
+      </c>
+      <c r="D13" s="3">
+        <v>4500</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F13" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G13" s="10"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="G13" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13" s="10"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>44</v>
       </c>
@@ -1558,20 +1784,23 @@
         <v>1</v>
       </c>
       <c r="C14" s="3">
+        <v>3500</v>
+      </c>
+      <c r="D14" s="3">
         <v>2500</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F14" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G14" s="10"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="G14" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" s="10"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>46</v>
       </c>
@@ -1579,22 +1808,25 @@
         <v>1</v>
       </c>
       <c r="C15" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D15" s="3">
         <v>3000</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G15" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="10" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>49</v>
       </c>
@@ -1602,22 +1834,25 @@
         <v>1</v>
       </c>
       <c r="C16" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D16" s="3" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D16" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F16" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G16" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H16" s="10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>52</v>
       </c>
@@ -1625,22 +1860,25 @@
         <v>1</v>
       </c>
       <c r="C17" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D17" s="3" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D17" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F17" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G17" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H17" s="10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>54</v>
       </c>
@@ -1648,20 +1886,23 @@
         <v>1</v>
       </c>
       <c r="C18" s="3">
-        <v>4500</v>
-      </c>
-      <c r="D18" s="3" t="s">
+        <v>5500</v>
+      </c>
+      <c r="D18" s="3">
+        <v>4500</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F18" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G18" s="10"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G18" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H18" s="10"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>56</v>
       </c>
@@ -1669,20 +1910,23 @@
         <v>1</v>
       </c>
       <c r="C19" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D19" s="3">
         <v>4000</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="F19" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G19" s="10"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G19" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H19" s="10"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>58</v>
       </c>
@@ -1690,20 +1934,23 @@
         <v>1</v>
       </c>
       <c r="C20" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D20" s="3" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D20" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="F20" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F20" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G20" s="10"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G20" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H20" s="10"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>60</v>
       </c>
@@ -1711,20 +1958,23 @@
         <v>1</v>
       </c>
       <c r="C21" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D21" s="3" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D21" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E21" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F21" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G21" s="10"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G21" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H21" s="10"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>62</v>
       </c>
@@ -1732,20 +1982,23 @@
         <v>1</v>
       </c>
       <c r="C22" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D22" s="3">
         <v>3000</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E22" s="1" t="s">
+      <c r="E22" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="F22" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G22" s="10"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G22" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H22" s="10"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>64</v>
       </c>
@@ -1753,20 +2006,23 @@
         <v>1</v>
       </c>
       <c r="C23" s="3">
+        <v>3500</v>
+      </c>
+      <c r="D23" s="3">
         <v>2500</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="F23" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G23" s="10"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G23" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H23" s="10"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>66</v>
       </c>
@@ -1774,20 +2030,23 @@
         <v>1</v>
       </c>
       <c r="C24" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D24" s="3">
         <v>3000</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E24" s="1" t="s">
+      <c r="E24" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F24" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G24" s="10"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G24" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H24" s="10"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>68</v>
       </c>
@@ -1795,20 +2054,23 @@
         <v>1</v>
       </c>
       <c r="C25" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D25" s="3">
         <v>3000</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="E25" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="F25" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F25" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G25" s="10"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G25" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H25" s="10"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>70</v>
       </c>
@@ -1816,22 +2078,25 @@
         <v>1</v>
       </c>
       <c r="C26" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E26" s="1" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D26" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F26" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G26" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H26" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>72</v>
       </c>
@@ -1839,22 +2104,25 @@
         <v>1</v>
       </c>
       <c r="C27" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D27" s="3" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D27" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="F27" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F27" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G27" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H27" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>74</v>
       </c>
@@ -1862,22 +2130,25 @@
         <v>1</v>
       </c>
       <c r="C28" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D28" s="3">
         <v>3000</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="E28" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="F28" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F28" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G28" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H28" s="10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>77</v>
       </c>
@@ -1885,22 +2156,25 @@
         <v>1</v>
       </c>
       <c r="C29" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D29" s="3">
         <v>3000</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="E29" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F29" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G29" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H29" s="10" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>267</v>
       </c>
@@ -1908,22 +2182,25 @@
         <v>1</v>
       </c>
       <c r="C30" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D30" s="3">
         <v>3000</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="E30" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="F30" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="F30" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G30" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H30" s="10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>79</v>
       </c>
@@ -1931,22 +2208,25 @@
         <v>1</v>
       </c>
       <c r="C31" s="3">
+        <v>3500</v>
+      </c>
+      <c r="D31" s="3">
         <v>2500</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="E31" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="F31" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="F31" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G31" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H31" s="10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>81</v>
       </c>
@@ -1954,22 +2234,25 @@
         <v>1</v>
       </c>
       <c r="C32" s="3">
+        <v>3000</v>
+      </c>
+      <c r="D32" s="3">
         <v>2000</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="E32" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="F32" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="F32" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G32" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H32" s="10" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>84</v>
       </c>
@@ -1977,22 +2260,25 @@
         <v>1</v>
       </c>
       <c r="C33" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D33" s="3" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D33" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="F33" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="F33" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G33" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H33" s="10" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>86</v>
       </c>
@@ -2000,20 +2286,23 @@
         <v>1</v>
       </c>
       <c r="C34" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E34" s="6" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D34" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F34" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F34" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G34" s="10"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G34" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H34" s="10"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>88</v>
       </c>
@@ -2021,22 +2310,25 @@
         <v>1</v>
       </c>
       <c r="C35" s="3">
+        <v>3500</v>
+      </c>
+      <c r="D35" s="3">
         <v>2500</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="E35" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="F35" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="F35" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G35" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H35" s="10" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>90</v>
       </c>
@@ -2044,20 +2336,23 @@
         <v>1</v>
       </c>
       <c r="C36" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D36" s="3">
         <v>4000</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="E36" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="F36" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="F36" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G36" s="10"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G36" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H36" s="10"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>92</v>
       </c>
@@ -2065,22 +2360,25 @@
         <v>1</v>
       </c>
       <c r="C37" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D37" s="3">
         <v>4000</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="E37" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E37" s="6" t="s">
+      <c r="F37" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="F37" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G37" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H37" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>95</v>
       </c>
@@ -2088,22 +2386,25 @@
         <v>1</v>
       </c>
       <c r="C38" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D38" s="3">
         <v>4000</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="E38" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="F38" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="F38" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G38" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H38" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>97</v>
       </c>
@@ -2111,20 +2412,23 @@
         <v>1</v>
       </c>
       <c r="C39" s="3">
+        <v>3500</v>
+      </c>
+      <c r="D39" s="3">
         <v>2500</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="E39" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="F39" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="F39" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G39" s="10"/>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G39" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H39" s="10"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>99</v>
       </c>
@@ -2132,20 +2436,23 @@
         <v>1</v>
       </c>
       <c r="C40" s="3">
-        <v>4500</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E40" s="1" t="s">
+        <v>5500</v>
+      </c>
+      <c r="D40" s="3">
+        <v>4500</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="F40" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G40" s="10"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G40" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H40" s="10"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>101</v>
       </c>
@@ -2153,22 +2460,25 @@
         <v>1</v>
       </c>
       <c r="C41" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D41" s="3">
         <v>3000</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="E41" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="F41" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="F41" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G41" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H41" s="10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>103</v>
       </c>
@@ -2176,22 +2486,25 @@
         <v>1</v>
       </c>
       <c r="C42" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D42" s="3">
         <v>3000</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="E42" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="F42" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="F42" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G42" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H42" s="10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>105</v>
       </c>
@@ -2199,22 +2512,25 @@
         <v>1</v>
       </c>
       <c r="C43" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E43" s="1" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D43" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="F43" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G43" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H43" s="10" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>108</v>
       </c>
@@ -2222,22 +2538,25 @@
         <v>1</v>
       </c>
       <c r="C44" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E44" s="6" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D44" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F44" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="F44" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G44" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H44" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>111</v>
       </c>
@@ -2245,22 +2564,25 @@
         <v>1</v>
       </c>
       <c r="C45" s="3">
+        <v>4000</v>
+      </c>
+      <c r="D45" s="3">
         <v>3000</v>
       </c>
-      <c r="D45" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E45" s="6" t="s">
+      <c r="E45" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F45" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="F45" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G45" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H45" s="10" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>113</v>
       </c>
@@ -2268,22 +2590,25 @@
         <v>1</v>
       </c>
       <c r="C46" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E46" s="1" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D46" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F46" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G46" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H46" s="10" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>116</v>
       </c>
@@ -2291,20 +2616,23 @@
         <v>1</v>
       </c>
       <c r="C47" s="3">
-        <v>4500</v>
-      </c>
-      <c r="D47" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E47" s="1" t="s">
+        <v>5500</v>
+      </c>
+      <c r="D47" s="3">
+        <v>4500</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F47" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F47" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G47" s="10"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G47" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H47" s="10"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>118</v>
       </c>
@@ -2312,20 +2640,23 @@
         <v>1</v>
       </c>
       <c r="C48" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D48" s="3" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D48" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E48" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E48" s="1" t="s">
+      <c r="F48" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="F48" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G48" s="10"/>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G48" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H48" s="10"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>120</v>
       </c>
@@ -2333,20 +2664,23 @@
         <v>1</v>
       </c>
       <c r="C49" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D49" s="3">
         <v>4000</v>
       </c>
-      <c r="D49" s="3" t="s">
+      <c r="E49" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="F49" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="F49" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G49" s="10"/>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G49" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H49" s="10"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>122</v>
       </c>
@@ -2354,20 +2688,23 @@
         <v>1</v>
       </c>
       <c r="C50" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D50" s="3" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D50" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E50" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E50" s="1" t="s">
+      <c r="F50" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F50" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G50" s="10"/>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G50" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H50" s="10"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>124</v>
       </c>
@@ -2375,22 +2712,25 @@
         <v>1</v>
       </c>
       <c r="C51" s="3">
-        <v>4500</v>
-      </c>
-      <c r="D51" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E51" s="1" t="s">
+        <v>5500</v>
+      </c>
+      <c r="D51" s="3">
+        <v>4500</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F51" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="F51" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G51" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H51" s="10" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>127</v>
       </c>
@@ -2398,22 +2738,25 @@
         <v>1</v>
       </c>
       <c r="C52" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D52" s="3">
         <v>4000</v>
       </c>
-      <c r="D52" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E52" s="6" t="s">
+      <c r="E52" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F52" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="F52" s="10" t="s">
-        <v>10</v>
-      </c>
       <c r="G52" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H52" s="10" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>129</v>
       </c>
@@ -2421,20 +2764,23 @@
         <v>1</v>
       </c>
       <c r="C53" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E53" s="1" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D53" s="3">
+        <v>3500</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="F53" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G53" s="10"/>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G53" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H53" s="10"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>131</v>
       </c>
@@ -2442,22 +2788,25 @@
         <v>1</v>
       </c>
       <c r="C54" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D54" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D54" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E54" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E54" s="4" t="s">
+      <c r="F54" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="F54" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G54" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H54" s="4" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>135</v>
       </c>
@@ -2465,22 +2814,25 @@
         <v>1</v>
       </c>
       <c r="C55" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D55" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D55" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E55" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E55" s="4" t="s">
+      <c r="F55" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="F55" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G55" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H55" s="4" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>138</v>
       </c>
@@ -2488,22 +2840,25 @@
         <v>1</v>
       </c>
       <c r="C56" s="4">
+        <v>6000</v>
+      </c>
+      <c r="D56" s="4">
         <v>5000</v>
       </c>
-      <c r="D56" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="E56" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F56" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="F56" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G56" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H56" s="4" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
         <v>259</v>
       </c>
@@ -2511,20 +2866,23 @@
         <v>1</v>
       </c>
       <c r="C57" s="4">
+        <v>6500</v>
+      </c>
+      <c r="D57" s="4">
         <v>5500</v>
       </c>
-      <c r="D57" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="E57" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F57" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="F57" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G57" s="4"/>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G57" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H57" s="4"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
         <v>141</v>
       </c>
@@ -2532,22 +2890,25 @@
         <v>1</v>
       </c>
       <c r="C58" s="4">
-        <v>4500</v>
-      </c>
-      <c r="D58" s="4" t="s">
+        <v>5500</v>
+      </c>
+      <c r="D58" s="4">
+        <v>4500</v>
+      </c>
+      <c r="E58" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E58" s="4" t="s">
+      <c r="F58" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="F58" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G58" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H58" s="4" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>144</v>
       </c>
@@ -2555,22 +2916,25 @@
         <v>1</v>
       </c>
       <c r="C59" s="4">
-        <v>4500</v>
-      </c>
-      <c r="D59" s="4" t="s">
+        <v>5500</v>
+      </c>
+      <c r="D59" s="4">
+        <v>4500</v>
+      </c>
+      <c r="E59" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E59" s="4" t="s">
+      <c r="F59" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="F59" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G59" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H59" s="4" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>264</v>
       </c>
@@ -2578,20 +2942,23 @@
         <v>1</v>
       </c>
       <c r="C60" s="4">
-        <v>4500</v>
-      </c>
-      <c r="D60" s="4" t="s">
+        <v>5500</v>
+      </c>
+      <c r="D60" s="4">
+        <v>4500</v>
+      </c>
+      <c r="E60" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E60" s="4" t="s">
+      <c r="F60" s="4" t="s">
         <v>265</v>
       </c>
-      <c r="F60" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G60" s="4"/>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G60" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H60" s="4"/>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
         <v>261</v>
       </c>
@@ -2599,20 +2966,23 @@
         <v>1</v>
       </c>
       <c r="C61" s="4">
+        <v>6500</v>
+      </c>
+      <c r="D61" s="4">
         <v>5500</v>
       </c>
-      <c r="D61" s="4" t="s">
+      <c r="E61" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E61" s="4" t="s">
+      <c r="F61" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="F61" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G61" s="4"/>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G61" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H61" s="4"/>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>147</v>
       </c>
@@ -2620,22 +2990,25 @@
         <v>1</v>
       </c>
       <c r="C62" s="4">
+        <v>5000</v>
+      </c>
+      <c r="D62" s="4">
         <v>4000</v>
       </c>
-      <c r="D62" s="4" t="s">
+      <c r="E62" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E62" s="4" t="s">
+      <c r="F62" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="F62" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G62" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H62" s="4" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
         <v>256</v>
       </c>
@@ -2643,22 +3016,25 @@
         <v>1</v>
       </c>
       <c r="C63" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D63" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D63" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E63" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E63" s="4" t="s">
+      <c r="F63" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="F63" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G63" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H63" s="4" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
         <v>254</v>
       </c>
@@ -2666,22 +3042,25 @@
         <v>1</v>
       </c>
       <c r="C64" s="4">
+        <v>4000</v>
+      </c>
+      <c r="D64" s="4">
         <v>3000</v>
       </c>
-      <c r="D64" s="4" t="s">
+      <c r="E64" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E64" s="4" t="s">
+      <c r="F64" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="F64" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G64" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H64" s="4" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
         <v>150</v>
       </c>
@@ -2689,20 +3068,23 @@
         <v>1</v>
       </c>
       <c r="C65" s="4">
+        <v>5000</v>
+      </c>
+      <c r="D65" s="4">
         <v>4000</v>
       </c>
-      <c r="D65" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="E65" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F65" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="F65" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G65" s="4"/>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G65" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H65" s="4"/>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
         <v>152</v>
       </c>
@@ -2710,22 +3092,25 @@
         <v>1</v>
       </c>
       <c r="C66" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D66" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D66" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E66" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E66" s="4" t="s">
+      <c r="F66" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="F66" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G66" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H66" s="4" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
         <v>155</v>
       </c>
@@ -2733,22 +3118,25 @@
         <v>1</v>
       </c>
       <c r="C67" s="4">
+        <v>4000</v>
+      </c>
+      <c r="D67" s="4">
         <v>3000</v>
       </c>
-      <c r="D67" s="4" t="s">
+      <c r="E67" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E67" s="4" t="s">
+      <c r="F67" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="F67" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G67" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H67" s="4" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
         <v>158</v>
       </c>
@@ -2756,20 +3144,23 @@
         <v>1</v>
       </c>
       <c r="C68" s="4">
+        <v>3500</v>
+      </c>
+      <c r="D68" s="4">
         <v>2500</v>
       </c>
-      <c r="D68" s="4" t="s">
+      <c r="E68" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E68" s="4" t="s">
+      <c r="F68" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="F68" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G68" s="4"/>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G68" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H68" s="4"/>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
         <v>160</v>
       </c>
@@ -2777,22 +3168,25 @@
         <v>1</v>
       </c>
       <c r="C69" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D69" s="4" t="s">
-        <v>8</v>
+        <v>4500</v>
+      </c>
+      <c r="D69" s="4">
+        <v>3500</v>
       </c>
       <c r="E69" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F69" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="F69" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G69" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H69" s="4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
         <v>163</v>
       </c>
@@ -2800,20 +3194,23 @@
         <v>1</v>
       </c>
       <c r="C70" s="4">
+        <v>3000</v>
+      </c>
+      <c r="D70" s="4">
         <v>2000</v>
       </c>
-      <c r="D70" s="4" t="s">
+      <c r="E70" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E70" s="4" t="s">
+      <c r="F70" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="F70" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G70" s="4"/>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G70" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H70" s="4"/>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
         <v>165</v>
       </c>
@@ -2821,22 +3218,25 @@
         <v>1</v>
       </c>
       <c r="C71" s="4">
+        <v>3500</v>
+      </c>
+      <c r="D71" s="4">
         <v>2500</v>
       </c>
-      <c r="D71" s="4" t="s">
+      <c r="E71" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E71" s="4" t="s">
+      <c r="F71" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="F71" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G71" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H71" s="4" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
         <v>168</v>
       </c>
@@ -2844,20 +3244,23 @@
         <v>1</v>
       </c>
       <c r="C72" s="4">
+        <v>3000</v>
+      </c>
+      <c r="D72" s="4">
         <v>2000</v>
       </c>
-      <c r="D72" s="4" t="s">
+      <c r="E72" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E72" s="4" t="s">
+      <c r="F72" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="F72" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G72" s="4"/>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G72" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H72" s="4"/>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
         <v>170</v>
       </c>
@@ -2865,22 +3268,25 @@
         <v>1</v>
       </c>
       <c r="C73" s="4">
+        <v>3000</v>
+      </c>
+      <c r="D73" s="4">
         <v>2000</v>
       </c>
-      <c r="D73" s="4" t="s">
+      <c r="E73" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E73" s="4" t="s">
+      <c r="F73" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="F73" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G73" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H73" s="4" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
         <v>173</v>
       </c>
@@ -2888,22 +3294,25 @@
         <v>1</v>
       </c>
       <c r="C74" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D74" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E74" s="8" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D74" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E74" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F74" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="F74" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G74" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H74" s="4" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="4" t="s">
         <v>175</v>
       </c>
@@ -2911,22 +3320,25 @@
         <v>1</v>
       </c>
       <c r="C75" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D75" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D75" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E75" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E75" s="4" t="s">
+      <c r="F75" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="F75" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G75" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H75" s="4" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
         <v>177</v>
       </c>
@@ -2934,22 +3346,25 @@
         <v>1</v>
       </c>
       <c r="C76" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D76" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D76" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E76" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E76" s="4" t="s">
+      <c r="F76" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="F76" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G76" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H76" s="4" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="4" t="s">
         <v>180</v>
       </c>
@@ -2957,22 +3372,25 @@
         <v>1</v>
       </c>
       <c r="C77" s="4">
+        <v>4000</v>
+      </c>
+      <c r="D77" s="4">
         <v>3000</v>
       </c>
-      <c r="D77" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="E77" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F77" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F77" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G77" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H77" s="4" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
         <v>182</v>
       </c>
@@ -2980,22 +3398,25 @@
         <v>1</v>
       </c>
       <c r="C78" s="4">
-        <v>4500</v>
-      </c>
-      <c r="D78" s="4" t="s">
-        <v>8</v>
+        <v>5500</v>
+      </c>
+      <c r="D78" s="4">
+        <v>4500</v>
       </c>
       <c r="E78" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="F78" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G78" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H78" s="4" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="4" t="s">
         <v>263</v>
       </c>
@@ -3003,22 +3424,25 @@
         <v>1</v>
       </c>
       <c r="C79" s="4">
+        <v>6000</v>
+      </c>
+      <c r="D79" s="4">
         <v>5000</v>
       </c>
-      <c r="D79" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="E79" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F79" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="F79" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G79" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H79" s="4" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
         <v>185</v>
       </c>
@@ -3026,22 +3450,25 @@
         <v>1</v>
       </c>
       <c r="C80" s="4">
-        <v>4500</v>
-      </c>
-      <c r="D80" s="4" t="s">
-        <v>8</v>
+        <v>5500</v>
+      </c>
+      <c r="D80" s="4">
+        <v>4500</v>
       </c>
       <c r="E80" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F80" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="F80" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G80" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H80" s="4" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
         <v>188</v>
       </c>
@@ -3049,20 +3476,23 @@
         <v>1</v>
       </c>
       <c r="C81" s="4">
+        <v>6000</v>
+      </c>
+      <c r="D81" s="4">
         <v>5000</v>
       </c>
-      <c r="D81" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="E81" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F81" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="F81" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G81" s="4"/>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G81" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H81" s="4"/>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
         <v>190</v>
       </c>
@@ -3070,20 +3500,23 @@
         <v>1</v>
       </c>
       <c r="C82" s="4">
+        <v>4000</v>
+      </c>
+      <c r="D82" s="4">
         <v>3000</v>
       </c>
-      <c r="D82" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="E82" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F82" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="F82" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G82" s="4"/>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G82" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H82" s="4"/>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="4" t="s">
         <v>192</v>
       </c>
@@ -3091,20 +3524,23 @@
         <v>1</v>
       </c>
       <c r="C83" s="4">
+        <v>5000</v>
+      </c>
+      <c r="D83" s="4">
         <v>4000</v>
       </c>
-      <c r="D83" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="E83" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F83" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="F83" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G83" s="4"/>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G83" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H83" s="4"/>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
         <v>194</v>
       </c>
@@ -3112,22 +3548,25 @@
         <v>1</v>
       </c>
       <c r="C84" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D84" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E84" s="7" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D84" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E84" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F84" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="F84" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G84" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H84" s="4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>196</v>
       </c>
@@ -3135,22 +3574,25 @@
         <v>1</v>
       </c>
       <c r="C85" s="4">
+        <v>4000</v>
+      </c>
+      <c r="D85" s="4">
         <v>3000</v>
       </c>
-      <c r="D85" s="4" t="s">
+      <c r="E85" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E85" s="4" t="s">
+      <c r="F85" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="F85" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G85" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H85" s="4" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
         <v>198</v>
       </c>
@@ -3158,20 +3600,23 @@
         <v>1</v>
       </c>
       <c r="C86" s="4">
+        <v>4000</v>
+      </c>
+      <c r="D86" s="4">
         <v>3000</v>
       </c>
-      <c r="D86" s="4" t="s">
+      <c r="E86" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E86" s="4" t="s">
+      <c r="F86" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="F86" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G86" s="4"/>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G86" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H86" s="4"/>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="4" t="s">
         <v>200</v>
       </c>
@@ -3179,20 +3624,23 @@
         <v>1</v>
       </c>
       <c r="C87" s="4">
+        <v>4000</v>
+      </c>
+      <c r="D87" s="4">
         <v>3000</v>
       </c>
-      <c r="D87" s="4" t="s">
+      <c r="E87" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E87" s="4" t="s">
+      <c r="F87" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="F87" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G87" s="4"/>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G87" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H87" s="4"/>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
         <v>202</v>
       </c>
@@ -3200,22 +3648,25 @@
         <v>1</v>
       </c>
       <c r="C88" s="4">
+        <v>5000</v>
+      </c>
+      <c r="D88" s="4">
         <v>4000</v>
       </c>
-      <c r="D88" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="E88" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F88" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="F88" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G88" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H88" s="4" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
         <v>205</v>
       </c>
@@ -3223,22 +3674,25 @@
         <v>1</v>
       </c>
       <c r="C89" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D89" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D89" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E89" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E89" s="4" t="s">
+      <c r="F89" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="F89" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G89" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H89" s="4" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
         <v>208</v>
       </c>
@@ -3246,22 +3700,25 @@
         <v>1</v>
       </c>
       <c r="C90" s="4">
+        <v>5000</v>
+      </c>
+      <c r="D90" s="4">
         <v>4000</v>
       </c>
-      <c r="D90" s="4" t="s">
+      <c r="E90" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E90" s="4" t="s">
+      <c r="F90" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="F90" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G90" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H90" s="4" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" s="4" t="s">
         <v>210</v>
       </c>
@@ -3269,22 +3726,25 @@
         <v>1</v>
       </c>
       <c r="C91" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D91" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D91" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E91" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E91" s="4" t="s">
+      <c r="F91" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="F91" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G91" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H91" s="4" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
         <v>212</v>
       </c>
@@ -3292,20 +3752,23 @@
         <v>1</v>
       </c>
       <c r="C92" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D92" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D92" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E92" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E92" s="4" t="s">
+      <c r="F92" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="F92" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G92" s="4"/>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G92" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H92" s="4"/>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
         <v>214</v>
       </c>
@@ -3313,22 +3776,25 @@
         <v>1</v>
       </c>
       <c r="C93" s="4">
+        <v>4000</v>
+      </c>
+      <c r="D93" s="4">
         <v>3000</v>
       </c>
-      <c r="D93" s="4" t="s">
+      <c r="E93" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E93" s="4" t="s">
+      <c r="F93" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="F93" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G93" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H93" s="4" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
         <v>216</v>
       </c>
@@ -3336,20 +3802,23 @@
         <v>1</v>
       </c>
       <c r="C94" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D94" s="4" t="s">
-        <v>8</v>
+        <v>4500</v>
+      </c>
+      <c r="D94" s="4">
+        <v>3500</v>
       </c>
       <c r="E94" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F94" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="F94" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G94" s="4"/>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G94" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H94" s="4"/>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" s="4" t="s">
         <v>218</v>
       </c>
@@ -3357,22 +3826,25 @@
         <v>1</v>
       </c>
       <c r="C95" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D95" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D95" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E95" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E95" s="4" t="s">
+      <c r="F95" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="F95" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G95" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H95" s="4" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
         <v>220</v>
       </c>
@@ -3380,22 +3852,25 @@
         <v>1</v>
       </c>
       <c r="C96" s="4">
+        <v>5000</v>
+      </c>
+      <c r="D96" s="4">
         <v>4000</v>
       </c>
-      <c r="D96" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="E96" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F96" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="F96" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G96" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H96" s="4" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" s="4" t="s">
         <v>223</v>
       </c>
@@ -3403,20 +3878,23 @@
         <v>1</v>
       </c>
       <c r="C97" s="4">
+        <v>4000</v>
+      </c>
+      <c r="D97" s="4">
         <v>3000</v>
       </c>
-      <c r="D97" s="4" t="s">
+      <c r="E97" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E97" s="4" t="s">
+      <c r="F97" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="F97" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G97" s="4"/>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G97" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H97" s="4"/>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
         <v>225</v>
       </c>
@@ -3424,22 +3902,25 @@
         <v>1</v>
       </c>
       <c r="C98" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D98" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D98" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E98" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E98" s="4" t="s">
+      <c r="F98" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="F98" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G98" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H98" s="4" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="4" t="s">
         <v>227</v>
       </c>
@@ -3447,20 +3928,23 @@
         <v>1</v>
       </c>
       <c r="C99" s="4">
+        <v>4000</v>
+      </c>
+      <c r="D99" s="4">
         <v>3000</v>
       </c>
-      <c r="D99" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="E99" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F99" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="F99" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G99" s="4"/>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G99" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H99" s="4"/>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
         <v>229</v>
       </c>
@@ -3468,20 +3952,23 @@
         <v>1</v>
       </c>
       <c r="C100" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D100" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D100" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E100" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E100" s="4" t="s">
+      <c r="F100" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="F100" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G100" s="4"/>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G100" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H100" s="4"/>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="4" t="s">
         <v>231</v>
       </c>
@@ -3489,20 +3976,23 @@
         <v>1</v>
       </c>
       <c r="C101" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D101" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D101" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E101" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E101" s="4" t="s">
+      <c r="F101" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="F101" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G101" s="4"/>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G101" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H101" s="4"/>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
         <v>233</v>
       </c>
@@ -3510,22 +4000,25 @@
         <v>1</v>
       </c>
       <c r="C102" s="4">
+        <v>5000</v>
+      </c>
+      <c r="D102" s="4">
         <v>4000</v>
       </c>
-      <c r="D102" s="4" t="s">
+      <c r="E102" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E102" s="4" t="s">
+      <c r="F102" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="F102" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G102" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H102" s="4" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" s="4" t="s">
         <v>235</v>
       </c>
@@ -3533,20 +4026,23 @@
         <v>1</v>
       </c>
       <c r="C103" s="4">
+        <v>3500</v>
+      </c>
+      <c r="D103" s="4">
         <v>2500</v>
       </c>
-      <c r="D103" s="4" t="s">
+      <c r="E103" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E103" s="4" t="s">
+      <c r="F103" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="F103" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G103" s="4"/>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G103" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H103" s="4"/>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
         <v>237</v>
       </c>
@@ -3554,20 +4050,23 @@
         <v>1</v>
       </c>
       <c r="C104" s="4">
+        <v>4000</v>
+      </c>
+      <c r="D104" s="4">
         <v>3000</v>
       </c>
-      <c r="D104" s="4" t="s">
+      <c r="E104" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E104" s="4" t="s">
+      <c r="F104" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="F104" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G104" s="4"/>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G104" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H104" s="4"/>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" s="4" t="s">
         <v>239</v>
       </c>
@@ -3575,20 +4074,23 @@
         <v>1</v>
       </c>
       <c r="C105" s="4">
+        <v>5000</v>
+      </c>
+      <c r="D105" s="4">
         <v>4000</v>
       </c>
-      <c r="D105" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="E105" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F105" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="F105" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G105" s="4"/>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G105" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H105" s="4"/>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
         <v>241</v>
       </c>
@@ -3596,20 +4098,23 @@
         <v>1</v>
       </c>
       <c r="C106" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D106" s="4" t="s">
-        <v>8</v>
+        <v>4500</v>
+      </c>
+      <c r="D106" s="4">
+        <v>3500</v>
       </c>
       <c r="E106" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F106" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="F106" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G106" s="4"/>
-    </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G106" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H106" s="4"/>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" s="4" t="s">
         <v>243</v>
       </c>
@@ -3617,20 +4122,23 @@
         <v>1</v>
       </c>
       <c r="C107" s="4">
+        <v>6000</v>
+      </c>
+      <c r="D107" s="4">
         <v>5000</v>
       </c>
-      <c r="D107" s="4" t="s">
+      <c r="E107" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E107" s="4" t="s">
+      <c r="F107" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="F107" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G107" s="4"/>
-    </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G107" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H107" s="4"/>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
         <v>245</v>
       </c>
@@ -3638,22 +4146,25 @@
         <v>1</v>
       </c>
       <c r="C108" s="4">
+        <v>5000</v>
+      </c>
+      <c r="D108" s="4">
         <v>4000</v>
       </c>
-      <c r="D108" s="4" t="s">
+      <c r="E108" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E108" s="4" t="s">
+      <c r="F108" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="F108" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G108" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H108" s="4" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" s="4" t="s">
         <v>247</v>
       </c>
@@ -3661,20 +4172,23 @@
         <v>1</v>
       </c>
       <c r="C109" s="4">
+        <v>3500</v>
+      </c>
+      <c r="D109" s="4">
         <v>2500</v>
       </c>
-      <c r="D109" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="E109" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F109" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="F109" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G109" s="4"/>
-    </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G109" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H109" s="4"/>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
         <v>249</v>
       </c>
@@ -3682,22 +4196,25 @@
         <v>1</v>
       </c>
       <c r="C110" s="4">
-        <v>4500</v>
-      </c>
-      <c r="D110" s="4" t="s">
-        <v>8</v>
+        <v>5500</v>
+      </c>
+      <c r="D110" s="4">
+        <v>4500</v>
       </c>
       <c r="E110" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F110" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="F110" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="G110" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H110" s="4" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" s="4" t="s">
         <v>251</v>
       </c>
@@ -3705,44 +4222,47 @@
         <v>1</v>
       </c>
       <c r="C111" s="4">
-        <v>3500</v>
-      </c>
-      <c r="D111" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E111" s="5" t="s">
+        <v>4500</v>
+      </c>
+      <c r="D111" s="4">
+        <v>3500</v>
+      </c>
+      <c r="E111" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F111" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="F111" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="G111" s="4"/>
+      <c r="G111" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H111" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="E6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="E7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="E8" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="E10" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="E34" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="E35" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="E36" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="E37" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="E38" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="E45" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="E52" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="E80" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="E84" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="E64" r:id="rId17" xr:uid="{B18A4056-2B5D-414C-A9F6-273D95C7ED18}"/>
-    <hyperlink ref="E63" r:id="rId18" xr:uid="{D80AB2AB-AFBA-474C-9099-56659D4F7343}"/>
-    <hyperlink ref="E57" r:id="rId19" xr:uid="{DBFEB124-BE06-49CC-A78E-75F68A01BDE0}"/>
-    <hyperlink ref="E61" r:id="rId20" xr:uid="{EA7715C1-7791-4747-91D3-03A4B27F1C4F}"/>
-    <hyperlink ref="E79" r:id="rId21" xr:uid="{94830BFD-52CC-4963-9874-F1F984E1589C}"/>
-    <hyperlink ref="E60" r:id="rId22" xr:uid="{92F7858F-B769-4909-A899-8246468D0096}"/>
-    <hyperlink ref="E30" r:id="rId23" xr:uid="{66D24E2B-EF6D-4417-A0A4-812E5961FB81}"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="F6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="F7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="F8" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="F10" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="F34" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="F35" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="F36" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="F37" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="F38" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="F45" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="F52" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="F80" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="F84" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="F64" r:id="rId17" xr:uid="{B18A4056-2B5D-414C-A9F6-273D95C7ED18}"/>
+    <hyperlink ref="F63" r:id="rId18" xr:uid="{D80AB2AB-AFBA-474C-9099-56659D4F7343}"/>
+    <hyperlink ref="F57" r:id="rId19" xr:uid="{DBFEB124-BE06-49CC-A78E-75F68A01BDE0}"/>
+    <hyperlink ref="F61" r:id="rId20" xr:uid="{EA7715C1-7791-4747-91D3-03A4B27F1C4F}"/>
+    <hyperlink ref="F79" r:id="rId21" xr:uid="{94830BFD-52CC-4963-9874-F1F984E1589C}"/>
+    <hyperlink ref="F60" r:id="rId22" xr:uid="{92F7858F-B769-4909-A899-8246468D0096}"/>
+    <hyperlink ref="F30" r:id="rId23" xr:uid="{66D24E2B-EF6D-4417-A0A4-812E5961FB81}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>

</xml_diff>

<commit_message>
Ajustes responsive horizontal (movil/tablet), UI y datos de cartas
Layout landscape en tablero, app-layout, mazos, jugarPartida y salud; actualizaciones en partida, mazos, tienda y recursos.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/resources/cartas.xlsx
+++ b/public/resources/cartas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EE1870F-4241-43AD-B147-C8D28C003057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D362B1BA-D3BA-4B0C-A5D6-B40E932C2058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="318">
   <si>
     <t>Nombre</t>
   </si>
@@ -883,9 +883,6 @@
     <t>Reduce el poder de todas las cartas enemigas en juego.</t>
   </si>
   <si>
-    <t>Cura 500 puntos de salud una carta aliada</t>
-  </si>
-  <si>
     <t>Revive una carta de tu elección del cementerio y la devuelve al mazo.</t>
   </si>
   <si>
@@ -911,6 +908,72 @@
   </si>
   <si>
     <t>Salud</t>
+  </si>
+  <si>
+    <t>Cura 500 puntos de salud a la carta aliada elegida</t>
+  </si>
+  <si>
+    <t>heal_all</t>
+  </si>
+  <si>
+    <t>Cura 500 puntos de salud a todos los aliados en juego</t>
+  </si>
+  <si>
+    <t>Curar++</t>
+  </si>
+  <si>
+    <t>bonus_buff</t>
+  </si>
+  <si>
+    <t>bonus_debuff</t>
+  </si>
+  <si>
+    <t>tank</t>
+  </si>
+  <si>
+    <t>salud*2</t>
+  </si>
+  <si>
+    <t>Duplica su salud y reduce su ataque a la mitad</t>
+  </si>
+  <si>
+    <t>Tanque</t>
+  </si>
+  <si>
+    <t>Potenciar Bonus</t>
+  </si>
+  <si>
+    <t>Anular Bonus</t>
+  </si>
+  <si>
+    <t>Potencia +500 el bonus de afiliación aliado que esté activo</t>
+  </si>
+  <si>
+    <t>Anula el bonus activo enemigo mientras esta carta esté en juego.</t>
+  </si>
+  <si>
+    <t>heal_debuff</t>
+  </si>
+  <si>
+    <t>Reduce un 25% la salud actual de los enemigos en juego, mientras esta carta esté activa</t>
+  </si>
+  <si>
+    <t>Debilitador</t>
+  </si>
+  <si>
+    <t>saludEnemigo*0.75</t>
+  </si>
+  <si>
+    <t>extra_attack</t>
+  </si>
+  <si>
+    <t>Ataque Extra</t>
+  </si>
+  <si>
+    <t>poder</t>
+  </si>
+  <si>
+    <t>Al activar esta habilidad, la carta realiza un ataque extra haciendo n de daño.</t>
   </si>
 </sst>
 </file>
@@ -1001,7 +1064,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1032,7 +1095,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1325,8 +1387,8 @@
     <col min="8" max="8" width="42.42578125" customWidth="1"/>
     <col min="9" max="9" width="71.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="63.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" customWidth="1"/>
+    <col min="11" max="11" width="79.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
@@ -1339,7 +1401,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -1368,10 +1430,10 @@
       <c r="L1" s="11" t="s">
         <v>270</v>
       </c>
-      <c r="M1" s="12" t="s">
+      <c r="M1" s="11" t="s">
         <v>273</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="N1" s="11" t="s">
         <v>279</v>
       </c>
     </row>
@@ -1413,7 +1475,7 @@
         <v>500</v>
       </c>
       <c r="N2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -1454,7 +1516,7 @@
         <v>500</v>
       </c>
       <c r="N3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -1486,7 +1548,7 @@
         <v>282</v>
       </c>
       <c r="K4" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
       <c r="L4" t="s">
         <v>276</v>
@@ -1495,7 +1557,7 @@
         <v>500</v>
       </c>
       <c r="N4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -1527,7 +1589,7 @@
         <v>283</v>
       </c>
       <c r="K5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="L5" t="s">
         <v>277</v>
@@ -1536,7 +1598,7 @@
         <v>1</v>
       </c>
       <c r="N5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -1568,7 +1630,7 @@
         <v>284</v>
       </c>
       <c r="K6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="L6" t="s">
         <v>278</v>
@@ -1577,7 +1639,7 @@
         <v>1000</v>
       </c>
       <c r="N6" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -1606,19 +1668,19 @@
         <v>28</v>
       </c>
       <c r="J7" t="s">
+        <v>293</v>
+      </c>
+      <c r="K7" t="s">
         <v>294</v>
       </c>
-      <c r="K7" t="s">
-        <v>295</v>
-      </c>
       <c r="L7" t="s">
+        <v>291</v>
+      </c>
+      <c r="M7" t="s">
         <v>292</v>
       </c>
-      <c r="M7" t="s">
-        <v>293</v>
-      </c>
       <c r="N7" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -1646,6 +1708,21 @@
       <c r="H8" s="10" t="s">
         <v>31</v>
       </c>
+      <c r="J8" t="s">
+        <v>299</v>
+      </c>
+      <c r="K8" t="s">
+        <v>298</v>
+      </c>
+      <c r="L8" t="s">
+        <v>297</v>
+      </c>
+      <c r="M8">
+        <v>500</v>
+      </c>
+      <c r="N8" t="s">
+        <v>290</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
@@ -1672,6 +1749,21 @@
       <c r="H9" s="10" t="s">
         <v>28</v>
       </c>
+      <c r="J9" t="s">
+        <v>306</v>
+      </c>
+      <c r="K9" t="s">
+        <v>308</v>
+      </c>
+      <c r="L9" t="s">
+        <v>300</v>
+      </c>
+      <c r="M9">
+        <v>500</v>
+      </c>
+      <c r="N9" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
@@ -1701,6 +1793,18 @@
       <c r="I10" t="s">
         <v>258</v>
       </c>
+      <c r="J10" t="s">
+        <v>307</v>
+      </c>
+      <c r="K10" t="s">
+        <v>309</v>
+      </c>
+      <c r="L10" t="s">
+        <v>301</v>
+      </c>
+      <c r="N10" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
@@ -1725,6 +1829,21 @@
         <v>10</v>
       </c>
       <c r="H11" s="10"/>
+      <c r="J11" t="s">
+        <v>305</v>
+      </c>
+      <c r="K11" t="s">
+        <v>304</v>
+      </c>
+      <c r="L11" t="s">
+        <v>302</v>
+      </c>
+      <c r="M11" t="s">
+        <v>303</v>
+      </c>
+      <c r="N11" t="s">
+        <v>290</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
@@ -1751,6 +1870,21 @@
       <c r="H12" s="10" t="s">
         <v>41</v>
       </c>
+      <c r="J12" t="s">
+        <v>312</v>
+      </c>
+      <c r="K12" t="s">
+        <v>311</v>
+      </c>
+      <c r="L12" t="s">
+        <v>310</v>
+      </c>
+      <c r="M12" t="s">
+        <v>313</v>
+      </c>
+      <c r="N12" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
@@ -1775,6 +1909,21 @@
         <v>10</v>
       </c>
       <c r="H13" s="10"/>
+      <c r="J13" t="s">
+        <v>315</v>
+      </c>
+      <c r="K13" t="s">
+        <v>317</v>
+      </c>
+      <c r="L13" t="s">
+        <v>314</v>
+      </c>
+      <c r="M13" t="s">
+        <v>316</v>
+      </c>
+      <c r="N13" t="s">
+        <v>290</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">

</xml_diff>

<commit_message>
Actualizar cartas.xlsx a la ultima version
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/resources/cartas.xlsx
+++ b/public/resources/cartas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D362B1BA-D3BA-4B0C-A5D6-B40E932C2058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17361BF3-3CB6-47E4-904B-DC77C435187B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1005,7 +1005,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1021,6 +1021,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF7C80"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF64DA89"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCBAAEC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF99CCFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1064,7 +1088,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1095,6 +1119,11 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1102,6 +1131,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFCBAAEC"/>
+      <color rgb="FF99CCFF"/>
+      <color rgb="FFFF7C80"/>
+      <color rgb="FF64DA89"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1380,12 +1417,14 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="2" width="6.85546875" customWidth="1"/>
-    <col min="3" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="105.85546875" customWidth="1"/>
-    <col min="7" max="7" width="10.5703125" customWidth="1"/>
+    <col min="2" max="2" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.42578125" customWidth="1"/>
+    <col min="7" max="7" width="7.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="42.42578125" customWidth="1"/>
-    <col min="9" max="9" width="71.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" customWidth="1"/>
     <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="79.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -1462,19 +1501,19 @@
       <c r="H2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="13" t="s">
         <v>280</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="13" t="s">
         <v>285</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="13" t="s">
         <v>274</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="13">
         <v>500</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" s="13" t="s">
         <v>289</v>
       </c>
     </row>
@@ -1503,19 +1542,19 @@
       <c r="H3" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="12" t="s">
         <v>281</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="12" t="s">
         <v>286</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="12" t="s">
         <v>275</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="12">
         <v>500</v>
       </c>
-      <c r="N3" t="s">
+      <c r="N3" s="12" t="s">
         <v>289</v>
       </c>
     </row>
@@ -1544,19 +1583,19 @@
       <c r="H4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="13" t="s">
         <v>282</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="13" t="s">
         <v>296</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" s="13" t="s">
         <v>276</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="13">
         <v>500</v>
       </c>
-      <c r="N4" t="s">
+      <c r="N4" s="13" t="s">
         <v>290</v>
       </c>
     </row>
@@ -1585,19 +1624,19 @@
       <c r="H5" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="15" t="s">
         <v>283</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="15" t="s">
         <v>287</v>
       </c>
-      <c r="L5" t="s">
+      <c r="L5" s="15" t="s">
         <v>277</v>
       </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-      <c r="N5" t="s">
+      <c r="M5" s="15">
+        <v>1</v>
+      </c>
+      <c r="N5" s="15" t="s">
         <v>290</v>
       </c>
     </row>
@@ -1626,19 +1665,19 @@
       <c r="H6" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="16" t="s">
         <v>284</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K6" s="16" t="s">
         <v>288</v>
       </c>
-      <c r="L6" t="s">
+      <c r="L6" s="16" t="s">
         <v>278</v>
       </c>
-      <c r="M6">
+      <c r="M6" s="16">
         <v>1000</v>
       </c>
-      <c r="N6" t="s">
+      <c r="N6" s="16" t="s">
         <v>290</v>
       </c>
     </row>
@@ -1667,19 +1706,19 @@
       <c r="H7" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="12" t="s">
         <v>293</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K7" s="12" t="s">
         <v>294</v>
       </c>
-      <c r="L7" t="s">
+      <c r="L7" s="12" t="s">
         <v>291</v>
       </c>
-      <c r="M7" t="s">
+      <c r="M7" s="12" t="s">
         <v>292</v>
       </c>
-      <c r="N7" t="s">
+      <c r="N7" s="12" t="s">
         <v>290</v>
       </c>
     </row>
@@ -1708,19 +1747,19 @@
       <c r="H8" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J8" s="13" t="s">
         <v>299</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K8" s="13" t="s">
         <v>298</v>
       </c>
-      <c r="L8" t="s">
+      <c r="L8" s="13" t="s">
         <v>297</v>
       </c>
-      <c r="M8">
+      <c r="M8" s="13">
         <v>500</v>
       </c>
-      <c r="N8" t="s">
+      <c r="N8" s="13" t="s">
         <v>290</v>
       </c>
     </row>
@@ -1749,19 +1788,19 @@
       <c r="H9" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="14" t="s">
         <v>308</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L9" s="14" t="s">
         <v>300</v>
       </c>
-      <c r="M9">
+      <c r="M9" s="14">
         <v>500</v>
       </c>
-      <c r="N9" t="s">
+      <c r="N9" s="14" t="s">
         <v>289</v>
       </c>
     </row>
@@ -1793,16 +1832,17 @@
       <c r="I10" t="s">
         <v>258</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J10" s="15" t="s">
         <v>307</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K10" s="15" t="s">
         <v>309</v>
       </c>
-      <c r="L10" t="s">
+      <c r="L10" s="15" t="s">
         <v>301</v>
       </c>
-      <c r="N10" t="s">
+      <c r="M10" s="15"/>
+      <c r="N10" s="15" t="s">
         <v>289</v>
       </c>
     </row>
@@ -1829,19 +1869,19 @@
         <v>10</v>
       </c>
       <c r="H11" s="10"/>
-      <c r="J11" t="s">
+      <c r="J11" s="16" t="s">
         <v>305</v>
       </c>
-      <c r="K11" t="s">
+      <c r="K11" s="16" t="s">
         <v>304</v>
       </c>
-      <c r="L11" t="s">
+      <c r="L11" s="16" t="s">
         <v>302</v>
       </c>
-      <c r="M11" t="s">
+      <c r="M11" s="16" t="s">
         <v>303</v>
       </c>
-      <c r="N11" t="s">
+      <c r="N11" s="16" t="s">
         <v>290</v>
       </c>
     </row>
@@ -1870,19 +1910,19 @@
       <c r="H12" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="15" t="s">
         <v>312</v>
       </c>
-      <c r="K12" t="s">
+      <c r="K12" s="15" t="s">
         <v>311</v>
       </c>
-      <c r="L12" t="s">
+      <c r="L12" s="15" t="s">
         <v>310</v>
       </c>
-      <c r="M12" t="s">
+      <c r="M12" s="15" t="s">
         <v>313</v>
       </c>
-      <c r="N12" t="s">
+      <c r="N12" s="15" t="s">
         <v>289</v>
       </c>
     </row>
@@ -1909,19 +1949,19 @@
         <v>10</v>
       </c>
       <c r="H13" s="10"/>
-      <c r="J13" t="s">
+      <c r="J13" s="12" t="s">
         <v>315</v>
       </c>
-      <c r="K13" t="s">
+      <c r="K13" s="12" t="s">
         <v>317</v>
       </c>
-      <c r="L13" t="s">
+      <c r="L13" s="12" t="s">
         <v>314</v>
       </c>
-      <c r="M13" t="s">
+      <c r="M13" s="12" t="s">
         <v>316</v>
       </c>
-      <c r="N13" t="s">
+      <c r="N13" s="12" t="s">
         <v>290</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar sistema de juego y UI para Beta-1.0.0.
Incluye cooldown de habilidades activas, mejoras visuales del menu/tienda, correcciones de progresion y badges, y agrega CHANGELOG para seguimiento de versiones.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/resources/cartas.xlsx
+++ b/public/resources/cartas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17361BF3-3CB6-47E4-904B-DC77C435187B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA14F89F-95D7-4D21-845E-D089CC373CB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="318">
   <si>
     <t>Nombre</t>
   </si>
@@ -877,18 +877,9 @@
     <t>Escudo</t>
   </si>
   <si>
-    <t>Aumenta el poder de todos las cartas aliadas en juego.</t>
-  </si>
-  <si>
-    <t>Reduce el poder de todas las cartas enemigas en juego.</t>
-  </si>
-  <si>
     <t>Revive una carta de tu elección del cementerio y la devuelve al mazo.</t>
   </si>
   <si>
-    <t>Aplica un escudo en esta carta, o en una carta aliada.</t>
-  </si>
-  <si>
     <t>auto</t>
   </si>
   <si>
@@ -910,15 +901,9 @@
     <t>Salud</t>
   </si>
   <si>
-    <t>Cura 500 puntos de salud a la carta aliada elegida</t>
-  </si>
-  <si>
     <t>heal_all</t>
   </si>
   <si>
-    <t>Cura 500 puntos de salud a todos los aliados en juego</t>
-  </si>
-  <si>
     <t>Curar++</t>
   </si>
   <si>
@@ -946,9 +931,6 @@
     <t>Anular Bonus</t>
   </si>
   <si>
-    <t>Potencia +500 el bonus de afiliación aliado que esté activo</t>
-  </si>
-  <si>
     <t>Anula el bonus activo enemigo mientras esta carta esté en juego.</t>
   </si>
   <si>
@@ -974,6 +956,24 @@
   </si>
   <si>
     <t>Al activar esta habilidad, la carta realiza un ataque extra haciendo n de daño.</t>
+  </si>
+  <si>
+    <t>Aumenta @skill_power el poder de todos las cartas aliadas en juego.</t>
+  </si>
+  <si>
+    <t>Reduce @skill_power el poder de todas las cartas enemigas en juego.</t>
+  </si>
+  <si>
+    <t>Cura @skill_power puntos de salud a la carta aliada elegida</t>
+  </si>
+  <si>
+    <t>Cura @skill_power puntos de salud a todos los aliados en juego</t>
+  </si>
+  <si>
+    <t>Aplica @skill_power puntos de escudo a esta carta, o a una carta aliada.</t>
+  </si>
+  <si>
+    <t>Potencia @skill_power el bonus de afiliación aliado que esté activo</t>
   </si>
 </sst>
 </file>
@@ -1119,11 +1119,21 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1428,11 +1438,11 @@
     <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="79.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.85546875" customWidth="1"/>
     <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1440,7 +1450,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -1476,7 +1486,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -1501,23 +1511,24 @@
       <c r="H2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="I2" s="2"/>
+      <c r="J2" s="12" t="s">
         <v>280</v>
       </c>
-      <c r="K2" s="13" t="s">
-        <v>285</v>
-      </c>
-      <c r="L2" s="13" t="s">
+      <c r="K2" s="12" t="s">
+        <v>312</v>
+      </c>
+      <c r="L2" s="12" t="s">
         <v>274</v>
       </c>
-      <c r="M2" s="13">
+      <c r="M2" s="12">
         <v>500</v>
       </c>
-      <c r="N2" s="13" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N2" s="12" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
@@ -1542,23 +1553,24 @@
       <c r="H3" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J3" s="12" t="s">
+      <c r="I3" s="2"/>
+      <c r="J3" s="13" t="s">
         <v>281</v>
       </c>
-      <c r="K3" s="12" t="s">
+      <c r="K3" s="13" t="s">
+        <v>313</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="M3" s="13">
+        <v>500</v>
+      </c>
+      <c r="N3" s="13" t="s">
         <v>286</v>
       </c>
-      <c r="L3" s="12" t="s">
-        <v>275</v>
-      </c>
-      <c r="M3" s="12">
-        <v>500</v>
-      </c>
-      <c r="N3" s="12" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -1583,23 +1595,24 @@
       <c r="H4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="I4" s="2"/>
+      <c r="J4" s="12" t="s">
         <v>282</v>
       </c>
-      <c r="K4" s="13" t="s">
-        <v>296</v>
-      </c>
-      <c r="L4" s="13" t="s">
+      <c r="K4" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="L4" s="12" t="s">
         <v>276</v>
       </c>
-      <c r="M4" s="13">
+      <c r="M4" s="12">
         <v>500</v>
       </c>
-      <c r="N4" s="13" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N4" s="12" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>18</v>
       </c>
@@ -1624,23 +1637,24 @@
       <c r="H5" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="J5" s="15" t="s">
+      <c r="I5" s="2"/>
+      <c r="J5" s="14" t="s">
         <v>283</v>
       </c>
-      <c r="K5" s="15" t="s">
+      <c r="K5" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="M5" s="14">
+        <v>1</v>
+      </c>
+      <c r="N5" s="14" t="s">
         <v>287</v>
       </c>
-      <c r="L5" s="15" t="s">
-        <v>277</v>
-      </c>
-      <c r="M5" s="15">
-        <v>1</v>
-      </c>
-      <c r="N5" s="15" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>22</v>
       </c>
@@ -1665,23 +1679,24 @@
       <c r="H6" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="J6" s="16" t="s">
+      <c r="I6" s="2"/>
+      <c r="J6" s="15" t="s">
         <v>284</v>
       </c>
-      <c r="K6" s="16" t="s">
-        <v>288</v>
-      </c>
-      <c r="L6" s="16" t="s">
+      <c r="K6" s="15" t="s">
+        <v>316</v>
+      </c>
+      <c r="L6" s="15" t="s">
         <v>278</v>
       </c>
-      <c r="M6" s="16">
+      <c r="M6" s="15">
         <v>1000</v>
       </c>
-      <c r="N6" s="16" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N6" s="15" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>26</v>
       </c>
@@ -1706,23 +1721,24 @@
       <c r="H7" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J7" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="K7" s="12" t="s">
-        <v>294</v>
-      </c>
-      <c r="L7" s="12" t="s">
+      <c r="I7" s="2"/>
+      <c r="J7" s="13" t="s">
+        <v>290</v>
+      </c>
+      <c r="K7" s="13" t="s">
         <v>291</v>
       </c>
-      <c r="M7" s="12" t="s">
-        <v>292</v>
-      </c>
-      <c r="N7" s="12" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="L7" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="M7" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="N7" s="13" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
@@ -1747,23 +1763,24 @@
       <c r="H8" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="J8" s="13" t="s">
-        <v>299</v>
-      </c>
-      <c r="K8" s="13" t="s">
-        <v>298</v>
-      </c>
-      <c r="L8" s="13" t="s">
-        <v>297</v>
-      </c>
-      <c r="M8" s="13">
+      <c r="I8" s="2"/>
+      <c r="J8" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="K8" s="12" t="s">
+        <v>315</v>
+      </c>
+      <c r="L8" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="M8" s="12">
         <v>500</v>
       </c>
-      <c r="N8" s="13" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N8" s="12" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>32</v>
       </c>
@@ -1788,23 +1805,24 @@
       <c r="H9" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J9" s="14" t="s">
-        <v>306</v>
-      </c>
-      <c r="K9" s="14" t="s">
-        <v>308</v>
-      </c>
-      <c r="L9" s="14" t="s">
-        <v>300</v>
-      </c>
-      <c r="M9" s="14">
+      <c r="I9" s="2"/>
+      <c r="J9" s="16" t="s">
+        <v>301</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>317</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="M9" s="16">
         <v>500</v>
       </c>
-      <c r="N9" s="14" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N9" s="16" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>34</v>
       </c>
@@ -1829,24 +1847,24 @@
       <c r="H10" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="J10" s="15" t="s">
-        <v>307</v>
-      </c>
-      <c r="K10" s="15" t="s">
-        <v>309</v>
-      </c>
-      <c r="L10" s="15" t="s">
-        <v>301</v>
-      </c>
-      <c r="M10" s="15"/>
-      <c r="N10" s="15" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J10" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="K10" s="14" t="s">
+        <v>303</v>
+      </c>
+      <c r="L10" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="M10" s="14"/>
+      <c r="N10" s="14" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>37</v>
       </c>
@@ -1869,23 +1887,24 @@
         <v>10</v>
       </c>
       <c r="H11" s="10"/>
-      <c r="J11" s="16" t="s">
-        <v>305</v>
-      </c>
-      <c r="K11" s="16" t="s">
-        <v>304</v>
-      </c>
-      <c r="L11" s="16" t="s">
-        <v>302</v>
-      </c>
-      <c r="M11" s="16" t="s">
-        <v>303</v>
-      </c>
-      <c r="N11" s="16" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I11" s="2"/>
+      <c r="J11" s="15" t="s">
+        <v>300</v>
+      </c>
+      <c r="K11" s="15" t="s">
+        <v>299</v>
+      </c>
+      <c r="L11" s="15" t="s">
+        <v>297</v>
+      </c>
+      <c r="M11" s="15" t="s">
+        <v>298</v>
+      </c>
+      <c r="N11" s="15" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>39</v>
       </c>
@@ -1910,23 +1929,24 @@
       <c r="H12" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="J12" s="15" t="s">
-        <v>312</v>
-      </c>
-      <c r="K12" s="15" t="s">
-        <v>311</v>
-      </c>
-      <c r="L12" s="15" t="s">
-        <v>310</v>
-      </c>
-      <c r="M12" s="15" t="s">
-        <v>313</v>
-      </c>
-      <c r="N12" s="15" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I12" s="2"/>
+      <c r="J12" s="14" t="s">
+        <v>306</v>
+      </c>
+      <c r="K12" s="14" t="s">
+        <v>305</v>
+      </c>
+      <c r="L12" s="14" t="s">
+        <v>304</v>
+      </c>
+      <c r="M12" s="14" t="s">
+        <v>307</v>
+      </c>
+      <c r="N12" s="14" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>42</v>
       </c>
@@ -1949,23 +1969,24 @@
         <v>10</v>
       </c>
       <c r="H13" s="10"/>
-      <c r="J13" s="12" t="s">
-        <v>315</v>
-      </c>
-      <c r="K13" s="12" t="s">
-        <v>317</v>
-      </c>
-      <c r="L13" s="12" t="s">
-        <v>314</v>
-      </c>
-      <c r="M13" s="12" t="s">
-        <v>316</v>
-      </c>
-      <c r="N13" s="12" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I13" s="2"/>
+      <c r="J13" s="13" t="s">
+        <v>309</v>
+      </c>
+      <c r="K13" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="L13" s="13" t="s">
+        <v>308</v>
+      </c>
+      <c r="M13" s="13" t="s">
+        <v>310</v>
+      </c>
+      <c r="N13" s="13" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>44</v>
       </c>
@@ -1989,7 +2010,7 @@
       </c>
       <c r="H14" s="10"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>46</v>
       </c>
@@ -2015,7 +2036,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>49</v>
       </c>
@@ -2041,7 +2062,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>52</v>
       </c>
@@ -2067,7 +2088,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>54</v>
       </c>
@@ -2091,7 +2112,7 @@
       </c>
       <c r="H18" s="10"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>56</v>
       </c>
@@ -2115,7 +2136,7 @@
       </c>
       <c r="H19" s="10"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>58</v>
       </c>
@@ -2139,7 +2160,7 @@
       </c>
       <c r="H20" s="10"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>60</v>
       </c>
@@ -2163,7 +2184,7 @@
       </c>
       <c r="H21" s="10"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>62</v>
       </c>
@@ -2187,7 +2208,7 @@
       </c>
       <c r="H22" s="10"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>64</v>
       </c>
@@ -2211,7 +2232,7 @@
       </c>
       <c r="H23" s="10"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>66</v>
       </c>
@@ -2235,7 +2256,7 @@
       </c>
       <c r="H24" s="10"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>68</v>
       </c>
@@ -2259,7 +2280,7 @@
       </c>
       <c r="H25" s="10"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>70</v>
       </c>
@@ -2285,7 +2306,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>72</v>
       </c>
@@ -2311,7 +2332,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>74</v>
       </c>
@@ -2337,7 +2358,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>77</v>
       </c>
@@ -2363,7 +2384,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>267</v>
       </c>
@@ -2389,7 +2410,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>79</v>
       </c>
@@ -2415,7 +2436,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>81</v>
       </c>
@@ -2441,7 +2462,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>84</v>
       </c>
@@ -2467,7 +2488,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>86</v>
       </c>
@@ -2491,7 +2512,7 @@
       </c>
       <c r="H34" s="10"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>88</v>
       </c>
@@ -2517,7 +2538,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>90</v>
       </c>
@@ -2541,7 +2562,7 @@
       </c>
       <c r="H36" s="10"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>92</v>
       </c>
@@ -2567,7 +2588,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>95</v>
       </c>
@@ -2593,7 +2614,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>97</v>
       </c>
@@ -2617,7 +2638,7 @@
       </c>
       <c r="H39" s="10"/>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>99</v>
       </c>
@@ -2641,7 +2662,7 @@
       </c>
       <c r="H40" s="10"/>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>101</v>
       </c>
@@ -2667,7 +2688,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>103</v>
       </c>
@@ -2693,7 +2714,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>105</v>
       </c>
@@ -2719,7 +2740,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>108</v>
       </c>
@@ -2745,7 +2766,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>111</v>
       </c>
@@ -2771,7 +2792,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>113</v>
       </c>
@@ -2797,7 +2818,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>116</v>
       </c>
@@ -2821,7 +2842,7 @@
       </c>
       <c r="H47" s="10"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>118</v>
       </c>
@@ -2843,9 +2864,11 @@
       <c r="G48" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H48" s="10"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H48" s="10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>120</v>
       </c>
@@ -2869,7 +2892,7 @@
       </c>
       <c r="H49" s="10"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>122</v>
       </c>
@@ -2893,7 +2916,7 @@
       </c>
       <c r="H50" s="10"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>124</v>
       </c>
@@ -2919,7 +2942,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>127</v>
       </c>
@@ -2945,7 +2968,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>129</v>
       </c>
@@ -2969,7 +2992,7 @@
       </c>
       <c r="H53" s="10"/>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>131</v>
       </c>
@@ -2995,7 +3018,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>135</v>
       </c>
@@ -3021,7 +3044,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>138</v>
       </c>
@@ -3047,7 +3070,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
         <v>259</v>
       </c>
@@ -3071,7 +3094,7 @@
       </c>
       <c r="H57" s="4"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
         <v>141</v>
       </c>
@@ -3097,7 +3120,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>144</v>
       </c>
@@ -3123,7 +3146,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>264</v>
       </c>
@@ -3147,7 +3170,7 @@
       </c>
       <c r="H60" s="4"/>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
         <v>261</v>
       </c>
@@ -3171,7 +3194,7 @@
       </c>
       <c r="H61" s="4"/>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>147</v>
       </c>
@@ -3197,7 +3220,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
         <v>256</v>
       </c>
@@ -3223,7 +3246,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
         <v>254</v>
       </c>
@@ -3249,7 +3272,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
         <v>150</v>
       </c>
@@ -3273,7 +3296,7 @@
       </c>
       <c r="H65" s="4"/>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
         <v>152</v>
       </c>
@@ -3299,7 +3322,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
         <v>155</v>
       </c>
@@ -3325,7 +3348,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
         <v>158</v>
       </c>
@@ -3349,7 +3372,7 @@
       </c>
       <c r="H68" s="4"/>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
         <v>160</v>
       </c>
@@ -3375,7 +3398,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
         <v>163</v>
       </c>
@@ -3399,7 +3422,7 @@
       </c>
       <c r="H70" s="4"/>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
         <v>165</v>
       </c>
@@ -3425,7 +3448,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
         <v>168</v>
       </c>
@@ -3449,7 +3472,7 @@
       </c>
       <c r="H72" s="4"/>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
         <v>170</v>
       </c>
@@ -3475,7 +3498,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
         <v>173</v>
       </c>
@@ -3501,7 +3524,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="4" t="s">
         <v>175</v>
       </c>
@@ -3527,7 +3550,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
         <v>177</v>
       </c>
@@ -3553,7 +3576,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="4" t="s">
         <v>180</v>
       </c>
@@ -3579,7 +3602,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
         <v>182</v>
       </c>
@@ -3605,7 +3628,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="4" t="s">
         <v>263</v>
       </c>
@@ -3631,7 +3654,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
         <v>185</v>
       </c>
@@ -3657,7 +3680,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
         <v>188</v>
       </c>
@@ -3681,7 +3704,7 @@
       </c>
       <c r="H81" s="4"/>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
         <v>190</v>
       </c>
@@ -3705,7 +3728,7 @@
       </c>
       <c r="H82" s="4"/>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="4" t="s">
         <v>192</v>
       </c>
@@ -3729,7 +3752,7 @@
       </c>
       <c r="H83" s="4"/>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
         <v>194</v>
       </c>
@@ -3755,7 +3778,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>196</v>
       </c>
@@ -3781,7 +3804,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
         <v>198</v>
       </c>
@@ -3805,7 +3828,7 @@
       </c>
       <c r="H86" s="4"/>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="4" t="s">
         <v>200</v>
       </c>
@@ -3829,7 +3852,7 @@
       </c>
       <c r="H87" s="4"/>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
         <v>202</v>
       </c>
@@ -3855,7 +3878,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
         <v>205</v>
       </c>
@@ -3881,7 +3904,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
         <v>208</v>
       </c>
@@ -3907,7 +3930,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="4" t="s">
         <v>210</v>
       </c>
@@ -3933,7 +3956,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
         <v>212</v>
       </c>
@@ -3957,7 +3980,7 @@
       </c>
       <c r="H92" s="4"/>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
         <v>214</v>
       </c>
@@ -3983,7 +4006,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
         <v>216</v>
       </c>
@@ -4007,7 +4030,7 @@
       </c>
       <c r="H94" s="4"/>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="4" t="s">
         <v>218</v>
       </c>
@@ -4033,7 +4056,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
         <v>220</v>
       </c>
@@ -4059,7 +4082,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="4" t="s">
         <v>223</v>
       </c>
@@ -4083,7 +4106,7 @@
       </c>
       <c r="H97" s="4"/>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
         <v>225</v>
       </c>
@@ -4109,7 +4132,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="4" t="s">
         <v>227</v>
       </c>
@@ -4133,7 +4156,7 @@
       </c>
       <c r="H99" s="4"/>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
         <v>229</v>
       </c>
@@ -4157,7 +4180,7 @@
       </c>
       <c r="H100" s="4"/>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="4" t="s">
         <v>231</v>
       </c>
@@ -4181,7 +4204,7 @@
       </c>
       <c r="H101" s="4"/>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
         <v>233</v>
       </c>
@@ -4207,7 +4230,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="4" t="s">
         <v>235</v>
       </c>
@@ -4231,7 +4254,7 @@
       </c>
       <c r="H103" s="4"/>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
         <v>237</v>
       </c>
@@ -4255,7 +4278,7 @@
       </c>
       <c r="H104" s="4"/>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="4" t="s">
         <v>239</v>
       </c>
@@ -4279,7 +4302,7 @@
       </c>
       <c r="H105" s="4"/>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
         <v>241</v>
       </c>
@@ -4303,7 +4326,7 @@
       </c>
       <c r="H106" s="4"/>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="4" t="s">
         <v>243</v>
       </c>
@@ -4327,7 +4350,7 @@
       </c>
       <c r="H107" s="4"/>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
         <v>245</v>
       </c>
@@ -4353,7 +4376,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="4" t="s">
         <v>247</v>
       </c>
@@ -4377,7 +4400,7 @@
       </c>
       <c r="H109" s="4"/>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
         <v>249</v>
       </c>
@@ -4403,7 +4426,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="4" t="s">
         <v>251</v>
       </c>

</xml_diff>

<commit_message>
Lanzar Beta-1.0.1 con nuevo escalado de habilidades.
Actualiza la version visible en vistas, documenta cambios en CHANGELOG y aplica la nueva formula de skill_power junto con ajustes de datos y migracion.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/resources/cartas.xlsx
+++ b/public/resources/cartas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09212922-2D36-4F2C-B74E-443F06F43B70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4156E30C-11D8-4F27-81D9-040D0138BD0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1522,7 +1522,7 @@
         <v>274</v>
       </c>
       <c r="M2" s="12">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="N2" s="12" t="s">
         <v>286</v>
@@ -1564,7 +1564,7 @@
         <v>275</v>
       </c>
       <c r="M3" s="13">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="N3" s="13" t="s">
         <v>286</v>
@@ -1606,7 +1606,7 @@
         <v>276</v>
       </c>
       <c r="M4" s="12">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="N4" s="12" t="s">
         <v>287</v>
@@ -1774,7 +1774,7 @@
         <v>293</v>
       </c>
       <c r="M8" s="12">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="N8" s="12" t="s">
         <v>287</v>
@@ -1816,7 +1816,7 @@
         <v>295</v>
       </c>
       <c r="M9" s="16">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="N9" s="16" t="s">
         <v>286</v>

</xml_diff>

<commit_message>
Actualizar archivos Excel de recursos del juego.
Se suben cartas.xlsx, desafios.xlsx y eventos.xlsx para alinear los datos locales con GitHub.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/resources/cartas.xlsx
+++ b/public/resources/cartas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4156E30C-11D8-4F27-81D9-040D0138BD0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A2A4E2B-157B-47BC-88A1-065B464F043B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="319">
   <si>
     <t>Nombre</t>
   </si>
@@ -974,6 +974,9 @@
   </si>
   <si>
     <t>Potencia @skill_power el bonus de afiliación aliado que esté activo</t>
+  </si>
+  <si>
+    <t>stun</t>
   </si>
 </sst>
 </file>
@@ -1431,10 +1434,10 @@
     <col min="3" max="3" width="5.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.42578125" customWidth="1"/>
+    <col min="6" max="6" width="94" customWidth="1"/>
     <col min="7" max="7" width="7.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="42.42578125" customWidth="1"/>
-    <col min="9" max="9" width="15.28515625" customWidth="1"/>
+    <col min="9" max="9" width="55.42578125" customWidth="1"/>
     <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="79.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -2009,6 +2012,9 @@
         <v>10</v>
       </c>
       <c r="H14" s="10"/>
+      <c r="L14" t="s">
+        <v>318</v>
+      </c>
     </row>
     <row r="15" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">

</xml_diff>

<commit_message>
Lanzar Beta-1.0.5 con ajustes de combate y UX de vistas.
Incluye la regla definitiva de tank (1 uso por partida salvo resurrección), reset de cooldown al revivir, rediseño de tablero, mejoras en desafíos/eventos y actualización de versión/changelog.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/resources/cartas.xlsx
+++ b/public/resources/cartas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{125390B1-8892-4930-9832-C74F3423C2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C445FE-36AA-4558-9EC1-D9D646A44837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1833" uniqueCount="761">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1832" uniqueCount="762">
   <si>
     <t>Nombre</t>
   </si>
@@ -1960,18 +1960,12 @@
     <t>Doble destino</t>
   </si>
   <si>
-    <t>Venom desatado</t>
-  </si>
-  <si>
     <t>Lázaro inmortal</t>
   </si>
   <si>
     <t>Revive una carta del cementerio y la devuelve al mazo.</t>
   </si>
   <si>
-    <t>Control vegetal</t>
-  </si>
-  <si>
     <t>Furia bestial</t>
   </si>
   <si>
@@ -2306,6 +2300,15 @@
   </si>
   <si>
     <t>https://i.pinimg.com/1200x/84/98/f6/8498f6f9f4b218a61bb9773d50aa946b.jpg</t>
+  </si>
+  <si>
+    <t>Ofrenda al verde</t>
+  </si>
+  <si>
+    <t>Toxina de Bane</t>
+  </si>
+  <si>
+    <t>Envenena al objetivo causando @skill_power de daño durante varios turnos.</t>
   </si>
 </sst>
 </file>
@@ -2438,7 +2441,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2497,12 +2500,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill>
@@ -2542,62 +2551,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFCC99FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF99CCFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF82D8B1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2906,7 +2859,7 @@
     <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="74.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.85546875" customWidth="1"/>
+    <col min="13" max="13" width="18.85546875" style="25" customWidth="1"/>
     <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2947,7 +2900,7 @@
       <c r="L1" s="11" t="s">
         <v>260</v>
       </c>
-      <c r="M1" s="11" t="s">
+      <c r="M1" s="9" t="s">
         <v>263</v>
       </c>
       <c r="N1" s="11" t="s">
@@ -3519,7 +3472,7 @@
         <v>501</v>
       </c>
       <c r="J15" s="14" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="K15" s="14" t="s">
         <v>289</v>
@@ -3599,7 +3552,7 @@
         <v>49</v>
       </c>
       <c r="J17" s="14" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="K17" s="14" t="s">
         <v>270</v>
@@ -3638,7 +3591,7 @@
       </c>
       <c r="H18" s="10"/>
       <c r="J18" s="12" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="K18" s="12" t="s">
         <v>298</v>
@@ -3685,7 +3638,7 @@
       <c r="L19" s="20" t="s">
         <v>273</v>
       </c>
-      <c r="M19" s="20" t="s">
+      <c r="M19" s="13" t="s">
         <v>274</v>
       </c>
       <c r="N19" s="20" t="s">
@@ -3724,7 +3677,7 @@
       <c r="L20" s="21" t="s">
         <v>268</v>
       </c>
-      <c r="M20" s="21">
+      <c r="M20" s="15">
         <v>1000</v>
       </c>
       <c r="N20" s="21" t="s">
@@ -3763,7 +3716,7 @@
       <c r="L21" s="21" t="s">
         <v>268</v>
       </c>
-      <c r="M21" s="21">
+      <c r="M21" s="15">
         <v>1000</v>
       </c>
       <c r="N21" s="21" t="s">
@@ -3841,7 +3794,7 @@
       <c r="L23" s="20" t="s">
         <v>292</v>
       </c>
-      <c r="M23" s="20" t="s">
+      <c r="M23" s="13" t="s">
         <v>294</v>
       </c>
       <c r="N23" s="20" t="s">
@@ -3993,7 +3946,7 @@
         <v>29</v>
       </c>
       <c r="J27" s="14" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="K27" s="14" t="s">
         <v>270</v>
@@ -4116,7 +4069,7 @@
         <v>73</v>
       </c>
       <c r="J30" s="22" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="K30" s="22" t="s">
         <v>295</v>
@@ -4360,7 +4313,7 @@
         <v>49</v>
       </c>
       <c r="J36" s="12" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="K36" s="12" t="s">
         <v>298</v>
@@ -4442,7 +4395,7 @@
         <v>344</v>
       </c>
       <c r="J38" s="22" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="K38" s="22" t="s">
         <v>295</v>
@@ -4725,7 +4678,7 @@
         <v>102</v>
       </c>
       <c r="J45" s="15" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="K45" s="15" t="s">
         <v>299</v>
@@ -4926,7 +4879,7 @@
         <v>341</v>
       </c>
       <c r="J50" s="12" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="K50" s="12" t="s">
         <v>297</v>
@@ -5008,7 +4961,7 @@
         <v>34</v>
       </c>
       <c r="J52" s="14" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="K52" s="14" t="s">
         <v>296</v>
@@ -5088,7 +5041,7 @@
       </c>
       <c r="H54" s="17"/>
       <c r="J54" s="12" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="K54" s="12" t="s">
         <v>297</v>
@@ -5773,7 +5726,7 @@
         <v>495</v>
       </c>
       <c r="J71" s="12" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="K71" s="12" t="s">
         <v>295</v>
@@ -6136,7 +6089,7 @@
       <c r="L80" s="21" t="s">
         <v>268</v>
       </c>
-      <c r="M80" s="21">
+      <c r="M80" s="15">
         <v>1000</v>
       </c>
       <c r="N80" s="21" t="s">
@@ -6175,7 +6128,7 @@
       <c r="L81" s="19" t="s">
         <v>532</v>
       </c>
-      <c r="M81" s="19" t="s">
+      <c r="M81" s="12" t="s">
         <v>534</v>
       </c>
       <c r="N81" s="19" t="s">
@@ -6214,7 +6167,7 @@
       <c r="L82" s="23" t="s">
         <v>265</v>
       </c>
-      <c r="M82" s="23">
+      <c r="M82" s="14">
         <v>100</v>
       </c>
       <c r="N82" s="23" t="s">
@@ -6255,7 +6208,7 @@
       <c r="L83" s="21" t="s">
         <v>268</v>
       </c>
-      <c r="M83" s="21">
+      <c r="M83" s="15">
         <v>1000</v>
       </c>
       <c r="N83" s="21" t="s">
@@ -6294,7 +6247,7 @@
       <c r="L84" s="20" t="s">
         <v>273</v>
       </c>
-      <c r="M84" s="20" t="s">
+      <c r="M84" s="13" t="s">
         <v>274</v>
       </c>
       <c r="N84" s="20" t="s">
@@ -6374,7 +6327,7 @@
       <c r="L86" s="20" t="s">
         <v>292</v>
       </c>
-      <c r="M86" s="20" t="s">
+      <c r="M86" s="13" t="s">
         <v>294</v>
       </c>
       <c r="N86" s="20" t="s">
@@ -6415,7 +6368,7 @@
       <c r="L87" s="23" t="s">
         <v>280</v>
       </c>
-      <c r="M87" s="23"/>
+      <c r="M87" s="14"/>
       <c r="N87" s="23" t="s">
         <v>271</v>
       </c>
@@ -6452,7 +6405,7 @@
       <c r="L88" s="20" t="s">
         <v>273</v>
       </c>
-      <c r="M88" s="20" t="s">
+      <c r="M88" s="13" t="s">
         <v>274</v>
       </c>
       <c r="N88" s="20" t="s">
@@ -6522,7 +6475,7 @@
         <v>343</v>
       </c>
       <c r="J90" s="12" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="K90" s="12" t="s">
         <v>297</v>
@@ -6563,7 +6516,7 @@
         <v>343</v>
       </c>
       <c r="J91" s="12" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="K91" s="12" t="s">
         <v>298</v>
@@ -6686,7 +6639,7 @@
         <v>110</v>
       </c>
       <c r="J94" s="12" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="K94" s="12" t="s">
         <v>295</v>
@@ -6733,7 +6686,7 @@
       <c r="L95" s="23" t="s">
         <v>265</v>
       </c>
-      <c r="M95" s="23">
+      <c r="M95" s="14">
         <v>100</v>
       </c>
       <c r="N95" s="23" t="s">
@@ -6774,7 +6727,7 @@
       <c r="L96" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="M96" s="2">
+      <c r="M96" s="24">
         <v>200</v>
       </c>
       <c r="N96" s="2" t="s">
@@ -6815,7 +6768,7 @@
       <c r="L97" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="M97" s="2"/>
+      <c r="M97" s="24"/>
       <c r="N97" s="2" t="s">
         <v>271</v>
       </c>
@@ -6854,7 +6807,7 @@
       <c r="L98" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M98" s="2">
+      <c r="M98" s="24">
         <v>100</v>
       </c>
       <c r="N98" s="2" t="s">
@@ -6895,7 +6848,7 @@
       <c r="L99" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="M99" s="2">
+      <c r="M99" s="24">
         <v>100</v>
       </c>
       <c r="N99" s="2" t="s">
@@ -6936,7 +6889,7 @@
       <c r="L100" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M100" s="2" t="s">
+      <c r="M100" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N100" s="2" t="s">
@@ -6975,7 +6928,7 @@
       <c r="L101" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M101" s="2">
+      <c r="M101" s="24">
         <v>100</v>
       </c>
       <c r="N101" s="2" t="s">
@@ -7014,7 +6967,7 @@
       <c r="L102" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M102" s="2" t="s">
+      <c r="M102" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N102" s="2" t="s">
@@ -7055,7 +7008,7 @@
       <c r="L103" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="M103" s="2">
+      <c r="M103" s="24">
         <v>100</v>
       </c>
       <c r="N103" s="2" t="s">
@@ -7096,7 +7049,7 @@
       <c r="L104" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="M104" s="2">
+      <c r="M104" s="24">
         <v>50</v>
       </c>
       <c r="N104" s="2" t="s">
@@ -7137,7 +7090,7 @@
       <c r="L105" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="M105" s="2">
+      <c r="M105" s="24">
         <v>1000</v>
       </c>
       <c r="N105" s="2" t="s">
@@ -7176,7 +7129,7 @@
       <c r="L106" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M106" s="2" t="s">
+      <c r="M106" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N106" s="2" t="s">
@@ -7217,7 +7170,7 @@
       <c r="L107" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M107" s="2" t="s">
+      <c r="M107" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N107" s="2" t="s">
@@ -7258,7 +7211,7 @@
       <c r="L108" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M108" s="2" t="s">
+      <c r="M108" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N108" s="2" t="s">
@@ -7297,7 +7250,7 @@
       <c r="L109" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="M109" s="2" t="s">
+      <c r="M109" s="24" t="s">
         <v>534</v>
       </c>
       <c r="N109" s="2" t="s">
@@ -7338,7 +7291,7 @@
       <c r="L110" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="M110" s="2">
+      <c r="M110" s="24">
         <v>200</v>
       </c>
       <c r="N110" s="2" t="s">
@@ -7377,7 +7330,7 @@
       <c r="L111" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M111" s="2">
+      <c r="M111" s="24">
         <v>100</v>
       </c>
       <c r="N111" s="2" t="s">
@@ -7418,7 +7371,7 @@
       <c r="L112" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="M112" s="2">
+      <c r="M112" s="24">
         <v>2</v>
       </c>
       <c r="N112" s="2" t="s">
@@ -7457,7 +7410,7 @@
       <c r="L113" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="M113" s="2">
+      <c r="M113" s="24">
         <v>50</v>
       </c>
       <c r="N113" s="2" t="s">
@@ -7498,7 +7451,7 @@
       <c r="L114" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M114" s="2" t="s">
+      <c r="M114" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N114" s="2" t="s">
@@ -7531,16 +7484,16 @@
         <v>167</v>
       </c>
       <c r="J115" s="2" t="s">
-        <v>645</v>
+        <v>760</v>
       </c>
       <c r="K115" s="2" t="s">
-        <v>578</v>
+        <v>761</v>
       </c>
       <c r="L115" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="M115" s="2" t="s">
-        <v>282</v>
+        <v>529</v>
+      </c>
+      <c r="M115" s="24">
+        <v>200</v>
       </c>
       <c r="N115" s="2" t="s">
         <v>272</v>
@@ -7572,15 +7525,15 @@
         <v>167</v>
       </c>
       <c r="J116" s="2" t="s">
+        <v>645</v>
+      </c>
+      <c r="K116" s="2" t="s">
         <v>646</v>
-      </c>
-      <c r="K116" s="2" t="s">
-        <v>647</v>
       </c>
       <c r="L116" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="M116" s="2">
+      <c r="M116" s="24">
         <v>1</v>
       </c>
       <c r="N116" s="2" t="s">
@@ -7613,7 +7566,7 @@
         <v>174</v>
       </c>
       <c r="J117" s="2" t="s">
-        <v>648</v>
+        <v>759</v>
       </c>
       <c r="K117" s="2" t="s">
         <v>575</v>
@@ -7621,7 +7574,7 @@
       <c r="L117" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="M117" s="2">
+      <c r="M117" s="24">
         <v>750</v>
       </c>
       <c r="N117" s="2" t="s">
@@ -7654,7 +7607,7 @@
         <v>149</v>
       </c>
       <c r="J118" s="2" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="K118" s="2" t="s">
         <v>628</v>
@@ -7662,7 +7615,7 @@
       <c r="L118" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M118" s="2" t="s">
+      <c r="M118" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N118" s="2" t="s">
@@ -7695,7 +7648,7 @@
         <v>179</v>
       </c>
       <c r="J119" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="K119" s="2" t="s">
         <v>628</v>
@@ -7703,7 +7656,7 @@
       <c r="L119" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M119" s="2" t="s">
+      <c r="M119" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N119" s="2" t="s">
@@ -7736,7 +7689,7 @@
         <v>179</v>
       </c>
       <c r="J120" s="2" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="K120" s="2" t="s">
         <v>618</v>
@@ -7744,7 +7697,7 @@
       <c r="L120" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M120" s="2" t="s">
+      <c r="M120" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N120" s="2" t="s">
@@ -7777,7 +7730,7 @@
         <v>182</v>
       </c>
       <c r="J121" s="2" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="K121" s="2" t="s">
         <v>628</v>
@@ -7785,7 +7738,7 @@
       <c r="L121" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M121" s="2" t="s">
+      <c r="M121" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N121" s="2" t="s">
@@ -7816,7 +7769,7 @@
       </c>
       <c r="H122" s="4"/>
       <c r="J122" s="2" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="K122" s="2" t="s">
         <v>578</v>
@@ -7824,7 +7777,7 @@
       <c r="L122" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="M122" s="2" t="s">
+      <c r="M122" s="24" t="s">
         <v>282</v>
       </c>
       <c r="N122" s="2" t="s">
@@ -7855,15 +7808,15 @@
       </c>
       <c r="H123" s="4"/>
       <c r="J123" s="2" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="K123" s="2" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="L123" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="M123" s="2" t="s">
+      <c r="M123" s="24" t="s">
         <v>534</v>
       </c>
       <c r="N123" s="2" t="s">
@@ -7894,7 +7847,7 @@
       </c>
       <c r="H124" s="4"/>
       <c r="J124" s="2" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="K124" s="2" t="s">
         <v>578</v>
@@ -7902,7 +7855,7 @@
       <c r="L124" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="M124" s="2" t="s">
+      <c r="M124" s="24" t="s">
         <v>282</v>
       </c>
       <c r="N124" s="2" t="s">
@@ -7935,7 +7888,7 @@
         <v>157</v>
       </c>
       <c r="J125" s="2" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="K125" s="2" t="s">
         <v>620</v>
@@ -7943,7 +7896,7 @@
       <c r="L125" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M125" s="2">
+      <c r="M125" s="24">
         <v>100</v>
       </c>
       <c r="N125" s="2" t="s">
@@ -7976,7 +7929,7 @@
         <v>135</v>
       </c>
       <c r="J126" s="2" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="K126" s="2" t="s">
         <v>580</v>
@@ -7984,7 +7937,7 @@
       <c r="L126" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="M126" s="2">
+      <c r="M126" s="24">
         <v>2</v>
       </c>
       <c r="N126" s="2" t="s">
@@ -8015,15 +7968,15 @@
       </c>
       <c r="H127" s="4"/>
       <c r="J127" s="2" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="K127" s="2" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="L127" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="M127" s="2">
+      <c r="M127" s="24">
         <v>200</v>
       </c>
       <c r="N127" s="2" t="s">
@@ -8054,15 +8007,15 @@
       </c>
       <c r="H128" s="4"/>
       <c r="J128" s="2" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="K128" s="2" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="L128" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="M128" s="2"/>
+      <c r="M128" s="24"/>
       <c r="N128" s="2" t="s">
         <v>271</v>
       </c>
@@ -8093,7 +8046,7 @@
         <v>199</v>
       </c>
       <c r="J129" s="2" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="K129" s="2" t="s">
         <v>628</v>
@@ -8101,7 +8054,7 @@
       <c r="L129" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M129" s="2" t="s">
+      <c r="M129" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N129" s="2" t="s">
@@ -8134,15 +8087,15 @@
         <v>202</v>
       </c>
       <c r="J130" s="2" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="K130" s="2" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="L130" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="M130" s="2">
+      <c r="M130" s="24">
         <v>1000</v>
       </c>
       <c r="N130" s="2" t="s">
@@ -8175,7 +8128,7 @@
         <v>141</v>
       </c>
       <c r="J131" s="2" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="K131" s="2" t="s">
         <v>580</v>
@@ -8183,7 +8136,7 @@
       <c r="L131" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="M131" s="2">
+      <c r="M131" s="24">
         <v>2</v>
       </c>
       <c r="N131" s="2" t="s">
@@ -8216,15 +8169,15 @@
         <v>182</v>
       </c>
       <c r="J132" s="2" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="K132" s="2" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="L132" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="M132" s="2">
+      <c r="M132" s="24">
         <v>200</v>
       </c>
       <c r="N132" s="2" t="s">
@@ -8255,7 +8208,7 @@
       </c>
       <c r="H133" s="4"/>
       <c r="J133" s="2" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="K133" s="2" t="s">
         <v>628</v>
@@ -8263,7 +8216,7 @@
       <c r="L133" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M133" s="2" t="s">
+      <c r="M133" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N133" s="2" t="s">
@@ -8296,7 +8249,7 @@
         <v>149</v>
       </c>
       <c r="J134" s="2" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="K134" s="2" t="s">
         <v>628</v>
@@ -8304,7 +8257,7 @@
       <c r="L134" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M134" s="2" t="s">
+      <c r="M134" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N134" s="2" t="s">
@@ -8335,15 +8288,15 @@
       </c>
       <c r="H135" s="4"/>
       <c r="J135" s="2" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="K135" s="2" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="L135" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="M135" s="2" t="s">
+      <c r="M135" s="24" t="s">
         <v>282</v>
       </c>
       <c r="N135" s="2" t="s">
@@ -8376,15 +8329,15 @@
         <v>179</v>
       </c>
       <c r="J136" s="2" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="K136" s="2" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="L136" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M136" s="2">
+      <c r="M136" s="24">
         <v>100</v>
       </c>
       <c r="N136" s="2" t="s">
@@ -8417,15 +8370,15 @@
         <v>217</v>
       </c>
       <c r="J137" s="2" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="K137" s="2" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="L137" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M137" s="2">
+      <c r="M137" s="24">
         <v>100</v>
       </c>
       <c r="N137" s="2" t="s">
@@ -8456,7 +8409,7 @@
       </c>
       <c r="H138" s="4"/>
       <c r="J138" s="2" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="K138" s="2" t="s">
         <v>580</v>
@@ -8464,7 +8417,7 @@
       <c r="L138" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="M138" s="2">
+      <c r="M138" s="24">
         <v>2</v>
       </c>
       <c r="N138" s="2" t="s">
@@ -8497,15 +8450,15 @@
         <v>141</v>
       </c>
       <c r="J139" s="2" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="K139" s="2" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="L139" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M139" s="2" t="s">
+      <c r="M139" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N139" s="2" t="s">
@@ -8536,15 +8489,15 @@
       </c>
       <c r="H140" s="4"/>
       <c r="J140" s="2" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="K140" s="2" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="L140" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="M140" s="2">
+      <c r="M140" s="24">
         <v>200</v>
       </c>
       <c r="N140" s="2" t="s">
@@ -8575,15 +8528,15 @@
       </c>
       <c r="H141" s="4"/>
       <c r="J141" s="2" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="K141" s="2" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="L141" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="M141" s="2" t="s">
+      <c r="M141" s="24" t="s">
         <v>534</v>
       </c>
       <c r="N141" s="2" t="s">
@@ -8616,15 +8569,15 @@
         <v>149</v>
       </c>
       <c r="J142" s="2" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="K142" s="2" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="L142" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M142" s="2" t="s">
+      <c r="M142" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N142" s="2" t="s">
@@ -8655,15 +8608,15 @@
       </c>
       <c r="H143" s="4"/>
       <c r="J143" s="2" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="K143" s="2" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="L143" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="M143" s="2">
+      <c r="M143" s="24">
         <v>200</v>
       </c>
       <c r="N143" s="2" t="s">
@@ -8694,15 +8647,15 @@
       </c>
       <c r="H144" s="4"/>
       <c r="J144" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="K144" s="2" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="L144" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="M144" s="2"/>
+      <c r="M144" s="24"/>
       <c r="N144" s="2" t="s">
         <v>271</v>
       </c>
@@ -8731,15 +8684,15 @@
       </c>
       <c r="H145" s="4"/>
       <c r="J145" s="2" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="K145" s="2" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="L145" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="M145" s="2" t="s">
+      <c r="M145" s="24" t="s">
         <v>534</v>
       </c>
       <c r="N145" s="2" t="s">
@@ -8770,15 +8723,15 @@
       </c>
       <c r="H146" s="4"/>
       <c r="J146" s="2" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="K146" s="2" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="L146" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M146" s="2" t="s">
+      <c r="M146" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N146" s="2" t="s">
@@ -8809,15 +8762,15 @@
       </c>
       <c r="H147" s="4"/>
       <c r="J147" s="2" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="K147" s="2" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="L147" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M147" s="2" t="s">
+      <c r="M147" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N147" s="2" t="s">
@@ -8850,15 +8803,15 @@
         <v>182</v>
       </c>
       <c r="J148" s="2" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="K148" s="2" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="L148" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="M148" s="2">
+      <c r="M148" s="24">
         <v>200</v>
       </c>
       <c r="N148" s="2" t="s">
@@ -8889,15 +8842,15 @@
       </c>
       <c r="H149" s="4"/>
       <c r="J149" s="2" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="K149" s="2" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="L149" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M149" s="2" t="s">
+      <c r="M149" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N149" s="2" t="s">
@@ -8930,15 +8883,15 @@
         <v>138</v>
       </c>
       <c r="J150" s="2" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="K150" s="2" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="L150" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M150" s="2">
+      <c r="M150" s="24">
         <v>100</v>
       </c>
       <c r="N150" s="2" t="s">
@@ -8969,15 +8922,15 @@
       </c>
       <c r="H151" s="4"/>
       <c r="J151" s="2" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="K151" s="2" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="L151" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="M151" s="2">
+      <c r="M151" s="24">
         <v>2</v>
       </c>
       <c r="N151" s="2" t="s">
@@ -9008,15 +8961,15 @@
       </c>
       <c r="H152" s="4"/>
       <c r="J152" s="2" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="K152" s="2" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="L152" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M152" s="2" t="s">
+      <c r="M152" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N152" s="2" t="s">
@@ -9047,7 +9000,7 @@
       </c>
       <c r="H153" s="4"/>
       <c r="J153" s="2" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="K153" s="2" t="s">
         <v>565</v>
@@ -9055,7 +9008,7 @@
       <c r="L153" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M153" s="2">
+      <c r="M153" s="24">
         <v>100</v>
       </c>
       <c r="N153" s="2" t="s">
@@ -9086,7 +9039,7 @@
       </c>
       <c r="H154" s="4"/>
       <c r="J154" s="2" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="K154" s="2" t="s">
         <v>618</v>
@@ -9094,7 +9047,7 @@
       <c r="L154" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M154" s="2" t="s">
+      <c r="M154" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N154" s="2" t="s">
@@ -9133,7 +9086,7 @@
       <c r="L155" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="M155" s="2">
+      <c r="M155" s="24">
         <v>50</v>
       </c>
       <c r="N155" s="2" t="s">
@@ -9164,7 +9117,7 @@
       </c>
       <c r="H156" s="4"/>
       <c r="J156" s="2" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="K156" s="2" t="s">
         <v>628</v>
@@ -9172,7 +9125,7 @@
       <c r="L156" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M156" s="2" t="s">
+      <c r="M156" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N156" s="2" t="s">
@@ -9203,7 +9156,7 @@
       </c>
       <c r="H157" s="4"/>
       <c r="J157" s="2" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="K157" s="2" t="s">
         <v>626</v>
@@ -9211,7 +9164,7 @@
       <c r="L157" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="M157" s="2">
+      <c r="M157" s="24">
         <v>100</v>
       </c>
       <c r="N157" s="2" t="s">
@@ -9242,7 +9195,7 @@
       </c>
       <c r="H158" s="4"/>
       <c r="J158" s="2" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="K158" s="2" t="s">
         <v>618</v>
@@ -9250,7 +9203,7 @@
       <c r="L158" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M158" s="2" t="s">
+      <c r="M158" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N158" s="2" t="s">
@@ -9281,15 +9234,15 @@
       </c>
       <c r="H159" s="4"/>
       <c r="J159" s="2" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="K159" s="2" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="L159" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="M159" s="2">
+      <c r="M159" s="24">
         <v>200</v>
       </c>
       <c r="N159" s="2" t="s">
@@ -9320,7 +9273,7 @@
       </c>
       <c r="H160" s="4"/>
       <c r="J160" s="2" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="K160" s="2" t="s">
         <v>628</v>
@@ -9328,7 +9281,7 @@
       <c r="L160" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M160" s="2" t="s">
+      <c r="M160" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N160" s="2" t="s">
@@ -9359,7 +9312,7 @@
       </c>
       <c r="H161" s="4"/>
       <c r="J161" s="2" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="K161" s="2" t="s">
         <v>610</v>
@@ -9367,7 +9320,7 @@
       <c r="L161" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M161" s="2">
+      <c r="M161" s="24">
         <v>100</v>
       </c>
       <c r="N161" s="2" t="s">
@@ -9398,7 +9351,7 @@
       </c>
       <c r="H162" s="4"/>
       <c r="J162" s="2" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="K162" s="2" t="s">
         <v>628</v>
@@ -9406,7 +9359,7 @@
       <c r="L162" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M162" s="2" t="s">
+      <c r="M162" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N162" s="2" t="s">
@@ -9439,7 +9392,7 @@
         <v>462</v>
       </c>
       <c r="J163" s="2" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="K163" s="2" t="s">
         <v>578</v>
@@ -9447,7 +9400,7 @@
       <c r="L163" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="M163" s="2" t="s">
+      <c r="M163" s="24" t="s">
         <v>282</v>
       </c>
       <c r="N163" s="2" t="s">
@@ -9478,15 +9431,15 @@
       </c>
       <c r="H164" s="4"/>
       <c r="J164" s="2" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="K164" s="2" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="L164" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M164" s="2">
+      <c r="M164" s="24">
         <v>100</v>
       </c>
       <c r="N164" s="2" t="s">
@@ -9517,15 +9470,15 @@
       </c>
       <c r="H165" s="4"/>
       <c r="J165" s="2" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="K165" s="2" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="L165" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="M165" s="2" t="s">
+      <c r="M165" s="24" t="s">
         <v>534</v>
       </c>
       <c r="N165" s="2" t="s">
@@ -9556,7 +9509,7 @@
       </c>
       <c r="H166" s="4"/>
       <c r="J166" s="2" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="K166" s="2" t="s">
         <v>600</v>
@@ -9564,7 +9517,7 @@
       <c r="L166" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="M166" s="2"/>
+      <c r="M166" s="24"/>
       <c r="N166" s="2" t="s">
         <v>271</v>
       </c>
@@ -9593,7 +9546,7 @@
       </c>
       <c r="H167" s="4"/>
       <c r="J167" s="2" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="K167" s="2" t="s">
         <v>628</v>
@@ -9601,7 +9554,7 @@
       <c r="L167" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M167" s="2" t="s">
+      <c r="M167" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N167" s="2" t="s">
@@ -9632,7 +9585,7 @@
       </c>
       <c r="H168" s="4"/>
       <c r="J168" s="2" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="K168" s="2" t="s">
         <v>618</v>
@@ -9640,7 +9593,7 @@
       <c r="L168" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M168" s="2" t="s">
+      <c r="M168" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N168" s="2" t="s">
@@ -9671,15 +9624,15 @@
       </c>
       <c r="H169" s="4"/>
       <c r="J169" s="2" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="K169" s="2" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="L169" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M169" s="2" t="s">
+      <c r="M169" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N169" s="2" t="s">
@@ -9710,15 +9663,15 @@
       </c>
       <c r="H170" s="4"/>
       <c r="J170" s="2" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="K170" s="2" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="L170" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="M170" s="2">
+      <c r="M170" s="24">
         <v>200</v>
       </c>
       <c r="N170" s="2" t="s">
@@ -9749,15 +9702,15 @@
       </c>
       <c r="H171" s="4"/>
       <c r="J171" s="2" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="K171" s="2" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="L171" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="M171" s="2"/>
+      <c r="M171" s="24"/>
       <c r="N171" s="2" t="s">
         <v>271</v>
       </c>
@@ -9796,7 +9749,7 @@
       <c r="L172" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M172" s="2" t="s">
+      <c r="M172" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N172" s="2" t="s">
@@ -9829,7 +9782,7 @@
         <v>462</v>
       </c>
       <c r="J173" s="2" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="K173" s="2" t="s">
         <v>618</v>
@@ -9837,7 +9790,7 @@
       <c r="L173" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M173" s="2" t="s">
+      <c r="M173" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N173" s="2" t="s">
@@ -9868,15 +9821,15 @@
       </c>
       <c r="H174" s="4"/>
       <c r="J174" s="2" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="K174" s="2" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="L174" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M174" s="2">
+      <c r="M174" s="24">
         <v>100</v>
       </c>
       <c r="N174" s="2" t="s">
@@ -9907,7 +9860,7 @@
       </c>
       <c r="H175" s="4"/>
       <c r="J175" s="2" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="K175" s="2" t="s">
         <v>589</v>
@@ -9915,7 +9868,7 @@
       <c r="L175" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="M175" s="2">
+      <c r="M175" s="24">
         <v>100</v>
       </c>
       <c r="N175" s="2" t="s">
@@ -9946,15 +9899,15 @@
       </c>
       <c r="H176" s="4"/>
       <c r="J176" s="2" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="K176" s="2" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="L176" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="M176" s="2" t="s">
+      <c r="M176" s="24" t="s">
         <v>534</v>
       </c>
       <c r="N176" s="2" t="s">
@@ -9985,15 +9938,15 @@
       </c>
       <c r="H177" s="4"/>
       <c r="J177" s="2" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="K177" s="2" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="L177" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="M177" s="2">
+      <c r="M177" s="24">
         <v>200</v>
       </c>
       <c r="N177" s="2" t="s">
@@ -10024,15 +9977,15 @@
       </c>
       <c r="H178" s="4"/>
       <c r="J178" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="K178" s="2" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="L178" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="M178" s="2"/>
+      <c r="M178" s="24"/>
       <c r="N178" s="2" t="s">
         <v>271</v>
       </c>
@@ -10061,7 +10014,7 @@
       </c>
       <c r="H179" s="4"/>
       <c r="J179" s="2" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="K179" s="2" t="s">
         <v>628</v>
@@ -10069,7 +10022,7 @@
       <c r="L179" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M179" s="2" t="s">
+      <c r="M179" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N179" s="2" t="s">
@@ -10102,15 +10055,15 @@
         <v>182</v>
       </c>
       <c r="J180" s="2" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="K180" s="2" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="L180" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="M180" s="2">
+      <c r="M180" s="24">
         <v>200</v>
       </c>
       <c r="N180" s="2" t="s">
@@ -10143,15 +10096,15 @@
         <v>182</v>
       </c>
       <c r="J181" s="2" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="K181" s="2" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="L181" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="M181" s="2" t="s">
+      <c r="M181" s="24" t="s">
         <v>282</v>
       </c>
       <c r="N181" s="2" t="s">
@@ -10182,7 +10135,7 @@
       </c>
       <c r="H182" s="4"/>
       <c r="J182" s="2" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="K182" s="2" t="s">
         <v>628</v>
@@ -10190,7 +10143,7 @@
       <c r="L182" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M182" s="2" t="s">
+      <c r="M182" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N182" s="2" t="s">
@@ -10221,7 +10174,7 @@
       </c>
       <c r="H183" s="4"/>
       <c r="J183" s="2" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="K183" s="2" t="s">
         <v>618</v>
@@ -10229,7 +10182,7 @@
       <c r="L183" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M183" s="2" t="s">
+      <c r="M183" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N183" s="2" t="s">
@@ -10260,15 +10213,15 @@
       </c>
       <c r="H184" s="4"/>
       <c r="J184" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="K184" s="2" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="L184" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="M184" s="2">
+      <c r="M184" s="24">
         <v>1</v>
       </c>
       <c r="N184" s="2" t="s">
@@ -10301,7 +10254,7 @@
         <v>179</v>
       </c>
       <c r="J185" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="K185" s="2" t="s">
         <v>628</v>
@@ -10309,7 +10262,7 @@
       <c r="L185" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M185" s="2" t="s">
+      <c r="M185" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N185" s="2" t="s">
@@ -10342,7 +10295,7 @@
         <v>179</v>
       </c>
       <c r="J186" s="2" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="K186" s="2" t="s">
         <v>628</v>
@@ -10350,7 +10303,7 @@
       <c r="L186" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M186" s="2" t="s">
+      <c r="M186" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N186" s="2" t="s">
@@ -10381,15 +10334,15 @@
       </c>
       <c r="H187" s="4"/>
       <c r="J187" s="2" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="K187" s="2" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="L187" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="M187" s="2" t="s">
+      <c r="M187" s="24" t="s">
         <v>534</v>
       </c>
       <c r="N187" s="2" t="s">
@@ -10420,15 +10373,15 @@
       </c>
       <c r="H188" s="4"/>
       <c r="J188" s="2" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="K188" s="2" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="L188" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M188" s="2">
+      <c r="M188" s="24">
         <v>100</v>
       </c>
       <c r="N188" s="2" t="s">
@@ -10461,7 +10414,7 @@
         <v>480</v>
       </c>
       <c r="J189" s="2" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="K189" s="2" t="s">
         <v>580</v>
@@ -10469,7 +10422,7 @@
       <c r="L189" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="M189" s="2">
+      <c r="M189" s="24">
         <v>2</v>
       </c>
       <c r="N189" s="2" t="s">
@@ -10505,12 +10458,12 @@
         <v>619</v>
       </c>
       <c r="K190" s="2" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="L190" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M190" s="2">
+      <c r="M190" s="24">
         <v>100</v>
       </c>
       <c r="N190" s="2" t="s">
@@ -10546,12 +10499,12 @@
         <v>566</v>
       </c>
       <c r="K191" s="2" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="L191" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M191" s="2">
+      <c r="M191" s="24">
         <v>100</v>
       </c>
       <c r="N191" s="2" t="s">
@@ -10584,15 +10537,15 @@
         <v>480</v>
       </c>
       <c r="J192" s="2" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="K192" s="2" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="L192" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="M192" s="2" t="s">
+      <c r="M192" s="24" t="s">
         <v>282</v>
       </c>
       <c r="N192" s="2" t="s">
@@ -10625,15 +10578,15 @@
         <v>480</v>
       </c>
       <c r="J193" s="2" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="K193" s="2" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="L193" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M193" s="2" t="s">
+      <c r="M193" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N193" s="2" t="s">
@@ -10666,7 +10619,7 @@
         <v>179</v>
       </c>
       <c r="J194" s="2" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="K194" s="2" t="s">
         <v>628</v>
@@ -10674,7 +10627,7 @@
       <c r="L194" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M194" s="2" t="s">
+      <c r="M194" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N194" s="2" t="s">
@@ -10698,7 +10651,7 @@
         <v>8</v>
       </c>
       <c r="F195" s="4" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="G195" s="4" t="s">
         <v>128</v>
@@ -10707,7 +10660,7 @@
         <v>179</v>
       </c>
       <c r="J195" s="2" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="K195" s="2" t="s">
         <v>628</v>
@@ -10715,7 +10668,7 @@
       <c r="L195" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M195" s="2" t="s">
+      <c r="M195" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N195" s="2" t="s">
@@ -10746,15 +10699,15 @@
       </c>
       <c r="H196" s="4"/>
       <c r="J196" s="2" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="K196" s="2" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="L196" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="M196" s="2" t="s">
+      <c r="M196" s="24" t="s">
         <v>534</v>
       </c>
       <c r="N196" s="2" t="s">
@@ -10785,15 +10738,15 @@
       </c>
       <c r="H197" s="4"/>
       <c r="J197" s="2" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="K197" s="2" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="L197" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="M197" s="2">
+      <c r="M197" s="24">
         <v>2</v>
       </c>
       <c r="N197" s="2" t="s">
@@ -10824,15 +10777,15 @@
       </c>
       <c r="H198" s="4"/>
       <c r="J198" s="2" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="K198" s="2" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="L198" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="M198" s="2" t="s">
+      <c r="M198" s="24" t="s">
         <v>274</v>
       </c>
       <c r="N198" s="2" t="s">
@@ -10865,7 +10818,7 @@
         <v>179</v>
       </c>
       <c r="J199" s="2" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="K199" s="2" t="s">
         <v>628</v>
@@ -10873,7 +10826,7 @@
       <c r="L199" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M199" s="2" t="s">
+      <c r="M199" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N199" s="2" t="s">
@@ -10904,15 +10857,15 @@
       </c>
       <c r="H200" s="4"/>
       <c r="J200" s="2" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="K200" s="2" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="L200" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="M200" s="2">
+      <c r="M200" s="24">
         <v>100</v>
       </c>
       <c r="N200" s="2" t="s">
@@ -10943,7 +10896,7 @@
       </c>
       <c r="H201" s="4"/>
       <c r="J201" s="2" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="K201" s="2" t="s">
         <v>575</v>
@@ -10951,7 +10904,7 @@
       <c r="L201" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="M201" s="2">
+      <c r="M201" s="24">
         <v>750</v>
       </c>
       <c r="N201" s="2" t="s">
@@ -10982,15 +10935,15 @@
       </c>
       <c r="H202" s="4"/>
       <c r="J202" s="2" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="K202" s="2" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="L202" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="M202" s="2"/>
+      <c r="M202" s="24"/>
       <c r="N202" s="2" t="s">
         <v>271</v>
       </c>
@@ -11019,7 +10972,7 @@
       </c>
       <c r="H203" s="4"/>
       <c r="J203" s="2" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="K203" s="2" t="s">
         <v>628</v>
@@ -11027,7 +10980,7 @@
       <c r="L203" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="M203" s="2" t="s">
+      <c r="M203" s="24" t="s">
         <v>294</v>
       </c>
       <c r="N203" s="2" t="s">

</xml_diff>

<commit_message>
Release Beta-1.0.10-03.05.26: evento cooperativo online vs BOT
Incluye sesión Socket.IO y revisiones en server.js, cliente multijugador, tablero coop (HTML/CSS/JS), partidaCoop con sincro de habilidades/AOE/fin de partida y robos desde mazo con mesa vacía. CHANGELOG, versión npm 1.0.10 y etiqueta lateral en cartas.js.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/cartas.xlsx
+++ b/public/resources/cartas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96293900-8D9A-4294-BBF8-1F68B884D5C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4E250D-0692-4A54-9091-57DCC9CA5CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2441,7 +2441,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2506,6 +2506,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -2854,7 +2855,7 @@
     <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="86.140625" customWidth="1"/>
     <col min="7" max="7" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="8" max="8" width="38" customWidth="1"/>
     <col min="9" max="9" width="5.5703125" customWidth="1"/>
     <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="74.7109375" bestFit="1" customWidth="1"/>
@@ -5874,7 +5875,7 @@
       <c r="E75" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="F75" s="1" t="s">
+      <c r="F75" s="26" t="s">
         <v>224</v>
       </c>
       <c r="G75" s="17" t="s">

</xml_diff>

<commit_message>
Release 1.0.2: misiones, boss, combate y recursos Excel
- Versión 1.0.2 en package.json, menú (cartas.js) y CHANGELOG.

- Misiones: cola serializada de track; conteo colección H/V y sobres con facción explícita.

- Misión boss: metadatos y coop; servidor y clientes leen variantes de columna boss.

- Combate: un solo ataque básico por confirmación; coop limpia selección al golpear al BOT.

- Servidor: fix getDoc en /update-user tras guardado.

- Actualiza cartas.xlsx, eventos.xlsx, eventos_online.xlsx, misiones_diarias.xlsx.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/cartas.xlsx
+++ b/public/resources/cartas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16CEEE0E-A733-4B10-A77A-548348CE4882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F2E8A1-5903-43E3-8852-8767327BA05D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2315" uniqueCount="945">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2319" uniqueCount="946">
   <si>
     <t>Nombre</t>
   </si>
@@ -2858,6 +2858,9 @@
   </si>
   <si>
     <t>https://i.ibb.co/20HYnX6v/Adamstrange.webp</t>
+  </si>
+  <si>
+    <t>Estimulante neuronal</t>
   </si>
 </sst>
 </file>
@@ -7734,7 +7737,7 @@
         <v>262</v>
       </c>
       <c r="M105" s="12">
-        <v>1250</v>
+        <v>1000</v>
       </c>
       <c r="N105" s="12" t="s">
         <v>268</v>
@@ -8388,11 +8391,21 @@
       <c r="H121" s="10" t="s">
         <v>922</v>
       </c>
-      <c r="J121" s="2"/>
-      <c r="K121" s="2"/>
-      <c r="L121" s="2"/>
-      <c r="M121" s="24"/>
-      <c r="N121" s="2"/>
+      <c r="J121" s="12" t="s">
+        <v>945</v>
+      </c>
+      <c r="K121" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="L121" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="M121" s="12">
+        <v>1000</v>
+      </c>
+      <c r="N121" s="12" t="s">
+        <v>268</v>
+      </c>
     </row>
     <row r="122" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="17" t="s">

</xml_diff>

<commit_message>
Release 1.1.0: objetos suprema/definitiva, tienda, mejorar cartas y catálogo
Incluye CHANGELOG, bump de versión en package.json y etiqueta del menú, cartas.xlsx e iconos nuevos. Ver CHANGELOG.md para el detalle.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/cartas.xlsx
+++ b/public/resources/cartas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{359C31A7-60AD-4B70-BE8D-C0BCE71668AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC11D6DC-86C6-411F-83DF-BE079354D21C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1345,9 +1345,6 @@
     <t>https://i.pinimg.com/736x/b8/ff/6d/b8ff6d771307cdfa3526bf5a55e8d407.jpg</t>
   </si>
   <si>
-    <t>https://i.pinimg.com/736x/07/7b/04/077b0409d32d20546af2b67a666d7a0d.jpg</t>
-  </si>
-  <si>
     <t>https://i.pinimg.com/736x/65/d2/21/65d221b257b9f7c1cfff9f3cedf471d2.jpg</t>
   </si>
   <si>
@@ -2861,6 +2858,9 @@
   </si>
   <si>
     <t>Estimulante neuronal</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/gMyfKdh3/Giganta-035.webp</t>
   </si>
 </sst>
 </file>
@@ -3531,10 +3531,10 @@
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="13" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="K2" s="13" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="L2" s="13" t="s">
         <v>288</v>
@@ -3573,10 +3573,10 @@
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="22" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="K3" s="22" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="L3" s="22" t="s">
         <v>275</v>
@@ -3615,10 +3615,10 @@
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="13" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="K4" s="13" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="L4" s="13" t="s">
         <v>269</v>
@@ -3657,7 +3657,7 @@
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="14" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="K5" s="14" t="s">
         <v>283</v>
@@ -3697,10 +3697,10 @@
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="15" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L6" s="15" t="s">
         <v>264</v>
@@ -3739,10 +3739,10 @@
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="13" t="s">
+        <v>499</v>
+      </c>
+      <c r="K7" s="13" t="s">
         <v>500</v>
-      </c>
-      <c r="K7" s="13" t="s">
-        <v>501</v>
       </c>
       <c r="L7" s="13" t="s">
         <v>288</v>
@@ -3781,10 +3781,10 @@
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="12" t="s">
+        <v>503</v>
+      </c>
+      <c r="K8" s="12" t="s">
         <v>504</v>
-      </c>
-      <c r="K8" s="12" t="s">
-        <v>505</v>
       </c>
       <c r="L8" s="12" t="s">
         <v>260</v>
@@ -3823,10 +3823,10 @@
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="14" t="s">
+        <v>501</v>
+      </c>
+      <c r="K9" s="14" t="s">
         <v>502</v>
-      </c>
-      <c r="K9" s="14" t="s">
-        <v>503</v>
       </c>
       <c r="L9" s="14" t="s">
         <v>261</v>
@@ -3855,20 +3855,20 @@
         <v>8</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="13" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="L10" s="13" t="s">
         <v>288</v>
@@ -3907,10 +3907,10 @@
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="13" t="s">
+        <v>522</v>
+      </c>
+      <c r="K11" s="13" t="s">
         <v>523</v>
-      </c>
-      <c r="K11" s="13" t="s">
-        <v>524</v>
       </c>
       <c r="L11" s="13" t="s">
         <v>288</v>
@@ -3949,10 +3949,10 @@
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="13" t="s">
+        <v>524</v>
+      </c>
+      <c r="K12" s="13" t="s">
         <v>525</v>
-      </c>
-      <c r="K12" s="13" t="s">
-        <v>526</v>
       </c>
       <c r="L12" s="13" t="s">
         <v>269</v>
@@ -4027,13 +4027,13 @@
         <v>10</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="J14" s="13" t="s">
         <v>289</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="L14" s="13" t="s">
         <v>288</v>
@@ -4062,19 +4062,19 @@
         <v>8</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="I15" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="J15" s="14" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="K15" s="14" t="s">
         <v>285</v>
@@ -4115,7 +4115,7 @@
         <v>47</v>
       </c>
       <c r="I16" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="J16" s="14" t="s">
         <v>282</v>
@@ -4157,7 +4157,7 @@
         <v>47</v>
       </c>
       <c r="J17" s="14" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="K17" s="14" t="s">
         <v>266</v>
@@ -4198,7 +4198,7 @@
         <v>47</v>
       </c>
       <c r="J18" s="12" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="K18" s="12" t="s">
         <v>294</v>
@@ -4237,10 +4237,10 @@
       </c>
       <c r="H19" s="10"/>
       <c r="J19" s="20" t="s">
+        <v>526</v>
+      </c>
+      <c r="K19" s="20" t="s">
         <v>527</v>
-      </c>
-      <c r="K19" s="20" t="s">
-        <v>528</v>
       </c>
       <c r="L19" s="20" t="s">
         <v>269</v>
@@ -4276,10 +4276,10 @@
       </c>
       <c r="H20" s="10"/>
       <c r="J20" s="21" t="s">
+        <v>528</v>
+      </c>
+      <c r="K20" s="21" t="s">
         <v>529</v>
-      </c>
-      <c r="K20" s="21" t="s">
-        <v>530</v>
       </c>
       <c r="L20" s="21" t="s">
         <v>264</v>
@@ -4315,10 +4315,10 @@
       </c>
       <c r="H21" s="10"/>
       <c r="J21" s="21" t="s">
+        <v>530</v>
+      </c>
+      <c r="K21" s="21" t="s">
         <v>531</v>
-      </c>
-      <c r="K21" s="21" t="s">
-        <v>532</v>
       </c>
       <c r="L21" s="21" t="s">
         <v>264</v>
@@ -4354,13 +4354,13 @@
       </c>
       <c r="H22" s="10"/>
       <c r="J22" s="18" t="s">
+        <v>516</v>
+      </c>
+      <c r="K22" s="18" t="s">
         <v>517</v>
       </c>
-      <c r="K22" s="18" t="s">
-        <v>518</v>
-      </c>
       <c r="L22" s="18" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M22" s="18">
         <v>200</v>
@@ -4393,10 +4393,10 @@
       </c>
       <c r="H23" s="10"/>
       <c r="J23" s="20" t="s">
+        <v>532</v>
+      </c>
+      <c r="K23" s="20" t="s">
         <v>533</v>
-      </c>
-      <c r="K23" s="20" t="s">
-        <v>534</v>
       </c>
       <c r="L23" s="20" t="s">
         <v>288</v>
@@ -4432,16 +4432,16 @@
       </c>
       <c r="H24" s="10"/>
       <c r="J24" s="12" t="s">
+        <v>534</v>
+      </c>
+      <c r="K24" s="12" t="s">
         <v>535</v>
       </c>
-      <c r="K24" s="12" t="s">
-        <v>536</v>
-      </c>
       <c r="L24" s="12" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="M24" s="12" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="N24" s="12" t="s">
         <v>267</v>
@@ -4471,10 +4471,10 @@
       </c>
       <c r="H25" s="10"/>
       <c r="J25" s="15" t="s">
+        <v>536</v>
+      </c>
+      <c r="K25" s="15" t="s">
         <v>537</v>
-      </c>
-      <c r="K25" s="15" t="s">
-        <v>538</v>
       </c>
       <c r="L25" s="15" t="s">
         <v>264</v>
@@ -4515,7 +4515,7 @@
         <v>289</v>
       </c>
       <c r="K26" s="13" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="L26" s="13" t="s">
         <v>288</v>
@@ -4553,7 +4553,7 @@
         <v>29</v>
       </c>
       <c r="J27" s="14" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="K27" s="14" t="s">
         <v>266</v>
@@ -4635,7 +4635,7 @@
         <v>255</v>
       </c>
       <c r="J29" s="13" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="K29" s="13" t="s">
         <v>272</v>
@@ -4676,7 +4676,7 @@
         <v>71</v>
       </c>
       <c r="J30" s="22" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="K30" s="22" t="s">
         <v>291</v>
@@ -4717,10 +4717,10 @@
         <v>71</v>
       </c>
       <c r="J31" s="14" t="s">
+        <v>509</v>
+      </c>
+      <c r="K31" s="14" t="s">
         <v>510</v>
-      </c>
-      <c r="K31" s="14" t="s">
-        <v>511</v>
       </c>
       <c r="L31" s="14" t="s">
         <v>261</v>
@@ -4761,7 +4761,7 @@
         <v>289</v>
       </c>
       <c r="K32" s="13" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="L32" s="13" t="s">
         <v>288</v>
@@ -4838,13 +4838,13 @@
       </c>
       <c r="H34" s="10"/>
       <c r="J34" s="18" t="s">
+        <v>538</v>
+      </c>
+      <c r="K34" s="18" t="s">
         <v>539</v>
       </c>
-      <c r="K34" s="18" t="s">
-        <v>540</v>
-      </c>
       <c r="L34" s="18" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M34" s="18">
         <v>200</v>
@@ -4879,10 +4879,10 @@
         <v>44</v>
       </c>
       <c r="J35" s="14" t="s">
+        <v>540</v>
+      </c>
+      <c r="K35" s="14" t="s">
         <v>541</v>
-      </c>
-      <c r="K35" s="14" t="s">
-        <v>542</v>
       </c>
       <c r="L35" s="14" t="s">
         <v>288</v>
@@ -4920,7 +4920,7 @@
         <v>47</v>
       </c>
       <c r="J36" s="12" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="K36" s="12" t="s">
         <v>294</v>
@@ -5002,7 +5002,7 @@
         <v>338</v>
       </c>
       <c r="J38" s="22" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="K38" s="22" t="s">
         <v>291</v>
@@ -5041,13 +5041,13 @@
       </c>
       <c r="H39" s="10"/>
       <c r="J39" s="18" t="s">
+        <v>516</v>
+      </c>
+      <c r="K39" s="18" t="s">
         <v>517</v>
       </c>
-      <c r="K39" s="18" t="s">
-        <v>518</v>
-      </c>
       <c r="L39" s="18" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M39" s="18">
         <v>200</v>
@@ -5080,10 +5080,10 @@
       </c>
       <c r="H40" s="10"/>
       <c r="J40" s="13" t="s">
+        <v>542</v>
+      </c>
+      <c r="K40" s="13" t="s">
         <v>543</v>
-      </c>
-      <c r="K40" s="13" t="s">
-        <v>544</v>
       </c>
       <c r="L40" s="13" t="s">
         <v>269</v>
@@ -5121,10 +5121,10 @@
         <v>71</v>
       </c>
       <c r="J41" s="13" t="s">
+        <v>544</v>
+      </c>
+      <c r="K41" s="13" t="s">
         <v>545</v>
-      </c>
-      <c r="K41" s="13" t="s">
-        <v>546</v>
       </c>
       <c r="L41" s="13" t="s">
         <v>288</v>
@@ -5162,10 +5162,10 @@
         <v>38</v>
       </c>
       <c r="J42" s="22" t="s">
+        <v>546</v>
+      </c>
+      <c r="K42" s="22" t="s">
         <v>547</v>
-      </c>
-      <c r="K42" s="22" t="s">
-        <v>548</v>
       </c>
       <c r="L42" s="22" t="s">
         <v>275</v>
@@ -5206,7 +5206,7 @@
         <v>289</v>
       </c>
       <c r="K43" s="13" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="L43" s="13" t="s">
         <v>288</v>
@@ -5244,10 +5244,10 @@
         <v>103</v>
       </c>
       <c r="J44" s="13" t="s">
+        <v>548</v>
+      </c>
+      <c r="K44" s="13" t="s">
         <v>549</v>
-      </c>
-      <c r="K44" s="13" t="s">
-        <v>550</v>
       </c>
       <c r="L44" s="13" t="s">
         <v>288</v>
@@ -5285,7 +5285,7 @@
         <v>100</v>
       </c>
       <c r="J45" s="15" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="K45" s="15" t="s">
         <v>295</v>
@@ -5302,7 +5302,7 @@
     </row>
     <row r="46" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B46" s="3">
         <v>1</v>
@@ -5317,7 +5317,7 @@
         <v>8</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="G46" s="10" t="s">
         <v>10</v>
@@ -5326,16 +5326,16 @@
         <v>108</v>
       </c>
       <c r="J46" s="19" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="K46" s="19" t="s">
+        <v>519</v>
+      </c>
+      <c r="L46" s="19" t="s">
+        <v>518</v>
+      </c>
+      <c r="M46" s="12" t="s">
         <v>520</v>
-      </c>
-      <c r="L46" s="19" t="s">
-        <v>519</v>
-      </c>
-      <c r="M46" s="12" t="s">
-        <v>521</v>
       </c>
       <c r="N46" s="19" t="s">
         <v>267</v>
@@ -5367,10 +5367,10 @@
         <v>108</v>
       </c>
       <c r="J47" s="14" t="s">
+        <v>550</v>
+      </c>
+      <c r="K47" s="14" t="s">
         <v>551</v>
-      </c>
-      <c r="K47" s="14" t="s">
-        <v>552</v>
       </c>
       <c r="L47" s="14" t="s">
         <v>261</v>
@@ -5405,13 +5405,13 @@
         <v>10</v>
       </c>
       <c r="H48" s="10" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="J48" s="14" t="s">
+        <v>552</v>
+      </c>
+      <c r="K48" s="14" t="s">
         <v>553</v>
-      </c>
-      <c r="K48" s="14" t="s">
-        <v>554</v>
       </c>
       <c r="L48" s="14" t="s">
         <v>261</v>
@@ -5446,7 +5446,7 @@
         <v>10</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="J49" s="15" t="s">
         <v>280</v>
@@ -5488,10 +5488,10 @@
       </c>
       <c r="H50" s="10"/>
       <c r="J50" s="13" t="s">
+        <v>554</v>
+      </c>
+      <c r="K50" s="13" t="s">
         <v>555</v>
-      </c>
-      <c r="K50" s="13" t="s">
-        <v>556</v>
       </c>
       <c r="L50" s="13" t="s">
         <v>288</v>
@@ -5520,7 +5520,7 @@
         <v>22</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G51" s="10" t="s">
         <v>10</v>
@@ -5529,10 +5529,10 @@
         <v>335</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="J51" s="12" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="K51" s="12" t="s">
         <v>293</v>
@@ -5614,7 +5614,7 @@
         <v>33</v>
       </c>
       <c r="J53" s="14" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="K53" s="14" t="s">
         <v>292</v>
@@ -5652,7 +5652,7 @@
         <v>10</v>
       </c>
       <c r="H54" s="10" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="J54" s="15" t="s">
         <v>280</v>
@@ -5694,7 +5694,7 @@
       </c>
       <c r="H55" s="17"/>
       <c r="J55" s="12" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="K55" s="12" t="s">
         <v>293</v>
@@ -5711,7 +5711,7 @@
     </row>
     <row r="56" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="17" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B56" s="17">
         <v>1</v>
@@ -5726,7 +5726,7 @@
         <v>19</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="G56" s="10" t="s">
         <v>10</v>
@@ -5735,10 +5735,10 @@
         <v>332</v>
       </c>
       <c r="J56" s="13" t="s">
+        <v>556</v>
+      </c>
+      <c r="K56" s="13" t="s">
         <v>557</v>
-      </c>
-      <c r="K56" s="13" t="s">
-        <v>558</v>
       </c>
       <c r="L56" s="13" t="s">
         <v>288</v>
@@ -5776,10 +5776,10 @@
         <v>332</v>
       </c>
       <c r="J57" s="13" t="s">
+        <v>558</v>
+      </c>
+      <c r="K57" s="13" t="s">
         <v>559</v>
-      </c>
-      <c r="K57" s="13" t="s">
-        <v>560</v>
       </c>
       <c r="L57" s="13" t="s">
         <v>269</v>
@@ -5817,10 +5817,10 @@
         <v>335</v>
       </c>
       <c r="J58" s="12" t="s">
+        <v>560</v>
+      </c>
+      <c r="K58" s="12" t="s">
         <v>561</v>
-      </c>
-      <c r="K58" s="12" t="s">
-        <v>562</v>
       </c>
       <c r="L58" s="12" t="s">
         <v>274</v>
@@ -5858,10 +5858,10 @@
         <v>71</v>
       </c>
       <c r="J59" s="14" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="K59" s="14" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="L59" s="14" t="s">
         <v>261</v>
@@ -5937,16 +5937,16 @@
         <v>10</v>
       </c>
       <c r="H61" s="10" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="I61" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="J61" s="15" t="s">
+        <v>563</v>
+      </c>
+      <c r="K61" s="15" t="s">
         <v>564</v>
-      </c>
-      <c r="K61" s="15" t="s">
-        <v>565</v>
       </c>
       <c r="L61" s="15" t="s">
         <v>277</v>
@@ -5982,10 +5982,10 @@
       </c>
       <c r="H62" s="17"/>
       <c r="J62" s="18" t="s">
+        <v>565</v>
+      </c>
+      <c r="K62" s="18" t="s">
         <v>566</v>
-      </c>
-      <c r="K62" s="18" t="s">
-        <v>567</v>
       </c>
       <c r="L62" s="18" t="s">
         <v>297</v>
@@ -6021,10 +6021,10 @@
       </c>
       <c r="H63" s="17"/>
       <c r="J63" s="13" t="s">
+        <v>567</v>
+      </c>
+      <c r="K63" s="13" t="s">
         <v>568</v>
-      </c>
-      <c r="K63" s="13" t="s">
-        <v>569</v>
       </c>
       <c r="L63" s="13" t="s">
         <v>269</v>
@@ -6062,13 +6062,13 @@
         <v>71</v>
       </c>
       <c r="J64" s="18" t="s">
+        <v>569</v>
+      </c>
+      <c r="K64" s="18" t="s">
         <v>570</v>
       </c>
-      <c r="K64" s="18" t="s">
-        <v>571</v>
-      </c>
       <c r="L64" s="18" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M64" s="18">
         <v>200</v>
@@ -6079,7 +6079,7 @@
     </row>
     <row r="65" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="17" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B65" s="17">
         <v>1</v>
@@ -6094,7 +6094,7 @@
         <v>22</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="G65" s="10" t="s">
         <v>10</v>
@@ -6103,10 +6103,10 @@
         <v>47</v>
       </c>
       <c r="J65" s="13" t="s">
+        <v>571</v>
+      </c>
+      <c r="K65" s="13" t="s">
         <v>572</v>
-      </c>
-      <c r="K65" s="13" t="s">
-        <v>573</v>
       </c>
       <c r="L65" s="13" t="s">
         <v>288</v>
@@ -6120,7 +6120,7 @@
     </row>
     <row r="66" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="17" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B66" s="17">
         <v>1</v>
@@ -6135,7 +6135,7 @@
         <v>22</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="G66" s="10" t="s">
         <v>10</v>
@@ -6185,10 +6185,10 @@
         <v>47</v>
       </c>
       <c r="J67" s="18" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="K67" s="18" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="L67" s="18" t="s">
         <v>297</v>
@@ -6202,7 +6202,7 @@
     </row>
     <row r="68" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="17" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="B68" s="17">
         <v>1</v>
@@ -6217,7 +6217,7 @@
         <v>8</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="G68" s="10" t="s">
         <v>10</v>
@@ -6226,10 +6226,10 @@
         <v>338</v>
       </c>
       <c r="J68" s="12" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="K68" s="12" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="L68" s="12" t="s">
         <v>274</v>
@@ -6267,10 +6267,10 @@
         <v>338</v>
       </c>
       <c r="J69" s="22" t="s">
+        <v>574</v>
+      </c>
+      <c r="K69" s="22" t="s">
         <v>575</v>
-      </c>
-      <c r="K69" s="22" t="s">
-        <v>576</v>
       </c>
       <c r="L69" s="22" t="s">
         <v>260</v>
@@ -6306,10 +6306,10 @@
       </c>
       <c r="H70" s="17"/>
       <c r="J70" s="12" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="K70" s="12" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="L70" s="12" t="s">
         <v>274</v>
@@ -6344,13 +6344,13 @@
         <v>10</v>
       </c>
       <c r="H71" s="10" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="J71" s="13" t="s">
+        <v>577</v>
+      </c>
+      <c r="K71" s="13" t="s">
         <v>578</v>
-      </c>
-      <c r="K71" s="13" t="s">
-        <v>579</v>
       </c>
       <c r="L71" s="13" t="s">
         <v>288</v>
@@ -6364,7 +6364,7 @@
     </row>
     <row r="72" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="17" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="B72" s="17">
         <v>1</v>
@@ -6379,7 +6379,7 @@
         <v>8</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="G72" s="10" t="s">
         <v>10</v>
@@ -6388,10 +6388,10 @@
         <v>335</v>
       </c>
       <c r="J72" s="12" t="s">
+        <v>579</v>
+      </c>
+      <c r="K72" s="12" t="s">
         <v>580</v>
-      </c>
-      <c r="K72" s="12" t="s">
-        <v>581</v>
       </c>
       <c r="L72" s="12" t="s">
         <v>262</v>
@@ -6426,10 +6426,10 @@
         <v>10</v>
       </c>
       <c r="H73" s="10" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="J73" s="12" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="K73" s="12" t="s">
         <v>291</v>
@@ -6446,7 +6446,7 @@
     </row>
     <row r="74" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="17" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="B74" s="17">
         <v>1</v>
@@ -6461,7 +6461,7 @@
         <v>8</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="G74" s="10" t="s">
         <v>10</v>
@@ -6470,10 +6470,10 @@
         <v>338</v>
       </c>
       <c r="J74" s="18" t="s">
+        <v>812</v>
+      </c>
+      <c r="K74" s="18" t="s">
         <v>813</v>
-      </c>
-      <c r="K74" s="18" t="s">
-        <v>814</v>
       </c>
       <c r="L74" s="18" t="s">
         <v>297</v>
@@ -6511,10 +6511,10 @@
         <v>338</v>
       </c>
       <c r="J75" s="15" t="s">
+        <v>581</v>
+      </c>
+      <c r="K75" s="15" t="s">
         <v>582</v>
-      </c>
-      <c r="K75" s="15" t="s">
-        <v>583</v>
       </c>
       <c r="L75" s="15" t="s">
         <v>264</v>
@@ -6550,10 +6550,10 @@
       </c>
       <c r="H76" s="17"/>
       <c r="J76" s="13" t="s">
+        <v>583</v>
+      </c>
+      <c r="K76" s="13" t="s">
         <v>584</v>
-      </c>
-      <c r="K76" s="13" t="s">
-        <v>585</v>
       </c>
       <c r="L76" s="13" t="s">
         <v>288</v>
@@ -6589,10 +6589,10 @@
       </c>
       <c r="H77" s="17"/>
       <c r="J77" s="14" t="s">
+        <v>585</v>
+      </c>
+      <c r="K77" s="14" t="s">
         <v>586</v>
-      </c>
-      <c r="K77" s="14" t="s">
-        <v>587</v>
       </c>
       <c r="L77" s="14" t="s">
         <v>276</v>
@@ -6628,13 +6628,13 @@
         <v>337</v>
       </c>
       <c r="I78" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="J78" s="12" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="K78" s="12" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="L78" s="12" t="s">
         <v>274</v>
@@ -6670,10 +6670,10 @@
       </c>
       <c r="H79" s="10"/>
       <c r="J79" s="18" t="s">
+        <v>513</v>
+      </c>
+      <c r="K79" s="18" t="s">
         <v>514</v>
-      </c>
-      <c r="K79" s="18" t="s">
-        <v>515</v>
       </c>
       <c r="L79" s="18" t="s">
         <v>297</v>
@@ -6711,16 +6711,16 @@
         <v>33</v>
       </c>
       <c r="J80" s="12" t="s">
+        <v>588</v>
+      </c>
+      <c r="K80" s="12" t="s">
         <v>589</v>
       </c>
-      <c r="K80" s="12" t="s">
-        <v>590</v>
-      </c>
       <c r="L80" s="12" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="M80" s="12" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="N80" s="12" t="s">
         <v>267</v>
@@ -6750,10 +6750,10 @@
       </c>
       <c r="H81" s="17"/>
       <c r="J81" s="14" t="s">
+        <v>590</v>
+      </c>
+      <c r="K81" s="14" t="s">
         <v>591</v>
-      </c>
-      <c r="K81" s="14" t="s">
-        <v>592</v>
       </c>
       <c r="L81" s="14" t="s">
         <v>261</v>
@@ -6789,10 +6789,10 @@
       </c>
       <c r="H82" s="17"/>
       <c r="J82" s="22" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="K82" s="22" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="L82" s="22" t="s">
         <v>260</v>
@@ -6827,13 +6827,13 @@
         <v>10</v>
       </c>
       <c r="H83" s="17" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="J83" s="21" t="s">
+        <v>593</v>
+      </c>
+      <c r="K83" s="21" t="s">
         <v>594</v>
-      </c>
-      <c r="K83" s="21" t="s">
-        <v>595</v>
       </c>
       <c r="L83" s="21" t="s">
         <v>264</v>
@@ -6869,16 +6869,16 @@
       </c>
       <c r="H84" s="17"/>
       <c r="J84" s="19" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="K84" s="19" t="s">
+        <v>519</v>
+      </c>
+      <c r="L84" s="19" t="s">
+        <v>518</v>
+      </c>
+      <c r="M84" s="12" t="s">
         <v>520</v>
-      </c>
-      <c r="L84" s="19" t="s">
-        <v>519</v>
-      </c>
-      <c r="M84" s="12" t="s">
-        <v>521</v>
       </c>
       <c r="N84" s="19" t="s">
         <v>267</v>
@@ -6908,10 +6908,10 @@
       </c>
       <c r="H85" s="17"/>
       <c r="J85" s="23" t="s">
+        <v>595</v>
+      </c>
+      <c r="K85" s="23" t="s">
         <v>596</v>
-      </c>
-      <c r="K85" s="23" t="s">
-        <v>597</v>
       </c>
       <c r="L85" s="23" t="s">
         <v>261</v>
@@ -6925,7 +6925,7 @@
     </row>
     <row r="86" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="17" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="B86" s="17">
         <v>1</v>
@@ -6940,7 +6940,7 @@
         <v>8</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="G86" s="10" t="s">
         <v>10</v>
@@ -6949,13 +6949,13 @@
         <v>338</v>
       </c>
       <c r="I86" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="J86" s="13" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="K86" s="13" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="L86" s="13" t="s">
         <v>288</v>
@@ -6969,7 +6969,7 @@
     </row>
     <row r="87" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="17" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="B87" s="17">
         <v>1</v>
@@ -6984,7 +6984,7 @@
         <v>8</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="G87" s="10" t="s">
         <v>10</v>
@@ -6993,13 +6993,13 @@
         <v>338</v>
       </c>
       <c r="I87" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="J87" s="18" t="s">
+        <v>848</v>
+      </c>
+      <c r="K87" s="18" t="s">
         <v>849</v>
-      </c>
-      <c r="K87" s="18" t="s">
-        <v>850</v>
       </c>
       <c r="L87" s="18" t="s">
         <v>297</v>
@@ -7037,10 +7037,10 @@
         <v>338</v>
       </c>
       <c r="J88" s="21" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="K88" s="21" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="L88" s="21" t="s">
         <v>264</v>
@@ -7054,7 +7054,7 @@
     </row>
     <row r="89" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="17" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="B89" s="17">
         <v>1</v>
@@ -7069,19 +7069,19 @@
         <v>19</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="G89" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H89" s="10" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="J89" s="20" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="K89" s="20" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="L89" s="20" t="s">
         <v>288</v>
@@ -7095,7 +7095,7 @@
     </row>
     <row r="90" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="17" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="B90" s="17">
         <v>1</v>
@@ -7110,19 +7110,19 @@
         <v>19</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="G90" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H90" s="10" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="J90" s="18" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="K90" s="18" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="L90" s="18" t="s">
         <v>297</v>
@@ -7136,7 +7136,7 @@
     </row>
     <row r="91" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="17" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="B91" s="17">
         <v>1</v>
@@ -7151,17 +7151,17 @@
         <v>8</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="G91" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H91" s="10"/>
       <c r="J91" s="18" t="s">
+        <v>931</v>
+      </c>
+      <c r="K91" s="18" t="s">
         <v>932</v>
-      </c>
-      <c r="K91" s="18" t="s">
-        <v>933</v>
       </c>
       <c r="L91" s="18" t="s">
         <v>297</v>
@@ -7196,13 +7196,13 @@
         <v>10</v>
       </c>
       <c r="H92" s="10" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="J92" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="K92" s="20" t="s">
         <v>599</v>
-      </c>
-      <c r="K92" s="20" t="s">
-        <v>600</v>
       </c>
       <c r="L92" s="20" t="s">
         <v>269</v>
@@ -7216,7 +7216,7 @@
     </row>
     <row r="93" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="17" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B93" s="17">
         <v>1</v>
@@ -7231,7 +7231,7 @@
         <v>19</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="G93" s="10" t="s">
         <v>10</v>
@@ -7240,10 +7240,10 @@
         <v>71</v>
       </c>
       <c r="J93" s="21" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="K93" s="21" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="L93" s="21" t="s">
         <v>264</v>
@@ -7272,7 +7272,7 @@
         <v>19</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="G94" s="10" t="s">
         <v>10</v>
@@ -7284,10 +7284,10 @@
         <v>375</v>
       </c>
       <c r="J94" s="18" t="s">
+        <v>511</v>
+      </c>
+      <c r="K94" s="18" t="s">
         <v>512</v>
-      </c>
-      <c r="K94" s="18" t="s">
-        <v>513</v>
       </c>
       <c r="L94" s="18" t="s">
         <v>297</v>
@@ -7323,10 +7323,10 @@
       </c>
       <c r="H95" s="17"/>
       <c r="J95" s="20" t="s">
+        <v>600</v>
+      </c>
+      <c r="K95" s="20" t="s">
         <v>601</v>
-      </c>
-      <c r="K95" s="20" t="s">
-        <v>602</v>
       </c>
       <c r="L95" s="20" t="s">
         <v>288</v>
@@ -7364,10 +7364,10 @@
         <v>71</v>
       </c>
       <c r="J96" s="23" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="K96" s="23" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="L96" s="23" t="s">
         <v>276</v>
@@ -7401,10 +7401,10 @@
       </c>
       <c r="H97" s="17"/>
       <c r="J97" s="20" t="s">
+        <v>603</v>
+      </c>
+      <c r="K97" s="20" t="s">
         <v>604</v>
-      </c>
-      <c r="K97" s="20" t="s">
-        <v>605</v>
       </c>
       <c r="L97" s="20" t="s">
         <v>269</v>
@@ -7455,7 +7455,7 @@
     </row>
     <row r="99" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="17" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="B99" s="17">
         <v>1</v>
@@ -7470,25 +7470,25 @@
         <v>22</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="G99" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H99" s="17" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="J99" s="19" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="K99" s="19" t="s">
+        <v>519</v>
+      </c>
+      <c r="L99" s="19" t="s">
+        <v>518</v>
+      </c>
+      <c r="M99" s="12" t="s">
         <v>520</v>
-      </c>
-      <c r="L99" s="19" t="s">
-        <v>519</v>
-      </c>
-      <c r="M99" s="12" t="s">
-        <v>521</v>
       </c>
       <c r="N99" s="19" t="s">
         <v>267</v>
@@ -7496,7 +7496,7 @@
     </row>
     <row r="100" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="17" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="B100" s="17">
         <v>1</v>
@@ -7511,16 +7511,16 @@
         <v>8</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="G100" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H100" s="17" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="J100" s="14" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="K100" s="14" t="s">
         <v>285</v>
@@ -7537,7 +7537,7 @@
     </row>
     <row r="101" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="17" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="B101" s="17">
         <v>1</v>
@@ -7552,19 +7552,19 @@
         <v>22</v>
       </c>
       <c r="F101" s="1" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="G101" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H101" s="17" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="J101" s="18" t="s">
+        <v>777</v>
+      </c>
+      <c r="K101" s="18" t="s">
         <v>778</v>
-      </c>
-      <c r="K101" s="18" t="s">
-        <v>779</v>
       </c>
       <c r="L101" s="18" t="s">
         <v>297</v>
@@ -7578,7 +7578,7 @@
     </row>
     <row r="102" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="17" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B102" s="17">
         <v>1</v>
@@ -7593,16 +7593,16 @@
         <v>22</v>
       </c>
       <c r="F102" s="1" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="G102" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H102" s="17" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="J102" s="15" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="K102" s="15" t="s">
         <v>279</v>
@@ -7619,7 +7619,7 @@
     </row>
     <row r="103" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="17" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="B103" s="17">
         <v>1</v>
@@ -7634,16 +7634,16 @@
         <v>22</v>
       </c>
       <c r="F103" s="1" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="G103" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H103" s="17" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="J103" s="12" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="K103" s="12" t="s">
         <v>294</v>
@@ -7660,7 +7660,7 @@
     </row>
     <row r="104" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="17" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="B104" s="17">
         <v>1</v>
@@ -7675,19 +7675,19 @@
         <v>22</v>
       </c>
       <c r="F104" s="1" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="G104" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H104" s="17" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="I104" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="J104" s="13" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="K104" s="13" t="s">
         <v>272</v>
@@ -7725,10 +7725,10 @@
         <v>10</v>
       </c>
       <c r="H105" s="17" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="J105" s="12" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="K105" s="12" t="s">
         <v>293</v>
@@ -7745,7 +7745,7 @@
     </row>
     <row r="106" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="17" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="B106" s="17">
         <v>1</v>
@@ -7760,19 +7760,19 @@
         <v>22</v>
       </c>
       <c r="F106" s="1" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="G106" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H106" s="17" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="J106" s="23" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="K106" s="23" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="L106" s="23" t="s">
         <v>261</v>
@@ -7786,7 +7786,7 @@
     </row>
     <row r="107" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="17" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="B107" s="17">
         <v>1</v>
@@ -7801,22 +7801,22 @@
         <v>22</v>
       </c>
       <c r="F107" s="1" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="G107" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H107" s="17" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="J107" s="2" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="K107" s="2" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="L107" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M107" s="24">
         <v>200</v>
@@ -7827,7 +7827,7 @@
     </row>
     <row r="108" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="17" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="B108" s="17">
         <v>1</v>
@@ -7842,7 +7842,7 @@
         <v>22</v>
       </c>
       <c r="F108" s="1" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="G108" s="10" t="s">
         <v>10</v>
@@ -7851,7 +7851,7 @@
         <v>337</v>
       </c>
       <c r="J108" s="15" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="K108" s="15" t="s">
         <v>279</v>
@@ -7868,7 +7868,7 @@
     </row>
     <row r="109" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="17" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B109" s="17">
         <v>1</v>
@@ -7883,7 +7883,7 @@
         <v>22</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="G109" s="10" t="s">
         <v>10</v>
@@ -7892,10 +7892,10 @@
         <v>337</v>
       </c>
       <c r="J109" s="2" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="K109" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="L109" s="2" t="s">
         <v>260</v>
@@ -7909,7 +7909,7 @@
     </row>
     <row r="110" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="17" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="B110" s="17">
         <v>1</v>
@@ -7930,13 +7930,13 @@
         <v>10</v>
       </c>
       <c r="H110" s="17" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="I110" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="J110" s="12" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="K110" s="12" t="s">
         <v>294</v>
@@ -7977,7 +7977,7 @@
         <v>108</v>
       </c>
       <c r="I111" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="J111" s="15" t="s">
         <v>280</v>
@@ -8012,7 +8012,7 @@
         <v>8</v>
       </c>
       <c r="F112" s="1" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="G112" s="10" t="s">
         <v>10</v>
@@ -8038,7 +8038,7 @@
     </row>
     <row r="113" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="17" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="B113" s="17">
         <v>1</v>
@@ -8053,7 +8053,7 @@
         <v>8</v>
       </c>
       <c r="F113" s="1" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="G113" s="10" t="s">
         <v>10</v>
@@ -8062,10 +8062,10 @@
         <v>108</v>
       </c>
       <c r="J113" s="20" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="K113" s="20" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="L113" s="20" t="s">
         <v>288</v>
@@ -8079,7 +8079,7 @@
     </row>
     <row r="114" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="17" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="B114" s="17">
         <v>1</v>
@@ -8094,20 +8094,20 @@
         <v>8</v>
       </c>
       <c r="F114" s="1" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="G114" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H114" s="10"/>
       <c r="J114" s="2" t="s">
+        <v>939</v>
+      </c>
+      <c r="K114" s="2" t="s">
         <v>940</v>
       </c>
-      <c r="K114" s="2" t="s">
-        <v>941</v>
-      </c>
       <c r="L114" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M114" s="24">
         <v>200</v>
@@ -8142,7 +8142,7 @@
         <v>108</v>
       </c>
       <c r="J115" s="12" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="K115" s="12" t="s">
         <v>291</v>
@@ -8159,7 +8159,7 @@
     </row>
     <row r="116" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="17" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="B116" s="17">
         <v>1</v>
@@ -8174,22 +8174,22 @@
         <v>22</v>
       </c>
       <c r="F116" s="1" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="G116" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H116" s="10" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="I116" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="J116" s="21" t="s">
+        <v>750</v>
+      </c>
+      <c r="K116" s="21" t="s">
         <v>751</v>
-      </c>
-      <c r="K116" s="21" t="s">
-        <v>752</v>
       </c>
       <c r="L116" s="21" t="s">
         <v>264</v>
@@ -8203,7 +8203,7 @@
     </row>
     <row r="117" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="17" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="B117" s="17">
         <v>1</v>
@@ -8218,19 +8218,19 @@
         <v>8</v>
       </c>
       <c r="F117" s="1" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G117" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H117" s="10" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="I117" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="J117" s="13" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="K117" s="13" t="s">
         <v>272</v>
@@ -8247,7 +8247,7 @@
     </row>
     <row r="118" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="17" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="B118" s="17">
         <v>1</v>
@@ -8262,25 +8262,25 @@
         <v>8</v>
       </c>
       <c r="F118" s="1" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="G118" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H118" s="10" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="J118" s="2" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="K118" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="L118" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="M118" s="24" t="s">
         <v>520</v>
-      </c>
-      <c r="L118" s="2" t="s">
-        <v>519</v>
-      </c>
-      <c r="M118" s="24" t="s">
-        <v>521</v>
       </c>
       <c r="N118" s="2" t="s">
         <v>267</v>
@@ -8288,7 +8288,7 @@
     </row>
     <row r="119" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="17" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="B119" s="17">
         <v>1</v>
@@ -8303,19 +8303,19 @@
         <v>8</v>
       </c>
       <c r="F119" s="1" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="G119" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H119" s="10" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="J119" s="23" t="s">
+        <v>605</v>
+      </c>
+      <c r="K119" s="23" t="s">
         <v>606</v>
-      </c>
-      <c r="K119" s="23" t="s">
-        <v>607</v>
       </c>
       <c r="L119" s="23" t="s">
         <v>261</v>
@@ -8329,7 +8329,7 @@
     </row>
     <row r="120" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="17" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="B120" s="17">
         <v>1</v>
@@ -8344,16 +8344,16 @@
         <v>8</v>
       </c>
       <c r="F120" s="1" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="G120" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H120" s="10" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="J120" s="2" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="K120" s="2" t="s">
         <v>283</v>
@@ -8368,7 +8368,7 @@
     </row>
     <row r="121" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="17" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="B121" s="17">
         <v>1</v>
@@ -8383,16 +8383,16 @@
         <v>19</v>
       </c>
       <c r="F121" s="1" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="G121" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H121" s="10" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="J121" s="12" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="K121" s="12" t="s">
         <v>293</v>
@@ -8409,7 +8409,7 @@
     </row>
     <row r="122" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="17" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B122" s="17">
         <v>1</v>
@@ -8424,16 +8424,16 @@
         <v>8</v>
       </c>
       <c r="F122" s="1" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="G122" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H122" s="10" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="J122" s="13" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="K122" s="13" t="s">
         <v>272</v>
@@ -8450,7 +8450,7 @@
     </row>
     <row r="123" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="17" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="B123" s="17">
         <v>1</v>
@@ -8465,16 +8465,16 @@
         <v>8</v>
       </c>
       <c r="F123" s="1" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="G123" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H123" s="10" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="J123" s="15" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="K123" s="15" t="s">
         <v>279</v>
@@ -8506,19 +8506,19 @@
         <v>8</v>
       </c>
       <c r="F124" s="1" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="G124" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H124" s="10" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="J124" s="2" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="K124" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="L124" s="2" t="s">
         <v>260</v>
@@ -8532,7 +8532,7 @@
     </row>
     <row r="125" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="17" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="B125" s="17">
         <v>1</v>
@@ -8547,19 +8547,19 @@
         <v>8</v>
       </c>
       <c r="F125" s="1" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="G125" s="10" t="s">
         <v>10</v>
       </c>
       <c r="H125" s="10" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="J125" s="2" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="K125" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="L125" s="2" t="s">
         <v>269</v>
@@ -8595,10 +8595,10 @@
       </c>
       <c r="H126" s="10"/>
       <c r="J126" s="23" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="K126" s="23" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="L126" s="23" t="s">
         <v>261</v>
@@ -8636,13 +8636,13 @@
         <v>126</v>
       </c>
       <c r="J127" s="2" t="s">
+        <v>607</v>
+      </c>
+      <c r="K127" s="2" t="s">
         <v>608</v>
       </c>
-      <c r="K127" s="2" t="s">
-        <v>609</v>
-      </c>
       <c r="L127" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M127" s="24">
         <v>200</v>
@@ -8677,7 +8677,7 @@
         <v>129</v>
       </c>
       <c r="J128" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="K128" s="2" t="s">
         <v>283</v>
@@ -8713,13 +8713,13 @@
         <v>125</v>
       </c>
       <c r="H129" s="4" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="J129" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="K129" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="L129" s="2" t="s">
         <v>261</v>
@@ -8757,10 +8757,10 @@
         <v>135</v>
       </c>
       <c r="J130" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="K130" s="2" t="s">
         <v>612</v>
-      </c>
-      <c r="K130" s="2" t="s">
-        <v>613</v>
       </c>
       <c r="L130" s="2" t="s">
         <v>260</v>
@@ -8798,10 +8798,10 @@
         <v>138</v>
       </c>
       <c r="J131" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="K131" s="2" t="s">
         <v>614</v>
-      </c>
-      <c r="K131" s="2" t="s">
-        <v>615</v>
       </c>
       <c r="L131" s="2" t="s">
         <v>288</v>
@@ -8837,10 +8837,10 @@
       </c>
       <c r="H132" s="4"/>
       <c r="J132" s="2" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="K132" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="L132" s="2" t="s">
         <v>261</v>
@@ -8876,10 +8876,10 @@
       </c>
       <c r="H133" s="4"/>
       <c r="J133" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="K133" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="L133" s="2" t="s">
         <v>269</v>
@@ -8917,10 +8917,10 @@
         <v>141</v>
       </c>
       <c r="J134" s="2" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="K134" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="L134" s="2" t="s">
         <v>260</v>
@@ -8949,7 +8949,7 @@
         <v>22</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="G135" s="4" t="s">
         <v>125</v>
@@ -8958,10 +8958,10 @@
         <v>213</v>
       </c>
       <c r="J135" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="K135" s="2" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="L135" s="2" t="s">
         <v>275</v>
@@ -8975,7 +8975,7 @@
     </row>
     <row r="136" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="B136" s="4">
         <v>1</v>
@@ -8990,7 +8990,7 @@
         <v>22</v>
       </c>
       <c r="F136" s="4" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="G136" s="4" t="s">
         <v>125</v>
@@ -8999,7 +8999,7 @@
         <v>213</v>
       </c>
       <c r="J136" s="2" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="K136" s="2" t="s">
         <v>283</v>
@@ -9014,7 +9014,7 @@
     </row>
     <row r="137" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="4" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B137" s="4">
         <v>1</v>
@@ -9029,7 +9029,7 @@
         <v>22</v>
       </c>
       <c r="F137" s="4" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="G137" s="4" t="s">
         <v>125</v>
@@ -9038,7 +9038,7 @@
         <v>213</v>
       </c>
       <c r="J137" s="14" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="K137" s="14" t="s">
         <v>285</v>
@@ -9079,10 +9079,10 @@
         <v>213</v>
       </c>
       <c r="J138" s="2" t="s">
+        <v>619</v>
+      </c>
+      <c r="K138" s="2" t="s">
         <v>620</v>
-      </c>
-      <c r="K138" s="2" t="s">
-        <v>621</v>
       </c>
       <c r="L138" s="2" t="s">
         <v>264</v>
@@ -9118,10 +9118,10 @@
       </c>
       <c r="H139" s="4"/>
       <c r="J139" s="2" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="K139" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L139" s="2" t="s">
         <v>288</v>
@@ -9159,10 +9159,10 @@
         <v>146</v>
       </c>
       <c r="J140" s="2" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="K140" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L140" s="2" t="s">
         <v>288</v>
@@ -9200,10 +9200,10 @@
         <v>149</v>
       </c>
       <c r="J141" s="2" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="K141" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="L141" s="2" t="s">
         <v>269</v>
@@ -9239,16 +9239,16 @@
       </c>
       <c r="H142" s="4"/>
       <c r="J142" s="2" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="K142" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="L142" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="M142" s="24" t="s">
         <v>520</v>
-      </c>
-      <c r="L142" s="2" t="s">
-        <v>519</v>
-      </c>
-      <c r="M142" s="24" t="s">
-        <v>521</v>
       </c>
       <c r="N142" s="2" t="s">
         <v>267</v>
@@ -9280,13 +9280,13 @@
         <v>154</v>
       </c>
       <c r="J143" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="K143" s="2" t="s">
         <v>626</v>
       </c>
-      <c r="K143" s="2" t="s">
-        <v>627</v>
-      </c>
       <c r="L143" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M143" s="24">
         <v>200</v>
@@ -9319,10 +9319,10 @@
       </c>
       <c r="H144" s="4"/>
       <c r="J144" s="2" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="K144" s="2" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="L144" s="2" t="s">
         <v>261</v>
@@ -9360,10 +9360,10 @@
         <v>159</v>
       </c>
       <c r="J145" s="2" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="K145" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="L145" s="2" t="s">
         <v>297</v>
@@ -9399,10 +9399,10 @@
       </c>
       <c r="H146" s="4"/>
       <c r="J146" s="2" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="K146" s="2" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="L146" s="2" t="s">
         <v>275</v>
@@ -9440,10 +9440,10 @@
         <v>164</v>
       </c>
       <c r="J147" s="2" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="K147" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L147" s="2" t="s">
         <v>288</v>
@@ -9481,13 +9481,13 @@
         <v>164</v>
       </c>
       <c r="J148" s="2" t="s">
+        <v>744</v>
+      </c>
+      <c r="K148" s="2" t="s">
         <v>745</v>
       </c>
-      <c r="K148" s="2" t="s">
-        <v>746</v>
-      </c>
       <c r="L148" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M148" s="24">
         <v>200</v>
@@ -9498,7 +9498,7 @@
     </row>
     <row r="149" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="4" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="B149" s="4">
         <v>1</v>
@@ -9513,13 +9513,13 @@
         <v>22</v>
       </c>
       <c r="F149" s="8" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="G149" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H149" s="4" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="J149" s="2"/>
       <c r="K149" s="2"/>
@@ -9529,7 +9529,7 @@
     </row>
     <row r="150" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="4" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="B150" s="4">
         <v>1</v>
@@ -9544,22 +9544,22 @@
         <v>22</v>
       </c>
       <c r="F150" s="8" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="G150" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H150" s="4" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="J150" s="2" t="s">
+        <v>912</v>
+      </c>
+      <c r="K150" s="2" t="s">
         <v>913</v>
       </c>
-      <c r="K150" s="2" t="s">
-        <v>914</v>
-      </c>
       <c r="L150" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M150" s="24">
         <v>200</v>
@@ -9594,10 +9594,10 @@
         <v>164</v>
       </c>
       <c r="J151" s="2" t="s">
+        <v>631</v>
+      </c>
+      <c r="K151" s="2" t="s">
         <v>632</v>
-      </c>
-      <c r="K151" s="2" t="s">
-        <v>633</v>
       </c>
       <c r="L151" s="2" t="s">
         <v>263</v>
@@ -9632,13 +9632,13 @@
         <v>125</v>
       </c>
       <c r="H152" s="4" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="J152" s="2" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="K152" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="L152" s="2" t="s">
         <v>274</v>
@@ -9676,10 +9676,10 @@
         <v>146</v>
       </c>
       <c r="J153" s="2" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="K153" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L153" s="2" t="s">
         <v>288</v>
@@ -9717,10 +9717,10 @@
         <v>175</v>
       </c>
       <c r="J154" s="2" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="K154" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L154" s="2" t="s">
         <v>288</v>
@@ -9734,7 +9734,7 @@
     </row>
     <row r="155" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="4" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="B155" s="4">
         <v>1</v>
@@ -9749,7 +9749,7 @@
         <v>8</v>
       </c>
       <c r="F155" s="4" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="G155" s="4" t="s">
         <v>125</v>
@@ -9758,10 +9758,10 @@
         <v>175</v>
       </c>
       <c r="J155" s="2" t="s">
+        <v>918</v>
+      </c>
+      <c r="K155" s="2" t="s">
         <v>919</v>
-      </c>
-      <c r="K155" s="2" t="s">
-        <v>920</v>
       </c>
       <c r="L155" s="2" t="s">
         <v>276</v>
@@ -9797,10 +9797,10 @@
         <v>175</v>
       </c>
       <c r="J156" s="2" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="K156" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="L156" s="2" t="s">
         <v>269</v>
@@ -9814,7 +9814,7 @@
     </row>
     <row r="157" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="4" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="B157" s="4">
         <v>1</v>
@@ -9829,7 +9829,7 @@
         <v>22</v>
       </c>
       <c r="F157" s="4" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="G157" s="4" t="s">
         <v>125</v>
@@ -9838,13 +9838,13 @@
         <v>178</v>
       </c>
       <c r="J157" s="2" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="K157" s="2" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="L157" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M157" s="24">
         <v>200</v>
@@ -9855,7 +9855,7 @@
     </row>
     <row r="158" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="4" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="B158" s="4">
         <v>1</v>
@@ -9870,7 +9870,7 @@
         <v>22</v>
       </c>
       <c r="F158" s="4" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="G158" s="4" t="s">
         <v>125</v>
@@ -9879,10 +9879,10 @@
         <v>178</v>
       </c>
       <c r="J158" s="2" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="K158" s="2" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="L158" s="2" t="s">
         <v>261</v>
@@ -9920,10 +9920,10 @@
         <v>178</v>
       </c>
       <c r="J159" s="2" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="K159" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L159" s="2" t="s">
         <v>288</v>
@@ -9959,10 +9959,10 @@
       </c>
       <c r="H160" s="4"/>
       <c r="J160" s="2" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="K160" s="2" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="L160" s="2" t="s">
         <v>277</v>
@@ -9998,16 +9998,16 @@
       </c>
       <c r="H161" s="4"/>
       <c r="J161" s="2" t="s">
+        <v>637</v>
+      </c>
+      <c r="K161" s="2" t="s">
         <v>638</v>
       </c>
-      <c r="K161" s="2" t="s">
-        <v>639</v>
-      </c>
       <c r="L161" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="M161" s="24" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="N161" s="2" t="s">
         <v>267</v>
@@ -10037,10 +10037,10 @@
       </c>
       <c r="H162" s="4"/>
       <c r="J162" s="2" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="K162" s="2" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="L162" s="2" t="s">
         <v>277</v>
@@ -10078,10 +10078,10 @@
         <v>154</v>
       </c>
       <c r="J163" s="2" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="K163" s="2" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="L163" s="2" t="s">
         <v>261</v>
@@ -10119,10 +10119,10 @@
         <v>132</v>
       </c>
       <c r="J164" s="2" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="K164" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="L164" s="2" t="s">
         <v>297</v>
@@ -10158,13 +10158,13 @@
       </c>
       <c r="H165" s="4"/>
       <c r="J165" s="2" t="s">
+        <v>642</v>
+      </c>
+      <c r="K165" s="2" t="s">
         <v>643</v>
       </c>
-      <c r="K165" s="2" t="s">
-        <v>644</v>
-      </c>
       <c r="L165" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M165" s="24">
         <v>200</v>
@@ -10197,10 +10197,10 @@
       </c>
       <c r="H166" s="4"/>
       <c r="J166" s="2" t="s">
+        <v>644</v>
+      </c>
+      <c r="K166" s="2" t="s">
         <v>645</v>
-      </c>
-      <c r="K166" s="2" t="s">
-        <v>646</v>
       </c>
       <c r="L166" s="2" t="s">
         <v>276</v>
@@ -10236,10 +10236,10 @@
         <v>195</v>
       </c>
       <c r="J167" s="2" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="K167" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L167" s="2" t="s">
         <v>288</v>
@@ -10253,7 +10253,7 @@
     </row>
     <row r="168" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="4" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="B168" s="4">
         <v>1</v>
@@ -10268,7 +10268,7 @@
         <v>19</v>
       </c>
       <c r="F168" s="4" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="G168" s="4" t="s">
         <v>125</v>
@@ -10277,10 +10277,10 @@
         <v>175</v>
       </c>
       <c r="J168" s="2" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="K168" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L168" s="2" t="s">
         <v>288</v>
@@ -10318,10 +10318,10 @@
         <v>198</v>
       </c>
       <c r="J169" s="2" t="s">
+        <v>647</v>
+      </c>
+      <c r="K169" s="2" t="s">
         <v>648</v>
-      </c>
-      <c r="K169" s="2" t="s">
-        <v>649</v>
       </c>
       <c r="L169" s="2" t="s">
         <v>264</v>
@@ -10356,13 +10356,13 @@
         <v>125</v>
       </c>
       <c r="H170" s="4" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J170" s="2" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="K170" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="L170" s="2" t="s">
         <v>297</v>
@@ -10376,7 +10376,7 @@
     </row>
     <row r="171" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="4" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B171" s="4">
         <v>1</v>
@@ -10391,7 +10391,7 @@
         <v>22</v>
       </c>
       <c r="F171" s="4" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="G171" s="4" t="s">
         <v>125</v>
@@ -10400,13 +10400,13 @@
         <v>178</v>
       </c>
       <c r="I171" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="J171" s="2" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="K171" s="2" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L171" s="2" t="s">
         <v>264</v>
@@ -10444,13 +10444,13 @@
         <v>178</v>
       </c>
       <c r="J172" s="2" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="K172" s="2" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="L172" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M172" s="24">
         <v>200</v>
@@ -10483,10 +10483,10 @@
       </c>
       <c r="H173" s="4"/>
       <c r="J173" s="2" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="K173" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L173" s="2" t="s">
         <v>288</v>
@@ -10524,10 +10524,10 @@
         <v>146</v>
       </c>
       <c r="J174" s="2" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="K174" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L174" s="2" t="s">
         <v>288</v>
@@ -10563,10 +10563,10 @@
       </c>
       <c r="H175" s="4"/>
       <c r="J175" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="K175" s="2" t="s">
         <v>654</v>
-      </c>
-      <c r="K175" s="2" t="s">
-        <v>655</v>
       </c>
       <c r="L175" s="2" t="s">
         <v>277</v>
@@ -10604,10 +10604,10 @@
         <v>175</v>
       </c>
       <c r="J176" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="K176" s="2" t="s">
         <v>656</v>
-      </c>
-      <c r="K176" s="2" t="s">
-        <v>657</v>
       </c>
       <c r="L176" s="2" t="s">
         <v>261</v>
@@ -10643,10 +10643,10 @@
       </c>
       <c r="H177" s="4"/>
       <c r="J177" s="2" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K177" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="L177" s="2" t="s">
         <v>261</v>
@@ -10682,10 +10682,10 @@
       </c>
       <c r="H178" s="4"/>
       <c r="J178" s="2" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="K178" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="L178" s="2" t="s">
         <v>297</v>
@@ -10723,10 +10723,10 @@
         <v>138</v>
       </c>
       <c r="J179" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="K179" s="2" t="s">
         <v>660</v>
-      </c>
-      <c r="K179" s="2" t="s">
-        <v>661</v>
       </c>
       <c r="L179" s="2" t="s">
         <v>288</v>
@@ -10762,13 +10762,13 @@
       </c>
       <c r="H180" s="4"/>
       <c r="J180" s="2" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="K180" s="2" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="L180" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M180" s="24">
         <v>200</v>
@@ -10801,16 +10801,16 @@
       </c>
       <c r="H181" s="4"/>
       <c r="J181" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="K181" s="2" t="s">
         <v>663</v>
       </c>
-      <c r="K181" s="2" t="s">
-        <v>664</v>
-      </c>
       <c r="L181" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="M181" s="24" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="N181" s="2" t="s">
         <v>267</v>
@@ -10842,10 +10842,10 @@
         <v>146</v>
       </c>
       <c r="J182" s="2" t="s">
+        <v>664</v>
+      </c>
+      <c r="K182" s="2" t="s">
         <v>665</v>
-      </c>
-      <c r="K182" s="2" t="s">
-        <v>666</v>
       </c>
       <c r="L182" s="2" t="s">
         <v>269</v>
@@ -10881,13 +10881,13 @@
       </c>
       <c r="H183" s="4"/>
       <c r="J183" s="2" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="K183" s="2" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="L183" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M183" s="24">
         <v>200</v>
@@ -10920,10 +10920,10 @@
       </c>
       <c r="H184" s="4"/>
       <c r="J184" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="K184" s="2" t="s">
         <v>668</v>
-      </c>
-      <c r="K184" s="2" t="s">
-        <v>669</v>
       </c>
       <c r="L184" s="2" t="s">
         <v>276</v>
@@ -10957,16 +10957,16 @@
       </c>
       <c r="H185" s="4"/>
       <c r="J185" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="K185" s="2" t="s">
         <v>670</v>
       </c>
-      <c r="K185" s="2" t="s">
-        <v>671</v>
-      </c>
       <c r="L185" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="M185" s="24" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="N185" s="2" t="s">
         <v>267</v>
@@ -10996,10 +10996,10 @@
       </c>
       <c r="H186" s="4"/>
       <c r="J186" s="2" t="s">
+        <v>671</v>
+      </c>
+      <c r="K186" s="2" t="s">
         <v>672</v>
-      </c>
-      <c r="K186" s="2" t="s">
-        <v>673</v>
       </c>
       <c r="L186" s="2" t="s">
         <v>269</v>
@@ -11035,10 +11035,10 @@
       </c>
       <c r="H187" s="4"/>
       <c r="J187" s="2" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="K187" s="2" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="L187" s="2" t="s">
         <v>269</v>
@@ -11076,13 +11076,13 @@
         <v>178</v>
       </c>
       <c r="J188" s="2" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="K188" s="2" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="L188" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M188" s="24">
         <v>200</v>
@@ -11115,10 +11115,10 @@
       </c>
       <c r="H189" s="4"/>
       <c r="J189" s="2" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="K189" s="2" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="L189" s="2" t="s">
         <v>269</v>
@@ -11156,10 +11156,10 @@
         <v>135</v>
       </c>
       <c r="J190" s="2" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="K190" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="L190" s="2" t="s">
         <v>261</v>
@@ -11195,10 +11195,10 @@
       </c>
       <c r="H191" s="4"/>
       <c r="J191" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="K191" s="2" t="s">
         <v>678</v>
-      </c>
-      <c r="K191" s="2" t="s">
-        <v>679</v>
       </c>
       <c r="L191" s="2" t="s">
         <v>297</v>
@@ -11212,7 +11212,7 @@
     </row>
     <row r="192" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="4" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B192" s="4">
         <v>1</v>
@@ -11227,16 +11227,16 @@
         <v>8</v>
       </c>
       <c r="F192" s="5" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="G192" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H192" s="4" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="J192" s="14" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="K192" s="14" t="s">
         <v>285</v>
@@ -11275,10 +11275,10 @@
       </c>
       <c r="H193" s="4"/>
       <c r="J193" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="K193" s="2" t="s">
         <v>680</v>
-      </c>
-      <c r="K193" s="2" t="s">
-        <v>681</v>
       </c>
       <c r="L193" s="2" t="s">
         <v>288</v>
@@ -11292,7 +11292,7 @@
     </row>
     <row r="194" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A194" s="4" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="B194" s="4">
         <v>1</v>
@@ -11307,7 +11307,7 @@
         <v>22</v>
       </c>
       <c r="F194" s="4" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="G194" s="4" t="s">
         <v>125</v>
@@ -11343,10 +11343,10 @@
       </c>
       <c r="H195" s="4"/>
       <c r="J195" s="2" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="K195" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="L195" s="2" t="s">
         <v>261</v>
@@ -11382,10 +11382,10 @@
       </c>
       <c r="H196" s="4"/>
       <c r="J196" s="2" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="K196" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="L196" s="2" t="s">
         <v>269</v>
@@ -11421,10 +11421,10 @@
       </c>
       <c r="H197" s="4"/>
       <c r="J197" s="2" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="K197" s="2" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="L197" s="2" t="s">
         <v>275</v>
@@ -11460,10 +11460,10 @@
       </c>
       <c r="H198" s="4"/>
       <c r="J198" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="K198" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L198" s="2" t="s">
         <v>288</v>
@@ -11499,10 +11499,10 @@
       </c>
       <c r="H199" s="4"/>
       <c r="J199" s="2" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="K199" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="L199" s="2" t="s">
         <v>260</v>
@@ -11538,10 +11538,10 @@
       </c>
       <c r="H200" s="4"/>
       <c r="J200" s="2" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="K200" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="L200" s="2" t="s">
         <v>269</v>
@@ -11577,13 +11577,13 @@
       </c>
       <c r="H201" s="4"/>
       <c r="J201" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="K201" s="2" t="s">
         <v>687</v>
       </c>
-      <c r="K201" s="2" t="s">
-        <v>688</v>
-      </c>
       <c r="L201" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M201" s="24">
         <v>200</v>
@@ -11616,10 +11616,10 @@
       </c>
       <c r="H202" s="4"/>
       <c r="J202" s="2" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="K202" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L202" s="2" t="s">
         <v>288</v>
@@ -11655,10 +11655,10 @@
       </c>
       <c r="H203" s="4"/>
       <c r="J203" s="2" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="K203" s="2" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="L203" s="2" t="s">
         <v>261</v>
@@ -11672,7 +11672,7 @@
     </row>
     <row r="204" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A204" s="4" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="B204" s="4">
         <v>1</v>
@@ -11687,14 +11687,14 @@
         <v>8</v>
       </c>
       <c r="F204" s="4" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="G204" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H204" s="4"/>
       <c r="J204" s="14" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="K204" s="14" t="s">
         <v>285</v>
@@ -11726,17 +11726,17 @@
         <v>8</v>
       </c>
       <c r="F205" s="4" t="s">
-        <v>440</v>
+        <v>945</v>
       </c>
       <c r="G205" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H205" s="4"/>
       <c r="J205" s="2" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="K205" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L205" s="2" t="s">
         <v>288</v>
@@ -11750,7 +11750,7 @@
     </row>
     <row r="206" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A206" s="4" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="B206" s="4">
         <v>1</v>
@@ -11765,19 +11765,19 @@
         <v>8</v>
       </c>
       <c r="F206" s="4" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="G206" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H206" s="4" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="J206" s="2" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="K206" s="2" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="L206" s="2" t="s">
         <v>275</v>
@@ -11791,7 +11791,7 @@
     </row>
     <row r="207" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A207" s="4" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="B207" s="4">
         <v>1</v>
@@ -11806,19 +11806,19 @@
         <v>8</v>
       </c>
       <c r="F207" s="4" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="G207" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H207" s="4" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="J207" s="2" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="K207" s="2" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="L207" s="2" t="s">
         <v>269</v>
@@ -11832,7 +11832,7 @@
     </row>
     <row r="208" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A208" s="4" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="B208" s="4">
         <v>1</v>
@@ -11847,19 +11847,19 @@
         <v>8</v>
       </c>
       <c r="F208" s="4" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="G208" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H208" s="4" t="s">
+        <v>875</v>
+      </c>
+      <c r="J208" s="2" t="s">
         <v>876</v>
       </c>
-      <c r="J208" s="2" t="s">
-        <v>877</v>
-      </c>
       <c r="K208" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L208" s="2" t="s">
         <v>288</v>
@@ -11873,7 +11873,7 @@
     </row>
     <row r="209" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A209" s="4" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B209" s="4">
         <v>1</v>
@@ -11888,16 +11888,16 @@
         <v>8</v>
       </c>
       <c r="F209" s="4" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="G209" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H209" s="4" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="J209" s="14" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="K209" s="14" t="s">
         <v>285</v>
@@ -11914,7 +11914,7 @@
     </row>
     <row r="210" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A210" s="4" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="B210" s="4">
         <v>1</v>
@@ -11929,19 +11929,19 @@
         <v>8</v>
       </c>
       <c r="F210" s="4" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G210" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H210" s="4" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="J210" s="2" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="K210" s="2" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="L210" s="2" t="s">
         <v>277</v>
@@ -11955,7 +11955,7 @@
     </row>
     <row r="211" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A211" s="4" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="B211" s="4">
         <v>1</v>
@@ -11970,25 +11970,25 @@
         <v>8</v>
       </c>
       <c r="F211" s="4" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="G211" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H211" s="4" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="I211" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="J211" s="2" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="K211" s="2" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="L211" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M211" s="24">
         <v>200</v>
@@ -12014,19 +12014,19 @@
         <v>8</v>
       </c>
       <c r="F212" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="G212" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H212" s="4" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="J212" s="2" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="K212" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="L212" s="2" t="s">
         <v>260</v>
@@ -12040,7 +12040,7 @@
     </row>
     <row r="213" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A213" s="4" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="B213" s="4">
         <v>1</v>
@@ -12055,13 +12055,13 @@
         <v>8</v>
       </c>
       <c r="F213" s="4" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="G213" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H213" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="214" spans="1:14" x14ac:dyDescent="0.25">
@@ -12081,17 +12081,17 @@
         <v>8</v>
       </c>
       <c r="F214" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="G214" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H214" s="4"/>
       <c r="J214" s="2" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="K214" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="L214" s="2" t="s">
         <v>261</v>
@@ -12120,23 +12120,23 @@
         <v>8</v>
       </c>
       <c r="F215" s="4" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="G215" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H215" s="4"/>
       <c r="J215" s="2" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="K215" s="2" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="L215" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="M215" s="24" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="N215" s="2" t="s">
         <v>267</v>
@@ -12159,17 +12159,17 @@
         <v>8</v>
       </c>
       <c r="F216" s="4" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="G216" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H216" s="4"/>
       <c r="J216" s="2" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="K216" s="2" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="L216" s="2" t="s">
         <v>276</v>
@@ -12196,17 +12196,17 @@
         <v>8</v>
       </c>
       <c r="F217" s="4" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="G217" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H217" s="4"/>
       <c r="J217" s="2" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="K217" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L217" s="2" t="s">
         <v>288</v>
@@ -12235,17 +12235,17 @@
         <v>8</v>
       </c>
       <c r="F218" s="4" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="G218" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H218" s="4"/>
       <c r="J218" s="2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="K218" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="L218" s="2" t="s">
         <v>269</v>
@@ -12274,17 +12274,17 @@
         <v>8</v>
       </c>
       <c r="F219" s="4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="G219" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H219" s="4"/>
       <c r="J219" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="K219" s="2" t="s">
         <v>697</v>
-      </c>
-      <c r="K219" s="2" t="s">
-        <v>698</v>
       </c>
       <c r="L219" s="2" t="s">
         <v>288</v>
@@ -12313,20 +12313,20 @@
         <v>19</v>
       </c>
       <c r="F220" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="G220" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H220" s="4"/>
       <c r="J220" s="2" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="K220" s="2" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="L220" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M220" s="24">
         <v>200</v>
@@ -12352,17 +12352,17 @@
         <v>19</v>
       </c>
       <c r="F221" s="4" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="G221" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H221" s="4"/>
       <c r="J221" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="K221" s="2" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="L221" s="2" t="s">
         <v>276</v>
@@ -12374,7 +12374,7 @@
     </row>
     <row r="222" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A222" s="4" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B222" s="4">
         <v>1</v>
@@ -12389,19 +12389,19 @@
         <v>8</v>
       </c>
       <c r="F222" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="G222" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H222" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="J222" s="2" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="K222" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L222" s="2" t="s">
         <v>288</v>
@@ -12430,19 +12430,19 @@
         <v>8</v>
       </c>
       <c r="F223" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="G223" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H223" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="J223" s="2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="K223" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="L223" s="2" t="s">
         <v>269</v>
@@ -12471,17 +12471,17 @@
         <v>19</v>
       </c>
       <c r="F224" s="4" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="G224" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H224" s="4"/>
       <c r="J224" s="2" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="K224" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="L224" s="2" t="s">
         <v>261</v>
@@ -12510,17 +12510,17 @@
         <v>8</v>
       </c>
       <c r="F225" s="4" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="G225" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H225" s="4"/>
       <c r="J225" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="K225" s="2" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="L225" s="2" t="s">
         <v>260</v>
@@ -12549,23 +12549,23 @@
         <v>8</v>
       </c>
       <c r="F226" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="G226" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H226" s="4"/>
       <c r="J226" s="2" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="K226" s="2" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="L226" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="M226" s="24" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="N226" s="2" t="s">
         <v>267</v>
@@ -12588,20 +12588,20 @@
         <v>19</v>
       </c>
       <c r="F227" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="G227" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H227" s="4"/>
       <c r="J227" s="2" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="K227" s="2" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="L227" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M227" s="24">
         <v>200</v>
@@ -12627,17 +12627,17 @@
         <v>19</v>
       </c>
       <c r="F228" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="G228" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H228" s="4"/>
       <c r="J228" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="K228" s="2" t="s">
         <v>668</v>
-      </c>
-      <c r="K228" s="2" t="s">
-        <v>669</v>
       </c>
       <c r="L228" s="2" t="s">
         <v>276</v>
@@ -12664,17 +12664,17 @@
         <v>8</v>
       </c>
       <c r="F229" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="G229" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H229" s="4"/>
       <c r="J229" s="2" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="K229" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L229" s="2" t="s">
         <v>288</v>
@@ -12703,7 +12703,7 @@
         <v>22</v>
       </c>
       <c r="F230" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="G230" s="4" t="s">
         <v>125</v>
@@ -12712,13 +12712,13 @@
         <v>178</v>
       </c>
       <c r="J230" s="2" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="K230" s="2" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="L230" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="M230" s="24">
         <v>200</v>
@@ -12744,7 +12744,7 @@
         <v>22</v>
       </c>
       <c r="F231" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="G231" s="4" t="s">
         <v>125</v>
@@ -12753,10 +12753,10 @@
         <v>178</v>
       </c>
       <c r="J231" s="2" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="K231" s="2" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="L231" s="2" t="s">
         <v>277</v>
@@ -12785,17 +12785,17 @@
         <v>22</v>
       </c>
       <c r="F232" s="4" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="G232" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H232" s="4"/>
       <c r="J232" s="2" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="K232" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L232" s="2" t="s">
         <v>288</v>
@@ -12824,20 +12824,20 @@
         <v>22</v>
       </c>
       <c r="F233" s="4" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="G233" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H233" s="4"/>
       <c r="I233" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="J233" s="2" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="K233" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="L233" s="2" t="s">
         <v>269</v>
@@ -12866,17 +12866,17 @@
         <v>22</v>
       </c>
       <c r="F234" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G234" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H234" s="4"/>
       <c r="J234" s="2" t="s">
+        <v>710</v>
+      </c>
+      <c r="K234" s="2" t="s">
         <v>711</v>
-      </c>
-      <c r="K234" s="2" t="s">
-        <v>712</v>
       </c>
       <c r="L234" s="2" t="s">
         <v>263</v>
@@ -12905,7 +12905,7 @@
         <v>8</v>
       </c>
       <c r="F235" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G235" s="4" t="s">
         <v>125</v>
@@ -12914,10 +12914,10 @@
         <v>175</v>
       </c>
       <c r="J235" s="2" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="K235" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L235" s="2" t="s">
         <v>288</v>
@@ -12946,7 +12946,7 @@
         <v>8</v>
       </c>
       <c r="F236" s="4" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="G236" s="4" t="s">
         <v>125</v>
@@ -12955,10 +12955,10 @@
         <v>175</v>
       </c>
       <c r="J236" s="2" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="K236" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L236" s="2" t="s">
         <v>288</v>
@@ -12987,23 +12987,23 @@
         <v>8</v>
       </c>
       <c r="F237" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="G237" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H237" s="4"/>
       <c r="J237" s="2" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="K237" s="2" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="L237" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="M237" s="24" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="N237" s="2" t="s">
         <v>267</v>
@@ -13026,17 +13026,17 @@
         <v>19</v>
       </c>
       <c r="F238" s="4" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="G238" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H238" s="4"/>
       <c r="J238" s="2" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="K238" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="L238" s="2" t="s">
         <v>261</v>
@@ -13065,19 +13065,19 @@
         <v>22</v>
       </c>
       <c r="F239" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="G239" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H239" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="J239" s="2" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="K239" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="L239" s="2" t="s">
         <v>297</v>
@@ -13106,19 +13106,19 @@
         <v>8</v>
       </c>
       <c r="F240" s="4" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="G240" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H240" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="J240" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="K240" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="L240" s="2" t="s">
         <v>261</v>
@@ -13147,19 +13147,19 @@
         <v>8</v>
       </c>
       <c r="F241" s="4" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="G241" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H241" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="J241" s="2" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="K241" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="L241" s="2" t="s">
         <v>261</v>
@@ -13188,19 +13188,19 @@
         <v>8</v>
       </c>
       <c r="F242" s="4" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="G242" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H242" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="J242" s="2" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="K242" s="2" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="L242" s="2" t="s">
         <v>277</v>
@@ -13229,19 +13229,19 @@
         <v>19</v>
       </c>
       <c r="F243" s="4" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="G243" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H243" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="J243" s="2" t="s">
+        <v>716</v>
+      </c>
+      <c r="K243" s="2" t="s">
         <v>717</v>
-      </c>
-      <c r="K243" s="2" t="s">
-        <v>718</v>
       </c>
       <c r="L243" s="2" t="s">
         <v>269</v>
@@ -13270,7 +13270,7 @@
         <v>8</v>
       </c>
       <c r="F244" s="4" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="G244" s="4" t="s">
         <v>125</v>
@@ -13279,10 +13279,10 @@
         <v>175</v>
       </c>
       <c r="J244" s="2" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="K244" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L244" s="2" t="s">
         <v>288</v>
@@ -13311,7 +13311,7 @@
         <v>8</v>
       </c>
       <c r="F245" s="4" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="G245" s="4" t="s">
         <v>125</v>
@@ -13320,10 +13320,10 @@
         <v>175</v>
       </c>
       <c r="J245" s="2" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="K245" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L245" s="2" t="s">
         <v>288</v>
@@ -13352,23 +13352,23 @@
         <v>22</v>
       </c>
       <c r="F246" s="4" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="G246" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H246" s="4"/>
       <c r="J246" s="2" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="K246" s="2" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="L246" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="M246" s="24" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="N246" s="2" t="s">
         <v>267</v>
@@ -13391,17 +13391,17 @@
         <v>22</v>
       </c>
       <c r="F247" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="G247" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H247" s="4"/>
       <c r="J247" s="2" t="s">
+        <v>721</v>
+      </c>
+      <c r="K247" s="2" t="s">
         <v>722</v>
-      </c>
-      <c r="K247" s="2" t="s">
-        <v>723</v>
       </c>
       <c r="L247" s="2" t="s">
         <v>297</v>
@@ -13415,7 +13415,7 @@
     </row>
     <row r="248" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A248" s="4" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="B248" s="4">
         <v>1</v>
@@ -13430,17 +13430,17 @@
         <v>22</v>
       </c>
       <c r="F248" s="4" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="G248" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H248" s="4"/>
       <c r="J248" s="2" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="K248" s="2" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="L248" s="2" t="s">
         <v>269</v>
@@ -13469,7 +13469,7 @@
         <v>8</v>
       </c>
       <c r="F249" s="4" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="G249" s="4" t="s">
         <v>125</v>
@@ -13478,10 +13478,10 @@
         <v>175</v>
       </c>
       <c r="J249" s="2" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="K249" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L249" s="2" t="s">
         <v>288</v>
@@ -13510,17 +13510,17 @@
         <v>8</v>
       </c>
       <c r="F250" s="4" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="G250" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H250" s="4"/>
       <c r="J250" s="2" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="K250" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="L250" s="2" t="s">
         <v>261</v>
@@ -13549,17 +13549,17 @@
         <v>22</v>
       </c>
       <c r="F251" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="G251" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H251" s="4"/>
       <c r="J251" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="K251" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="L251" s="2" t="s">
         <v>274</v>
@@ -13588,17 +13588,17 @@
         <v>19</v>
       </c>
       <c r="F252" s="4" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="G252" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H252" s="4"/>
       <c r="J252" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="K252" s="2" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="L252" s="2" t="s">
         <v>276</v>
@@ -13625,17 +13625,17 @@
         <v>8</v>
       </c>
       <c r="F253" s="4" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="G253" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H253" s="4"/>
       <c r="J253" s="2" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="K253" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="L253" s="2" t="s">
         <v>288</v>
@@ -13649,7 +13649,7 @@
     </row>
     <row r="254" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A254" s="26" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="B254" s="26">
         <v>1</v>
@@ -13664,14 +13664,14 @@
         <v>22</v>
       </c>
       <c r="F254" s="4" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="G254" s="26" t="s">
         <v>125</v>
       </c>
       <c r="H254" s="4"/>
       <c r="J254" s="14" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="K254" s="14" t="s">
         <v>285</v>
@@ -13853,6 +13853,7 @@
     <hyperlink ref="F209" r:id="rId74" xr:uid="{4ADCEE38-28CD-43D8-9123-B30FA02F7AB5}"/>
     <hyperlink ref="I94" r:id="rId75" xr:uid="{FE3AAB39-C871-4F64-AA22-E89C4CD15539}"/>
     <hyperlink ref="F89" r:id="rId76" xr:uid="{3D7B2B26-3280-40AF-A4C5-1389477FB9D2}"/>
+    <hyperlink ref="F205" r:id="rId77" xr:uid="{E1BA550E-4266-46F1-900F-62B4237C6D85}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>

</xml_diff>

<commit_message>
Incluye mejoras en Asaltos (panel overlay, carrusel y foco), vistas públicas, tablero, recursos xlsx y server.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/cartas.xlsx
+++ b/public/resources/cartas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9040C916-1E31-4BEC-9C81-2B24749B8741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18ED96AA-82C8-4370-8FD3-CE366C75A492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$N$265</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$N$272</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2426" uniqueCount="982">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2500" uniqueCount="1005">
   <si>
     <t>Nombre</t>
   </si>
@@ -2969,6 +2969,75 @@
   </si>
   <si>
     <t>Avalancha</t>
+  </si>
+  <si>
+    <t>Grim Knight</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/3tM4V9k/batman-who-laughs-the-grim-knight-textless-variant-cover-by-v0-rgxncsng34h21.webp</t>
+  </si>
+  <si>
+    <t>Multiverso oscuro</t>
+  </si>
+  <si>
+    <t>Pistolas duales</t>
+  </si>
+  <si>
+    <t>The Drowned</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/rR8N8Y8z/drowned.jpg</t>
+  </si>
+  <si>
+    <t>Lamentos ahogados</t>
+  </si>
+  <si>
+    <t>The Devastator</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/4Z0zW9RP/Batman-The-Devastator-Vol-1-1-Textless.webp</t>
+  </si>
+  <si>
+    <t>Devastación</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/1fYh5DHs/The-Murder-Machine.jpg</t>
+  </si>
+  <si>
+    <t>The Murder Machine</t>
+  </si>
+  <si>
+    <t>Ataque sorpresa</t>
+  </si>
+  <si>
+    <t>The Dawnbreaker</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/DfG6DH5R/Dawnbreaker.jpg</t>
+  </si>
+  <si>
+    <t>Escudo de luz</t>
+  </si>
+  <si>
+    <t>The Merciless</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/60txDWyh/Merciless.jpg</t>
+  </si>
+  <si>
+    <t>Sin piedad</t>
+  </si>
+  <si>
+    <t>The Red Death</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/qF1HGBz8/red-death-by-mariano1990-de2weby-fullview.jpg</t>
+  </si>
+  <si>
+    <t>Acechador veloz</t>
+  </si>
+  <si>
+    <t>Oscuridad caótica</t>
   </si>
 </sst>
 </file>
@@ -3549,7 +3618,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N266"/>
+  <dimension ref="A1:N273"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -11880,58 +11949,72 @@
     </row>
     <row r="206" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A206" s="4" t="s">
-        <v>913</v>
+        <v>1001</v>
       </c>
       <c r="B206" s="4">
         <v>1</v>
       </c>
       <c r="C206" s="4">
-        <v>2500</v>
+        <v>4000</v>
       </c>
       <c r="D206" s="4">
-        <v>1000</v>
+        <v>3000</v>
       </c>
       <c r="E206" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F206" s="4" t="s">
-        <v>914</v>
+        <v>1002</v>
       </c>
       <c r="G206" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H206" s="4"/>
-      <c r="J206" s="2"/>
-      <c r="K206" s="2"/>
-      <c r="L206" s="2"/>
-      <c r="M206" s="24"/>
-      <c r="N206" s="2"/>
+      <c r="H206" s="4" t="s">
+        <v>984</v>
+      </c>
+      <c r="J206" s="2" t="s">
+        <v>1003</v>
+      </c>
+      <c r="K206" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="L206" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="M206" s="24" t="s">
+        <v>270</v>
+      </c>
+      <c r="N206" s="2" t="s">
+        <v>268</v>
+      </c>
     </row>
     <row r="207" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A207" s="4" t="s">
-        <v>379</v>
+        <v>998</v>
       </c>
       <c r="B207" s="4">
         <v>1</v>
       </c>
       <c r="C207" s="4">
-        <v>5500</v>
+        <v>4500</v>
       </c>
       <c r="D207" s="4">
-        <v>3500</v>
+        <v>2500</v>
       </c>
       <c r="E207" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F207" s="4" t="s">
-        <v>431</v>
+        <v>999</v>
       </c>
       <c r="G207" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H207" s="4"/>
+      <c r="H207" s="4" t="s">
+        <v>984</v>
+      </c>
       <c r="J207" s="2" t="s">
-        <v>681</v>
+        <v>1000</v>
       </c>
       <c r="K207" s="2" t="s">
         <v>551</v>
@@ -11948,38 +12031,40 @@
     </row>
     <row r="208" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A208" s="4" t="s">
-        <v>380</v>
+        <v>995</v>
       </c>
       <c r="B208" s="4">
         <v>1</v>
       </c>
       <c r="C208" s="4">
-        <v>5500</v>
+        <v>4000</v>
       </c>
       <c r="D208" s="4">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="E208" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F208" s="4" t="s">
-        <v>432</v>
+        <v>996</v>
       </c>
       <c r="G208" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H208" s="4"/>
+      <c r="H208" s="4" t="s">
+        <v>984</v>
+      </c>
       <c r="J208" s="2" t="s">
-        <v>682</v>
+        <v>997</v>
       </c>
       <c r="K208" s="2" t="s">
-        <v>604</v>
+        <v>620</v>
       </c>
       <c r="L208" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="M208" s="24" t="s">
-        <v>270</v>
+        <v>264</v>
+      </c>
+      <c r="M208" s="24">
+        <v>1000</v>
       </c>
       <c r="N208" s="2" t="s">
         <v>268</v>
@@ -11987,7 +12072,7 @@
     </row>
     <row r="209" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A209" s="4" t="s">
-        <v>381</v>
+        <v>993</v>
       </c>
       <c r="B209" s="4">
         <v>1</v>
@@ -11996,62 +12081,64 @@
         <v>3500</v>
       </c>
       <c r="D209" s="4">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="E209" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F209" s="4" t="s">
-        <v>433</v>
+        <v>992</v>
       </c>
       <c r="G209" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H209" s="4"/>
+      <c r="H209" s="4" t="s">
+        <v>984</v>
+      </c>
       <c r="J209" s="2" t="s">
-        <v>629</v>
+        <v>994</v>
       </c>
       <c r="K209" s="2" t="s">
-        <v>547</v>
+        <v>668</v>
       </c>
       <c r="L209" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="M209" s="24">
-        <v>50</v>
-      </c>
+        <v>276</v>
+      </c>
+      <c r="M209" s="24"/>
       <c r="N209" s="2" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="210" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A210" s="4" t="s">
-        <v>382</v>
+        <v>989</v>
       </c>
       <c r="B210" s="4">
         <v>1</v>
       </c>
       <c r="C210" s="4">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="D210" s="4">
         <v>2000</v>
       </c>
       <c r="E210" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F210" s="4" t="s">
-        <v>434</v>
+        <v>990</v>
       </c>
       <c r="G210" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H210" s="4"/>
+      <c r="H210" s="4" t="s">
+        <v>984</v>
+      </c>
       <c r="J210" s="2" t="s">
-        <v>683</v>
+        <v>991</v>
       </c>
       <c r="K210" s="2" t="s">
-        <v>614</v>
+        <v>680</v>
       </c>
       <c r="L210" s="2" t="s">
         <v>288</v>
@@ -12065,29 +12152,31 @@
     </row>
     <row r="211" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A211" s="4" t="s">
-        <v>383</v>
+        <v>913</v>
       </c>
       <c r="B211" s="4">
         <v>1</v>
       </c>
       <c r="C211" s="4">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="D211" s="4">
         <v>1000</v>
       </c>
       <c r="E211" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F211" s="4" t="s">
-        <v>435</v>
+        <v>914</v>
       </c>
       <c r="G211" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H211" s="4"/>
+      <c r="H211" s="4" t="s">
+        <v>984</v>
+      </c>
       <c r="J211" s="2" t="s">
-        <v>684</v>
+        <v>1004</v>
       </c>
       <c r="K211" s="2" t="s">
         <v>612</v>
@@ -12104,77 +12193,81 @@
     </row>
     <row r="212" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A212" s="4" t="s">
-        <v>384</v>
+        <v>986</v>
       </c>
       <c r="B212" s="4">
         <v>1</v>
       </c>
       <c r="C212" s="4">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="D212" s="4">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="E212" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F212" s="4" t="s">
-        <v>436</v>
+        <v>987</v>
       </c>
       <c r="G212" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H212" s="4"/>
-      <c r="J212" s="2" t="s">
-        <v>685</v>
-      </c>
-      <c r="K212" s="2" t="s">
-        <v>604</v>
-      </c>
-      <c r="L212" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="M212" s="24" t="s">
-        <v>270</v>
-      </c>
-      <c r="N212" s="2" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="213" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H212" s="4" t="s">
+        <v>984</v>
+      </c>
+      <c r="J212" s="14" t="s">
+        <v>988</v>
+      </c>
+      <c r="K212" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="L212" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="M212" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="N212" s="14" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="213" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A213" s="4" t="s">
-        <v>385</v>
+        <v>982</v>
       </c>
       <c r="B213" s="4">
         <v>1</v>
       </c>
       <c r="C213" s="4">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="D213" s="4">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E213" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F213" s="4" t="s">
-        <v>437</v>
+        <v>983</v>
       </c>
       <c r="G213" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H213" s="4"/>
+      <c r="H213" s="4" t="s">
+        <v>984</v>
+      </c>
       <c r="J213" s="2" t="s">
-        <v>686</v>
+        <v>985</v>
       </c>
       <c r="K213" s="2" t="s">
-        <v>687</v>
+        <v>672</v>
       </c>
       <c r="L213" s="2" t="s">
-        <v>515</v>
-      </c>
-      <c r="M213" s="24">
-        <v>200</v>
+        <v>269</v>
+      </c>
+      <c r="M213" s="24" t="s">
+        <v>270</v>
       </c>
       <c r="N213" s="2" t="s">
         <v>268</v>
@@ -12182,85 +12275,89 @@
     </row>
     <row r="214" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A214" s="4" t="s">
-        <v>386</v>
+        <v>379</v>
       </c>
       <c r="B214" s="4">
         <v>1</v>
       </c>
       <c r="C214" s="4">
-        <v>5000</v>
+        <v>5500</v>
       </c>
       <c r="D214" s="4">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="E214" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F214" s="4" t="s">
-        <v>438</v>
+        <v>431</v>
       </c>
       <c r="G214" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H214" s="4"/>
+      <c r="H214" s="4" t="s">
+        <v>984</v>
+      </c>
       <c r="J214" s="2" t="s">
-        <v>688</v>
+        <v>681</v>
       </c>
       <c r="K214" s="2" t="s">
-        <v>614</v>
+        <v>551</v>
       </c>
       <c r="L214" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="M214" s="24" t="s">
-        <v>290</v>
+        <v>261</v>
+      </c>
+      <c r="M214" s="24">
+        <v>100</v>
       </c>
       <c r="N214" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="215" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A215" s="4" t="s">
-        <v>387</v>
+        <v>380</v>
       </c>
       <c r="B215" s="4">
         <v>1</v>
       </c>
       <c r="C215" s="4">
-        <v>4500</v>
+        <v>5500</v>
       </c>
       <c r="D215" s="4">
-        <v>2500</v>
+        <v>4000</v>
       </c>
       <c r="E215" s="4" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F215" s="4" t="s">
-        <v>439</v>
+        <v>432</v>
       </c>
       <c r="G215" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H215" s="4"/>
+      <c r="H215" s="4" t="s">
+        <v>984</v>
+      </c>
       <c r="J215" s="2" t="s">
-        <v>689</v>
+        <v>682</v>
       </c>
       <c r="K215" s="2" t="s">
-        <v>596</v>
+        <v>604</v>
       </c>
       <c r="L215" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="M215" s="24">
-        <v>100</v>
+        <v>269</v>
+      </c>
+      <c r="M215" s="24" t="s">
+        <v>270</v>
       </c>
       <c r="N215" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="216" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A216" s="4" t="s">
-        <v>795</v>
+        <v>381</v>
       </c>
       <c r="B216" s="4">
         <v>1</v>
@@ -12269,59 +12366,59 @@
         <v>3500</v>
       </c>
       <c r="D216" s="4">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E216" s="4" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F216" s="4" t="s">
-        <v>796</v>
+        <v>433</v>
       </c>
       <c r="G216" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H216" s="4"/>
-      <c r="J216" s="14" t="s">
-        <v>797</v>
-      </c>
-      <c r="K216" s="14" t="s">
-        <v>285</v>
-      </c>
-      <c r="L216" s="14" t="s">
-        <v>284</v>
-      </c>
-      <c r="M216" s="14" t="s">
-        <v>287</v>
-      </c>
-      <c r="N216" s="14" t="s">
+      <c r="J216" s="2" t="s">
+        <v>629</v>
+      </c>
+      <c r="K216" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="L216" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="M216" s="24">
+        <v>50</v>
+      </c>
+      <c r="N216" s="2" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="217" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A217" s="4" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="B217" s="4">
         <v>1</v>
       </c>
       <c r="C217" s="4">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="D217" s="4">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="E217" s="4" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F217" s="4" t="s">
-        <v>944</v>
+        <v>434</v>
       </c>
       <c r="G217" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H217" s="4"/>
       <c r="J217" s="2" t="s">
-        <v>690</v>
+        <v>683</v>
       </c>
       <c r="K217" s="2" t="s">
         <v>614</v>
@@ -12338,40 +12435,38 @@
     </row>
     <row r="218" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A218" s="4" t="s">
-        <v>876</v>
+        <v>383</v>
       </c>
       <c r="B218" s="4">
         <v>1</v>
       </c>
       <c r="C218" s="4">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="D218" s="4">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="E218" s="4" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F218" s="4" t="s">
-        <v>877</v>
+        <v>435</v>
       </c>
       <c r="G218" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H218" s="4" t="s">
-        <v>874</v>
-      </c>
+      <c r="H218" s="4"/>
       <c r="J218" s="2" t="s">
-        <v>878</v>
+        <v>684</v>
       </c>
       <c r="K218" s="2" t="s">
-        <v>547</v>
+        <v>612</v>
       </c>
       <c r="L218" s="2" t="s">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="M218" s="24">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="N218" s="2" t="s">
         <v>267</v>
@@ -12379,7 +12474,7 @@
     </row>
     <row r="219" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A219" s="4" t="s">
-        <v>861</v>
+        <v>384</v>
       </c>
       <c r="B219" s="4">
         <v>1</v>
@@ -12388,25 +12483,23 @@
         <v>4000</v>
       </c>
       <c r="D219" s="4">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="E219" s="4" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F219" s="4" t="s">
-        <v>862</v>
+        <v>436</v>
       </c>
       <c r="G219" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H219" s="4" t="s">
-        <v>874</v>
-      </c>
+      <c r="H219" s="4"/>
       <c r="J219" s="2" t="s">
-        <v>863</v>
+        <v>685</v>
       </c>
       <c r="K219" s="2" t="s">
-        <v>665</v>
+        <v>604</v>
       </c>
       <c r="L219" s="2" t="s">
         <v>269</v>
@@ -12420,7 +12513,7 @@
     </row>
     <row r="220" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A220" s="4" t="s">
-        <v>872</v>
+        <v>385</v>
       </c>
       <c r="B220" s="4">
         <v>1</v>
@@ -12432,28 +12525,26 @@
         <v>2000</v>
       </c>
       <c r="E220" s="4" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F220" s="4" t="s">
-        <v>873</v>
+        <v>437</v>
       </c>
       <c r="G220" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H220" s="4" t="s">
-        <v>874</v>
-      </c>
+      <c r="H220" s="4"/>
       <c r="J220" s="2" t="s">
-        <v>875</v>
+        <v>686</v>
       </c>
       <c r="K220" s="2" t="s">
-        <v>614</v>
+        <v>687</v>
       </c>
       <c r="L220" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="M220" s="24" t="s">
-        <v>290</v>
+        <v>515</v>
+      </c>
+      <c r="M220" s="24">
+        <v>200</v>
       </c>
       <c r="N220" s="2" t="s">
         <v>268</v>
@@ -12461,48 +12552,46 @@
     </row>
     <row r="221" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A221" s="4" t="s">
-        <v>855</v>
+        <v>386</v>
       </c>
       <c r="B221" s="4">
         <v>1</v>
       </c>
       <c r="C221" s="4">
-        <v>3500</v>
+        <v>5000</v>
       </c>
       <c r="D221" s="4">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="E221" s="4" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F221" s="4" t="s">
-        <v>856</v>
+        <v>438</v>
       </c>
       <c r="G221" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H221" s="4" t="s">
-        <v>874</v>
-      </c>
-      <c r="J221" s="14" t="s">
-        <v>858</v>
-      </c>
-      <c r="K221" s="14" t="s">
-        <v>285</v>
-      </c>
-      <c r="L221" s="14" t="s">
-        <v>284</v>
-      </c>
-      <c r="M221" s="14" t="s">
-        <v>287</v>
-      </c>
-      <c r="N221" s="14" t="s">
-        <v>267</v>
+      <c r="H221" s="4"/>
+      <c r="J221" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="K221" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="L221" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="M221" s="24" t="s">
+        <v>290</v>
+      </c>
+      <c r="N221" s="2" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="222" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A222" s="4" t="s">
-        <v>869</v>
+        <v>387</v>
       </c>
       <c r="B222" s="4">
         <v>1</v>
@@ -12511,39 +12600,37 @@
         <v>4500</v>
       </c>
       <c r="D222" s="4">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="E222" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F222" s="4" t="s">
-        <v>870</v>
+        <v>439</v>
       </c>
       <c r="G222" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H222" s="4" t="s">
-        <v>874</v>
-      </c>
+      <c r="H222" s="4"/>
       <c r="J222" s="2" t="s">
-        <v>871</v>
+        <v>689</v>
       </c>
       <c r="K222" s="2" t="s">
-        <v>654</v>
+        <v>596</v>
       </c>
       <c r="L222" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="M222" s="24" t="s">
-        <v>278</v>
+        <v>261</v>
+      </c>
+      <c r="M222" s="24">
+        <v>100</v>
       </c>
       <c r="N222" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="223" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A223" s="4" t="s">
-        <v>864</v>
+        <v>795</v>
       </c>
       <c r="B223" s="4">
         <v>1</v>
@@ -12558,109 +12645,117 @@
         <v>8</v>
       </c>
       <c r="F223" s="4" t="s">
-        <v>865</v>
+        <v>796</v>
       </c>
       <c r="G223" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H223" s="4" t="s">
-        <v>874</v>
-      </c>
-      <c r="I223" t="s">
-        <v>868</v>
-      </c>
-      <c r="J223" s="2" t="s">
-        <v>867</v>
-      </c>
-      <c r="K223" s="2" t="s">
-        <v>687</v>
-      </c>
-      <c r="L223" s="2" t="s">
-        <v>515</v>
-      </c>
-      <c r="M223" s="24">
-        <v>200</v>
-      </c>
-      <c r="N223" s="2" t="s">
-        <v>268</v>
+      <c r="H223" s="4"/>
+      <c r="J223" s="14" t="s">
+        <v>797</v>
+      </c>
+      <c r="K223" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="L223" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="M223" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="N223" s="14" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="224" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A224" s="4" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B224" s="4">
         <v>1</v>
       </c>
       <c r="C224" s="4">
-        <v>5000</v>
+        <v>4500</v>
       </c>
       <c r="D224" s="4">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="E224" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F224" s="4" t="s">
-        <v>440</v>
+        <v>944</v>
       </c>
       <c r="G224" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H224" s="4" t="s">
-        <v>874</v>
-      </c>
+      <c r="H224" s="4"/>
       <c r="J224" s="2" t="s">
-        <v>866</v>
+        <v>690</v>
       </c>
       <c r="K224" s="2" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="L224" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="M224" s="24">
-        <v>100</v>
+        <v>288</v>
+      </c>
+      <c r="M224" s="24" t="s">
+        <v>290</v>
       </c>
       <c r="N224" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="225" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A225" s="4" t="s">
-        <v>859</v>
+        <v>876</v>
       </c>
       <c r="B225" s="4">
         <v>1</v>
       </c>
       <c r="C225" s="4">
+        <v>4000</v>
+      </c>
+      <c r="D225" s="4">
         <v>3000</v>
-      </c>
-      <c r="D225" s="4">
-        <v>1000</v>
       </c>
       <c r="E225" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F225" s="4" t="s">
-        <v>860</v>
+        <v>877</v>
       </c>
       <c r="G225" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H225" s="4" t="s">
-        <v>453</v>
+        <v>874</v>
+      </c>
+      <c r="J225" s="2" t="s">
+        <v>878</v>
+      </c>
+      <c r="K225" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="L225" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="M225" s="24">
+        <v>50</v>
+      </c>
+      <c r="N225" s="2" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="226" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A226" s="4" t="s">
-        <v>390</v>
+        <v>861</v>
       </c>
       <c r="B226" s="4">
         <v>1</v>
       </c>
       <c r="C226" s="4">
-        <v>4500</v>
+        <v>4000</v>
       </c>
       <c r="D226" s="4">
         <v>2500</v>
@@ -12669,70 +12764,74 @@
         <v>8</v>
       </c>
       <c r="F226" s="4" t="s">
-        <v>441</v>
+        <v>862</v>
       </c>
       <c r="G226" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H226" s="4"/>
+      <c r="H226" s="4" t="s">
+        <v>874</v>
+      </c>
       <c r="J226" s="2" t="s">
-        <v>691</v>
+        <v>863</v>
       </c>
       <c r="K226" s="2" t="s">
-        <v>656</v>
+        <v>665</v>
       </c>
       <c r="L226" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="M226" s="24">
-        <v>100</v>
+        <v>269</v>
+      </c>
+      <c r="M226" s="24" t="s">
+        <v>270</v>
       </c>
       <c r="N226" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="227" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A227" s="4" t="s">
-        <v>391</v>
+        <v>872</v>
       </c>
       <c r="B227" s="4">
         <v>1</v>
       </c>
       <c r="C227" s="4">
-        <v>4500</v>
+        <v>4000</v>
       </c>
       <c r="D227" s="4">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="E227" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F227" s="4" t="s">
-        <v>442</v>
+        <v>873</v>
       </c>
       <c r="G227" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H227" s="4"/>
+      <c r="H227" s="4" t="s">
+        <v>874</v>
+      </c>
       <c r="J227" s="2" t="s">
-        <v>692</v>
+        <v>875</v>
       </c>
       <c r="K227" s="2" t="s">
-        <v>638</v>
+        <v>614</v>
       </c>
       <c r="L227" s="2" t="s">
-        <v>518</v>
+        <v>288</v>
       </c>
       <c r="M227" s="24" t="s">
-        <v>520</v>
+        <v>290</v>
       </c>
       <c r="N227" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="228" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A228" s="4" t="s">
-        <v>392</v>
+        <v>855</v>
       </c>
       <c r="B228" s="4">
         <v>1</v>
@@ -12747,60 +12846,66 @@
         <v>8</v>
       </c>
       <c r="F228" s="4" t="s">
-        <v>443</v>
+        <v>856</v>
       </c>
       <c r="G228" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H228" s="4"/>
-      <c r="J228" s="2" t="s">
-        <v>693</v>
-      </c>
-      <c r="K228" s="2" t="s">
-        <v>586</v>
-      </c>
-      <c r="L228" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="M228" s="24"/>
-      <c r="N228" s="2" t="s">
+      <c r="H228" s="4" t="s">
+        <v>874</v>
+      </c>
+      <c r="J228" s="14" t="s">
+        <v>858</v>
+      </c>
+      <c r="K228" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="L228" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="M228" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="N228" s="14" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="229" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A229" s="4" t="s">
-        <v>411</v>
+        <v>869</v>
       </c>
       <c r="B229" s="4">
         <v>1</v>
       </c>
       <c r="C229" s="4">
-        <v>5000</v>
+        <v>4500</v>
       </c>
       <c r="D229" s="4">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="E229" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F229" s="4" t="s">
-        <v>444</v>
+        <v>870</v>
       </c>
       <c r="G229" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H229" s="4"/>
+      <c r="H229" s="4" t="s">
+        <v>874</v>
+      </c>
       <c r="J229" s="2" t="s">
-        <v>694</v>
+        <v>871</v>
       </c>
       <c r="K229" s="2" t="s">
-        <v>614</v>
+        <v>654</v>
       </c>
       <c r="L229" s="2" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="M229" s="24" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
       <c r="N229" s="2" t="s">
         <v>268</v>
@@ -12808,38 +12913,43 @@
     </row>
     <row r="230" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A230" s="4" t="s">
-        <v>393</v>
+        <v>864</v>
       </c>
       <c r="B230" s="4">
         <v>1</v>
       </c>
       <c r="C230" s="4">
-        <v>4500</v>
+        <v>3500</v>
       </c>
       <c r="D230" s="4">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="E230" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F230" s="4" t="s">
-        <v>445</v>
+        <v>865</v>
       </c>
       <c r="G230" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H230" s="4"/>
+      <c r="H230" s="4" t="s">
+        <v>874</v>
+      </c>
+      <c r="I230" t="s">
+        <v>868</v>
+      </c>
       <c r="J230" s="2" t="s">
-        <v>695</v>
+        <v>867</v>
       </c>
       <c r="K230" s="2" t="s">
-        <v>604</v>
+        <v>687</v>
       </c>
       <c r="L230" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="M230" s="24" t="s">
-        <v>270</v>
+        <v>515</v>
+      </c>
+      <c r="M230" s="24">
+        <v>200</v>
       </c>
       <c r="N230" s="2" t="s">
         <v>268</v>
@@ -12847,343 +12957,328 @@
     </row>
     <row r="231" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A231" s="4" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="B231" s="4">
         <v>1</v>
       </c>
       <c r="C231" s="4">
-        <v>5500</v>
+        <v>5000</v>
       </c>
       <c r="D231" s="4">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="E231" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F231" s="4" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="G231" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H231" s="4"/>
+      <c r="H231" s="4" t="s">
+        <v>874</v>
+      </c>
       <c r="J231" s="2" t="s">
-        <v>696</v>
+        <v>866</v>
       </c>
       <c r="K231" s="2" t="s">
-        <v>697</v>
+        <v>612</v>
       </c>
       <c r="L231" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="M231" s="24" t="s">
-        <v>290</v>
+        <v>260</v>
+      </c>
+      <c r="M231" s="24">
+        <v>100</v>
       </c>
       <c r="N231" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="232" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A232" s="4" t="s">
-        <v>395</v>
+        <v>859</v>
       </c>
       <c r="B232" s="4">
         <v>1</v>
       </c>
       <c r="C232" s="4">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="D232" s="4">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="E232" s="4" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F232" s="4" t="s">
-        <v>448</v>
+        <v>860</v>
       </c>
       <c r="G232" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H232" s="4"/>
-      <c r="J232" s="2" t="s">
-        <v>698</v>
-      </c>
-      <c r="K232" s="2" t="s">
-        <v>643</v>
-      </c>
-      <c r="L232" s="2" t="s">
-        <v>515</v>
-      </c>
-      <c r="M232" s="24">
-        <v>200</v>
-      </c>
-      <c r="N232" s="2" t="s">
-        <v>268</v>
+      <c r="H232" s="4" t="s">
+        <v>453</v>
       </c>
     </row>
     <row r="233" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A233" s="4" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="B233" s="4">
         <v>1</v>
       </c>
       <c r="C233" s="4">
-        <v>3000</v>
+        <v>4500</v>
       </c>
       <c r="D233" s="4">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="E233" s="4" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F233" s="4" t="s">
-        <v>449</v>
+        <v>441</v>
       </c>
       <c r="G233" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H233" s="4"/>
       <c r="J233" s="2" t="s">
-        <v>699</v>
+        <v>691</v>
       </c>
       <c r="K233" s="2" t="s">
-        <v>645</v>
+        <v>656</v>
       </c>
       <c r="L233" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="M233" s="24"/>
+        <v>261</v>
+      </c>
+      <c r="M233" s="24">
+        <v>100</v>
+      </c>
       <c r="N233" s="2" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="234" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A234" s="4" t="s">
-        <v>451</v>
+        <v>391</v>
       </c>
       <c r="B234" s="4">
         <v>1</v>
       </c>
       <c r="C234" s="4">
-        <v>5000</v>
+        <v>4500</v>
       </c>
       <c r="D234" s="4">
-        <v>3500</v>
+        <v>2500</v>
       </c>
       <c r="E234" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F234" s="4" t="s">
-        <v>452</v>
+        <v>442</v>
       </c>
       <c r="G234" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H234" s="4" t="s">
-        <v>453</v>
-      </c>
+      <c r="H234" s="4"/>
       <c r="J234" s="2" t="s">
-        <v>548</v>
+        <v>692</v>
       </c>
       <c r="K234" s="2" t="s">
-        <v>614</v>
+        <v>638</v>
       </c>
       <c r="L234" s="2" t="s">
-        <v>288</v>
+        <v>518</v>
       </c>
       <c r="M234" s="24" t="s">
-        <v>290</v>
+        <v>520</v>
       </c>
       <c r="N234" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="235" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A235" s="4" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="B235" s="4">
         <v>1</v>
       </c>
       <c r="C235" s="4">
-        <v>5500</v>
+        <v>3500</v>
       </c>
       <c r="D235" s="4">
-        <v>3500</v>
+        <v>2500</v>
       </c>
       <c r="E235" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F235" s="4" t="s">
-        <v>450</v>
+        <v>443</v>
       </c>
       <c r="G235" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H235" s="4" t="s">
-        <v>453</v>
-      </c>
+      <c r="H235" s="4"/>
       <c r="J235" s="2" t="s">
-        <v>700</v>
+        <v>693</v>
       </c>
       <c r="K235" s="2" t="s">
-        <v>604</v>
+        <v>586</v>
       </c>
       <c r="L235" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="M235" s="24" t="s">
-        <v>270</v>
-      </c>
+        <v>276</v>
+      </c>
+      <c r="M235" s="24"/>
       <c r="N235" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="236" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A236" s="4" t="s">
-        <v>398</v>
+        <v>411</v>
       </c>
       <c r="B236" s="4">
         <v>1</v>
       </c>
       <c r="C236" s="4">
-        <v>3500</v>
+        <v>5000</v>
       </c>
       <c r="D236" s="4">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E236" s="4" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F236" s="4" t="s">
-        <v>454</v>
+        <v>444</v>
       </c>
       <c r="G236" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H236" s="4"/>
       <c r="J236" s="2" t="s">
-        <v>701</v>
+        <v>694</v>
       </c>
       <c r="K236" s="2" t="s">
-        <v>656</v>
+        <v>614</v>
       </c>
       <c r="L236" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="M236" s="24">
-        <v>100</v>
+        <v>288</v>
+      </c>
+      <c r="M236" s="24" t="s">
+        <v>290</v>
       </c>
       <c r="N236" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="237" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A237" s="4" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B237" s="4">
         <v>1</v>
       </c>
       <c r="C237" s="4">
-        <v>5500</v>
+        <v>4500</v>
       </c>
       <c r="D237" s="4">
-        <v>3500</v>
+        <v>2500</v>
       </c>
       <c r="E237" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F237" s="4" t="s">
-        <v>455</v>
+        <v>445</v>
       </c>
       <c r="G237" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H237" s="4"/>
       <c r="J237" s="2" t="s">
-        <v>702</v>
+        <v>695</v>
       </c>
       <c r="K237" s="2" t="s">
-        <v>575</v>
+        <v>604</v>
       </c>
       <c r="L237" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="M237" s="24">
-        <v>100</v>
+        <v>269</v>
+      </c>
+      <c r="M237" s="24" t="s">
+        <v>270</v>
       </c>
       <c r="N237" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="238" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A238" s="4" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="B238" s="4">
         <v>1</v>
       </c>
       <c r="C238" s="4">
-        <v>5000</v>
+        <v>5500</v>
       </c>
       <c r="D238" s="4">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="E238" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F238" s="4" t="s">
-        <v>456</v>
+        <v>446</v>
       </c>
       <c r="G238" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H238" s="4"/>
       <c r="J238" s="2" t="s">
-        <v>703</v>
+        <v>696</v>
       </c>
       <c r="K238" s="2" t="s">
-        <v>638</v>
+        <v>697</v>
       </c>
       <c r="L238" s="2" t="s">
-        <v>518</v>
+        <v>288</v>
       </c>
       <c r="M238" s="24" t="s">
-        <v>520</v>
+        <v>290</v>
       </c>
       <c r="N238" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="239" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A239" s="4" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
       <c r="B239" s="4">
         <v>1</v>
       </c>
       <c r="C239" s="4">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="D239" s="4">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="E239" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F239" s="4" t="s">
-        <v>457</v>
+        <v>448</v>
       </c>
       <c r="G239" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H239" s="4"/>
       <c r="J239" s="2" t="s">
-        <v>704</v>
+        <v>698</v>
       </c>
       <c r="K239" s="2" t="s">
         <v>643</v>
@@ -13200,7 +13295,7 @@
     </row>
     <row r="240" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A240" s="4" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
       <c r="B240" s="4">
         <v>1</v>
@@ -13215,17 +13310,17 @@
         <v>19</v>
       </c>
       <c r="F240" s="4" t="s">
-        <v>458</v>
+        <v>449</v>
       </c>
       <c r="G240" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H240" s="4"/>
       <c r="J240" s="2" t="s">
-        <v>667</v>
+        <v>699</v>
       </c>
       <c r="K240" s="2" t="s">
-        <v>668</v>
+        <v>645</v>
       </c>
       <c r="L240" s="2" t="s">
         <v>276</v>
@@ -13237,29 +13332,31 @@
     </row>
     <row r="241" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A241" s="4" t="s">
-        <v>403</v>
+        <v>451</v>
       </c>
       <c r="B241" s="4">
         <v>1</v>
       </c>
       <c r="C241" s="4">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="D241" s="4">
-        <v>1000</v>
+        <v>3500</v>
       </c>
       <c r="E241" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F241" s="4" t="s">
-        <v>459</v>
+        <v>452</v>
       </c>
       <c r="G241" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H241" s="4"/>
+      <c r="H241" s="4" t="s">
+        <v>453</v>
+      </c>
       <c r="J241" s="2" t="s">
-        <v>705</v>
+        <v>548</v>
       </c>
       <c r="K241" s="2" t="s">
         <v>614</v>
@@ -13276,201 +13373,196 @@
     </row>
     <row r="242" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A242" s="4" t="s">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="B242" s="4">
         <v>1</v>
       </c>
       <c r="C242" s="4">
-        <v>4000</v>
+        <v>5500</v>
       </c>
       <c r="D242" s="4">
-        <v>2000</v>
+        <v>3500</v>
       </c>
       <c r="E242" s="4" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F242" s="4" t="s">
-        <v>460</v>
+        <v>450</v>
       </c>
       <c r="G242" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H242" s="4" t="s">
-        <v>178</v>
+        <v>453</v>
       </c>
       <c r="J242" s="2" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="K242" s="2" t="s">
-        <v>643</v>
+        <v>604</v>
       </c>
       <c r="L242" s="2" t="s">
-        <v>515</v>
-      </c>
-      <c r="M242" s="24">
-        <v>200</v>
+        <v>269</v>
+      </c>
+      <c r="M242" s="24" t="s">
+        <v>270</v>
       </c>
       <c r="N242" s="2" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="243" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A243" s="4" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="B243" s="4">
         <v>1</v>
       </c>
       <c r="C243" s="4">
-        <v>4500</v>
+        <v>3500</v>
       </c>
       <c r="D243" s="4">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="E243" s="4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F243" s="4" t="s">
-        <v>461</v>
+        <v>454</v>
       </c>
       <c r="G243" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H243" s="4" t="s">
-        <v>178</v>
-      </c>
+      <c r="H243" s="4"/>
       <c r="J243" s="2" t="s">
-        <v>707</v>
+        <v>701</v>
       </c>
       <c r="K243" s="2" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="L243" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="M243" s="24" t="s">
-        <v>278</v>
+        <v>261</v>
+      </c>
+      <c r="M243" s="24">
+        <v>100</v>
       </c>
       <c r="N243" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="244" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A244" s="4" t="s">
-        <v>406</v>
+        <v>399</v>
       </c>
       <c r="B244" s="4">
         <v>1</v>
       </c>
       <c r="C244" s="4">
-        <v>4500</v>
+        <v>5500</v>
       </c>
       <c r="D244" s="4">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="E244" s="4" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F244" s="4" t="s">
-        <v>747</v>
+        <v>455</v>
       </c>
       <c r="G244" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H244" s="4"/>
       <c r="J244" s="2" t="s">
-        <v>708</v>
+        <v>702</v>
       </c>
       <c r="K244" s="2" t="s">
-        <v>614</v>
+        <v>575</v>
       </c>
       <c r="L244" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="M244" s="24" t="s">
-        <v>290</v>
+        <v>260</v>
+      </c>
+      <c r="M244" s="24">
+        <v>100</v>
       </c>
       <c r="N244" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="245" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A245" s="4" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="B245" s="4">
         <v>1</v>
       </c>
       <c r="C245" s="4">
-        <v>6000</v>
+        <v>5000</v>
       </c>
       <c r="D245" s="4">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="E245" s="4" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F245" s="4" t="s">
-        <v>899</v>
+        <v>456</v>
       </c>
       <c r="G245" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H245" s="4"/>
-      <c r="I245" t="s">
-        <v>900</v>
-      </c>
       <c r="J245" s="2" t="s">
-        <v>709</v>
+        <v>703</v>
       </c>
       <c r="K245" s="2" t="s">
-        <v>604</v>
+        <v>638</v>
       </c>
       <c r="L245" s="2" t="s">
-        <v>269</v>
+        <v>518</v>
       </c>
       <c r="M245" s="24" t="s">
-        <v>270</v>
+        <v>520</v>
       </c>
       <c r="N245" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="246" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A246" s="4" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="B246" s="4">
         <v>1</v>
       </c>
       <c r="C246" s="4">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="D246" s="4">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="E246" s="4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F246" s="4" t="s">
-        <v>462</v>
+        <v>457</v>
       </c>
       <c r="G246" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H246" s="4"/>
       <c r="J246" s="2" t="s">
-        <v>710</v>
+        <v>704</v>
       </c>
       <c r="K246" s="2" t="s">
-        <v>711</v>
+        <v>643</v>
       </c>
       <c r="L246" s="2" t="s">
-        <v>263</v>
+        <v>515</v>
       </c>
       <c r="M246" s="24">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="N246" s="2" t="s">
         <v>268</v>
@@ -13478,72 +13570,66 @@
     </row>
     <row r="247" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A247" s="4" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="B247" s="4">
         <v>1</v>
       </c>
       <c r="C247" s="4">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="D247" s="4">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="E247" s="4" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F247" s="4" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="G247" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H247" s="4" t="s">
-        <v>175</v>
-      </c>
+      <c r="H247" s="4"/>
       <c r="J247" s="2" t="s">
-        <v>634</v>
+        <v>667</v>
       </c>
       <c r="K247" s="2" t="s">
-        <v>614</v>
+        <v>668</v>
       </c>
       <c r="L247" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="M247" s="24" t="s">
-        <v>290</v>
-      </c>
+        <v>276</v>
+      </c>
+      <c r="M247" s="24"/>
       <c r="N247" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="248" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A248" s="4" t="s">
-        <v>410</v>
+        <v>403</v>
       </c>
       <c r="B248" s="4">
         <v>1</v>
       </c>
       <c r="C248" s="4">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="D248" s="4">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="E248" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F248" s="4" t="s">
-        <v>464</v>
+        <v>459</v>
       </c>
       <c r="G248" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H248" s="4" t="s">
-        <v>175</v>
-      </c>
+      <c r="H248" s="4"/>
       <c r="J248" s="2" t="s">
-        <v>712</v>
+        <v>705</v>
       </c>
       <c r="K248" s="2" t="s">
         <v>614</v>
@@ -13560,7 +13646,7 @@
     </row>
     <row r="249" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A249" s="4" t="s">
-        <v>181</v>
+        <v>404</v>
       </c>
       <c r="B249" s="4">
         <v>1</v>
@@ -13572,34 +13658,36 @@
         <v>2000</v>
       </c>
       <c r="E249" s="4" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F249" s="4" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="G249" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H249" s="4"/>
+      <c r="H249" s="4" t="s">
+        <v>178</v>
+      </c>
       <c r="J249" s="2" t="s">
-        <v>637</v>
+        <v>706</v>
       </c>
       <c r="K249" s="2" t="s">
-        <v>663</v>
+        <v>643</v>
       </c>
       <c r="L249" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="M249" s="24" t="s">
-        <v>520</v>
+        <v>515</v>
+      </c>
+      <c r="M249" s="24">
+        <v>200</v>
       </c>
       <c r="N249" s="2" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="250" spans="1:14" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="250" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A250" s="4" t="s">
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="B250" s="4">
         <v>1</v>
@@ -13611,34 +13699,36 @@
         <v>2500</v>
       </c>
       <c r="E250" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F250" s="4" t="s">
-        <v>746</v>
+        <v>461</v>
       </c>
       <c r="G250" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H250" s="4"/>
+      <c r="H250" s="4" t="s">
+        <v>178</v>
+      </c>
       <c r="J250" s="2" t="s">
-        <v>713</v>
+        <v>707</v>
       </c>
       <c r="K250" s="2" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="L250" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="M250" s="24">
-        <v>100</v>
+        <v>277</v>
+      </c>
+      <c r="M250" s="24" t="s">
+        <v>278</v>
       </c>
       <c r="N250" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="251" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A251" s="4" t="s">
-        <v>413</v>
+        <v>406</v>
       </c>
       <c r="B251" s="4">
         <v>1</v>
@@ -13653,148 +13743,145 @@
         <v>22</v>
       </c>
       <c r="F251" s="4" t="s">
-        <v>466</v>
+        <v>747</v>
       </c>
       <c r="G251" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H251" s="4" t="s">
-        <v>467</v>
-      </c>
+      <c r="H251" s="4"/>
       <c r="J251" s="2" t="s">
-        <v>714</v>
+        <v>708</v>
       </c>
       <c r="K251" s="2" t="s">
-        <v>566</v>
+        <v>614</v>
       </c>
       <c r="L251" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="M251" s="24">
-        <v>2</v>
+        <v>288</v>
+      </c>
+      <c r="M251" s="24" t="s">
+        <v>290</v>
       </c>
       <c r="N251" s="2" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="252" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A252" s="4" t="s">
-        <v>414</v>
+        <v>407</v>
       </c>
       <c r="B252" s="4">
         <v>1</v>
       </c>
       <c r="C252" s="4">
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="D252" s="4">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="E252" s="4" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F252" s="4" t="s">
-        <v>468</v>
+        <v>899</v>
       </c>
       <c r="G252" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H252" s="4" t="s">
-        <v>467</v>
+      <c r="H252" s="4"/>
+      <c r="I252" t="s">
+        <v>900</v>
       </c>
       <c r="J252" s="2" t="s">
-        <v>605</v>
+        <v>709</v>
       </c>
       <c r="K252" s="2" t="s">
-        <v>656</v>
+        <v>604</v>
       </c>
       <c r="L252" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="M252" s="24">
-        <v>100</v>
+        <v>269</v>
+      </c>
+      <c r="M252" s="24" t="s">
+        <v>270</v>
       </c>
       <c r="N252" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="253" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A253" s="4" t="s">
-        <v>415</v>
+        <v>408</v>
       </c>
       <c r="B253" s="4">
         <v>1</v>
       </c>
       <c r="C253" s="4">
-        <v>4500</v>
+        <v>5000</v>
       </c>
       <c r="D253" s="4">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="E253" s="4" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F253" s="4" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="G253" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H253" s="4" t="s">
-        <v>467</v>
-      </c>
+      <c r="H253" s="4"/>
       <c r="J253" s="2" t="s">
-        <v>552</v>
+        <v>710</v>
       </c>
       <c r="K253" s="2" t="s">
-        <v>656</v>
+        <v>711</v>
       </c>
       <c r="L253" s="2" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="M253" s="24">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="N253" s="2" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="254" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="254" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A254" s="4" t="s">
-        <v>416</v>
+        <v>409</v>
       </c>
       <c r="B254" s="4">
         <v>1</v>
       </c>
       <c r="C254" s="4">
-        <v>4500</v>
+        <v>5000</v>
       </c>
       <c r="D254" s="4">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="E254" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F254" s="4" t="s">
-        <v>470</v>
+        <v>463</v>
       </c>
       <c r="G254" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H254" s="4" t="s">
-        <v>467</v>
+        <v>175</v>
       </c>
       <c r="J254" s="2" t="s">
-        <v>715</v>
+        <v>634</v>
       </c>
       <c r="K254" s="2" t="s">
-        <v>654</v>
+        <v>614</v>
       </c>
       <c r="L254" s="2" t="s">
-        <v>277</v>
+        <v>288</v>
       </c>
       <c r="M254" s="24" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
       <c r="N254" s="2" t="s">
         <v>268</v>
@@ -13802,40 +13889,40 @@
     </row>
     <row r="255" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A255" s="4" t="s">
-        <v>417</v>
+        <v>410</v>
       </c>
       <c r="B255" s="4">
         <v>1</v>
       </c>
       <c r="C255" s="4">
-        <v>3500</v>
+        <v>5000</v>
       </c>
       <c r="D255" s="4">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="E255" s="4" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F255" s="4" t="s">
-        <v>471</v>
+        <v>464</v>
       </c>
       <c r="G255" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H255" s="4" t="s">
-        <v>467</v>
+        <v>175</v>
       </c>
       <c r="J255" s="2" t="s">
-        <v>716</v>
+        <v>712</v>
       </c>
       <c r="K255" s="2" t="s">
-        <v>717</v>
+        <v>614</v>
       </c>
       <c r="L255" s="2" t="s">
-        <v>269</v>
+        <v>288</v>
       </c>
       <c r="M255" s="24" t="s">
-        <v>270</v>
+        <v>290</v>
       </c>
       <c r="N255" s="2" t="s">
         <v>268</v>
@@ -13843,48 +13930,46 @@
     </row>
     <row r="256" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A256" s="4" t="s">
-        <v>418</v>
+        <v>181</v>
       </c>
       <c r="B256" s="4">
         <v>1</v>
       </c>
       <c r="C256" s="4">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="D256" s="4">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="E256" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F256" s="4" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="G256" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H256" s="4" t="s">
-        <v>175</v>
-      </c>
+      <c r="H256" s="4"/>
       <c r="J256" s="2" t="s">
-        <v>718</v>
+        <v>637</v>
       </c>
       <c r="K256" s="2" t="s">
-        <v>614</v>
+        <v>663</v>
       </c>
       <c r="L256" s="2" t="s">
-        <v>288</v>
+        <v>518</v>
       </c>
       <c r="M256" s="24" t="s">
-        <v>290</v>
+        <v>520</v>
       </c>
       <c r="N256" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="257" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A257" s="4" t="s">
-        <v>419</v>
+        <v>412</v>
       </c>
       <c r="B257" s="4">
         <v>1</v>
@@ -13893,78 +13978,78 @@
         <v>4500</v>
       </c>
       <c r="D257" s="4">
-        <v>3500</v>
+        <v>2500</v>
       </c>
       <c r="E257" s="4" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F257" s="4" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="G257" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H257" s="4" t="s">
-        <v>175</v>
-      </c>
+      <c r="H257" s="4"/>
       <c r="J257" s="2" t="s">
-        <v>719</v>
+        <v>713</v>
       </c>
       <c r="K257" s="2" t="s">
-        <v>614</v>
+        <v>656</v>
       </c>
       <c r="L257" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="M257" s="24" t="s">
-        <v>290</v>
+        <v>261</v>
+      </c>
+      <c r="M257" s="24">
+        <v>100</v>
       </c>
       <c r="N257" s="2" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="258" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="258" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A258" s="4" t="s">
-        <v>420</v>
+        <v>413</v>
       </c>
       <c r="B258" s="4">
         <v>1</v>
       </c>
       <c r="C258" s="4">
-        <v>4000</v>
+        <v>4500</v>
       </c>
       <c r="D258" s="4">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="E258" s="4" t="s">
         <v>22</v>
       </c>
       <c r="F258" s="4" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="G258" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H258" s="4"/>
+      <c r="H258" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J258" s="2" t="s">
-        <v>720</v>
+        <v>714</v>
       </c>
       <c r="K258" s="2" t="s">
-        <v>670</v>
+        <v>566</v>
       </c>
       <c r="L258" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="M258" s="24" t="s">
-        <v>520</v>
+        <v>297</v>
+      </c>
+      <c r="M258" s="24">
+        <v>2</v>
       </c>
       <c r="N258" s="2" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="259" spans="1:14" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="259" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A259" s="4" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
       <c r="B259" s="4">
         <v>1</v>
@@ -13973,109 +14058,113 @@
         <v>4000</v>
       </c>
       <c r="D259" s="4">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="E259" s="4" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F259" s="4" t="s">
-        <v>447</v>
+        <v>468</v>
       </c>
       <c r="G259" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H259" s="4"/>
+      <c r="H259" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J259" s="2" t="s">
-        <v>721</v>
+        <v>605</v>
       </c>
       <c r="K259" s="2" t="s">
-        <v>722</v>
+        <v>656</v>
       </c>
       <c r="L259" s="2" t="s">
-        <v>297</v>
+        <v>261</v>
       </c>
       <c r="M259" s="24">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="N259" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="260" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A260" s="4" t="s">
-        <v>919</v>
+        <v>415</v>
       </c>
       <c r="B260" s="4">
         <v>1</v>
       </c>
       <c r="C260" s="4">
-        <v>5000</v>
+        <v>4500</v>
       </c>
       <c r="D260" s="4">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="E260" s="4" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F260" s="4" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="G260" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H260" s="4"/>
+      <c r="H260" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J260" s="2" t="s">
-        <v>664</v>
+        <v>552</v>
       </c>
       <c r="K260" s="2" t="s">
-        <v>717</v>
+        <v>656</v>
       </c>
       <c r="L260" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="M260" s="24" t="s">
-        <v>270</v>
+        <v>261</v>
+      </c>
+      <c r="M260" s="24">
+        <v>100</v>
       </c>
       <c r="N260" s="2" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="261" spans="1:14" x14ac:dyDescent="0.25">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="261" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A261" s="4" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="B261" s="4">
         <v>1</v>
       </c>
       <c r="C261" s="4">
-        <v>5500</v>
+        <v>4500</v>
       </c>
       <c r="D261" s="4">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="E261" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F261" s="4" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="G261" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H261" s="4" t="s">
-        <v>175</v>
+        <v>467</v>
       </c>
       <c r="J261" s="2" t="s">
-        <v>723</v>
+        <v>715</v>
       </c>
       <c r="K261" s="2" t="s">
-        <v>614</v>
+        <v>654</v>
       </c>
       <c r="L261" s="2" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="M261" s="24" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
       <c r="N261" s="2" t="s">
         <v>268</v>
@@ -14083,77 +14172,81 @@
     </row>
     <row r="262" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A262" s="4" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
       <c r="B262" s="4">
         <v>1</v>
       </c>
       <c r="C262" s="4">
-        <v>4500</v>
+        <v>3500</v>
       </c>
       <c r="D262" s="4">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="E262" s="4" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F262" s="4" t="s">
-        <v>476</v>
+        <v>471</v>
       </c>
       <c r="G262" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H262" s="4"/>
+      <c r="H262" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J262" s="2" t="s">
-        <v>691</v>
+        <v>716</v>
       </c>
       <c r="K262" s="2" t="s">
-        <v>656</v>
+        <v>717</v>
       </c>
       <c r="L262" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="M262" s="24">
-        <v>100</v>
+        <v>269</v>
+      </c>
+      <c r="M262" s="24" t="s">
+        <v>270</v>
       </c>
       <c r="N262" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="263" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A263" s="4" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
       <c r="B263" s="4">
         <v>1</v>
       </c>
       <c r="C263" s="4">
-        <v>4500</v>
+        <v>5000</v>
       </c>
       <c r="D263" s="4">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="E263" s="4" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F263" s="4" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="G263" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H263" s="4"/>
+      <c r="H263" s="4" t="s">
+        <v>175</v>
+      </c>
       <c r="J263" s="2" t="s">
-        <v>724</v>
+        <v>718</v>
       </c>
       <c r="K263" s="2" t="s">
-        <v>561</v>
+        <v>614</v>
       </c>
       <c r="L263" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="M263" s="24">
-        <v>750</v>
+        <v>288</v>
+      </c>
+      <c r="M263" s="24" t="s">
+        <v>290</v>
       </c>
       <c r="N263" s="2" t="s">
         <v>268</v>
@@ -14161,7 +14254,7 @@
     </row>
     <row r="264" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A264" s="4" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
       <c r="B264" s="4">
         <v>1</v>
@@ -14170,113 +14263,390 @@
         <v>4500</v>
       </c>
       <c r="D264" s="4">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="E264" s="4" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F264" s="4" t="s">
-        <v>478</v>
+        <v>742</v>
       </c>
       <c r="G264" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H264" s="4"/>
+      <c r="H264" s="4" t="s">
+        <v>175</v>
+      </c>
       <c r="J264" s="2" t="s">
-        <v>725</v>
+        <v>719</v>
       </c>
       <c r="K264" s="2" t="s">
-        <v>645</v>
+        <v>614</v>
       </c>
       <c r="L264" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="M264" s="24"/>
+        <v>288</v>
+      </c>
+      <c r="M264" s="24" t="s">
+        <v>290</v>
+      </c>
       <c r="N264" s="2" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="265" spans="1:14" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="265" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A265" s="4" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
       <c r="B265" s="4">
         <v>1</v>
       </c>
       <c r="C265" s="4">
-        <v>4500</v>
+        <v>4000</v>
       </c>
       <c r="D265" s="4">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="E265" s="4" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F265" s="4" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
       <c r="G265" s="4" t="s">
         <v>125</v>
       </c>
       <c r="H265" s="4"/>
       <c r="J265" s="2" t="s">
+        <v>720</v>
+      </c>
+      <c r="K265" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="L265" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="M265" s="24" t="s">
+        <v>520</v>
+      </c>
+      <c r="N265" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="266" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A266" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="B266" s="4">
+        <v>1</v>
+      </c>
+      <c r="C266" s="4">
+        <v>4000</v>
+      </c>
+      <c r="D266" s="4">
+        <v>2500</v>
+      </c>
+      <c r="E266" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F266" s="4" t="s">
+        <v>447</v>
+      </c>
+      <c r="G266" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="H266" s="4"/>
+      <c r="J266" s="2" t="s">
+        <v>721</v>
+      </c>
+      <c r="K266" s="2" t="s">
+        <v>722</v>
+      </c>
+      <c r="L266" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="M266" s="24">
+        <v>2</v>
+      </c>
+      <c r="N266" s="2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="267" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A267" s="4" t="s">
+        <v>919</v>
+      </c>
+      <c r="B267" s="4">
+        <v>1</v>
+      </c>
+      <c r="C267" s="4">
+        <v>5000</v>
+      </c>
+      <c r="D267" s="4">
+        <v>3000</v>
+      </c>
+      <c r="E267" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F267" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="G267" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="H267" s="4"/>
+      <c r="J267" s="2" t="s">
+        <v>664</v>
+      </c>
+      <c r="K267" s="2" t="s">
+        <v>717</v>
+      </c>
+      <c r="L267" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="M267" s="24" t="s">
+        <v>270</v>
+      </c>
+      <c r="N267" s="2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="268" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A268" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="B268" s="4">
+        <v>1</v>
+      </c>
+      <c r="C268" s="4">
+        <v>5500</v>
+      </c>
+      <c r="D268" s="4">
+        <v>4000</v>
+      </c>
+      <c r="E268" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F268" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="G268" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="H268" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J268" s="2" t="s">
+        <v>723</v>
+      </c>
+      <c r="K268" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="L268" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="M268" s="24" t="s">
+        <v>290</v>
+      </c>
+      <c r="N268" s="2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="269" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A269" s="4" t="s">
+        <v>423</v>
+      </c>
+      <c r="B269" s="4">
+        <v>1</v>
+      </c>
+      <c r="C269" s="4">
+        <v>4500</v>
+      </c>
+      <c r="D269" s="4">
+        <v>2500</v>
+      </c>
+      <c r="E269" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F269" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="G269" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="H269" s="4"/>
+      <c r="J269" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="K269" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="L269" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="M269" s="24">
+        <v>100</v>
+      </c>
+      <c r="N269" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="270" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A270" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="B270" s="4">
+        <v>1</v>
+      </c>
+      <c r="C270" s="4">
+        <v>4500</v>
+      </c>
+      <c r="D270" s="4">
+        <v>2500</v>
+      </c>
+      <c r="E270" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F270" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="G270" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="H270" s="4"/>
+      <c r="J270" s="2" t="s">
+        <v>724</v>
+      </c>
+      <c r="K270" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="L270" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="M270" s="24">
+        <v>750</v>
+      </c>
+      <c r="N270" s="2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="271" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A271" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="B271" s="4">
+        <v>1</v>
+      </c>
+      <c r="C271" s="4">
+        <v>4500</v>
+      </c>
+      <c r="D271" s="4">
+        <v>2500</v>
+      </c>
+      <c r="E271" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F271" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="G271" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="H271" s="4"/>
+      <c r="J271" s="2" t="s">
+        <v>725</v>
+      </c>
+      <c r="K271" s="2" t="s">
+        <v>645</v>
+      </c>
+      <c r="L271" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="M271" s="24"/>
+      <c r="N271" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="272" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A272" s="4" t="s">
+        <v>426</v>
+      </c>
+      <c r="B272" s="4">
+        <v>1</v>
+      </c>
+      <c r="C272" s="4">
+        <v>4500</v>
+      </c>
+      <c r="D272" s="4">
+        <v>3000</v>
+      </c>
+      <c r="E272" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F272" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="G272" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="H272" s="4"/>
+      <c r="J272" s="2" t="s">
         <v>726</v>
       </c>
-      <c r="K265" s="2" t="s">
+      <c r="K272" s="2" t="s">
         <v>614</v>
       </c>
-      <c r="L265" s="2" t="s">
+      <c r="L272" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="M265" s="24" t="s">
+      <c r="M272" s="24" t="s">
         <v>290</v>
       </c>
-      <c r="N265" s="2" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="266" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A266" s="26" t="s">
+      <c r="N272" s="2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="273" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A273" s="26" t="s">
         <v>761</v>
       </c>
-      <c r="B266" s="26">
-        <v>1</v>
-      </c>
-      <c r="C266" s="26">
+      <c r="B273" s="26">
+        <v>1</v>
+      </c>
+      <c r="C273" s="26">
         <v>5000</v>
       </c>
-      <c r="D266" s="26">
+      <c r="D273" s="26">
         <v>3000</v>
       </c>
-      <c r="E266" s="26" t="s">
+      <c r="E273" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="F266" s="4" t="s">
+      <c r="F273" s="4" t="s">
         <v>762</v>
       </c>
-      <c r="G266" s="26" t="s">
+      <c r="G273" s="26" t="s">
         <v>125</v>
       </c>
-      <c r="H266" s="4"/>
-      <c r="J266" s="14" t="s">
+      <c r="H273" s="4"/>
+      <c r="J273" s="14" t="s">
         <v>763</v>
       </c>
-      <c r="K266" s="14" t="s">
+      <c r="K273" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="L266" s="14" t="s">
+      <c r="L273" s="14" t="s">
         <v>284</v>
       </c>
-      <c r="M266" s="14" t="s">
+      <c r="M273" s="14" t="s">
         <v>287</v>
       </c>
-      <c r="N266" s="14" t="s">
+      <c r="N273" s="14" t="s">
         <v>267</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N265" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="C205:C265">
+  <autoFilter ref="A1:N272" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="C205:C272">
     <cfRule type="colorScale" priority="89">
       <colorScale>
         <cfvo type="min"/>
@@ -14288,7 +14658,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C266:C1048576 C2:C204">
+  <conditionalFormatting sqref="C273:C1048576 C2:C204">
     <cfRule type="colorScale" priority="55">
       <colorScale>
         <cfvo type="min"/>
@@ -14300,7 +14670,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D205:D265">
+  <conditionalFormatting sqref="D205:D272">
     <cfRule type="colorScale" priority="91">
       <colorScale>
         <cfvo type="min"/>
@@ -14312,7 +14682,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D266:D1048576 D2:D204">
+  <conditionalFormatting sqref="D273:D1048576 D2:D204">
     <cfRule type="colorScale" priority="56">
       <colorScale>
         <cfvo type="min"/>
@@ -14324,7 +14694,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:N224">
+  <conditionalFormatting sqref="J2:N231">
     <cfRule type="expression" dxfId="11" priority="7">
       <formula>OR($L2="debuff",$L2="bonus_debuff",$L2="revive")</formula>
     </cfRule>
@@ -14344,24 +14714,24 @@
       <formula>OR($L2="extra_attack",$L2="aoe")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J226:N266">
+  <conditionalFormatting sqref="J233:N273">
     <cfRule type="expression" dxfId="5" priority="37">
-      <formula>OR($L226="debuff",$L226="bonus_debuff",$L226="revive")</formula>
+      <formula>OR($L233="debuff",$L233="bonus_debuff",$L233="revive")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="4" priority="38">
-      <formula>OR($L226="buff",$L226="bonus_buff")</formula>
+      <formula>OR($L233="buff",$L233="bonus_buff")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="3" priority="39">
-      <formula>OR($L226="dot",$L226="stun")</formula>
+      <formula>OR($L233="dot",$L233="stun")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="40">
-      <formula>OR($L226="tank",$L226="shield")</formula>
+      <formula>OR($L233="tank",$L233="shield")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="41">
-      <formula>OR($L226="heal",$L226="heal_all",$L226="life_steal")</formula>
+      <formula>OR($L233="heal",$L233="heal_all",$L233="life_steal")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="0" priority="42">
-      <formula>OR($L226="extra_attack",$L226="aoe")</formula>
+      <formula>OR($L233="extra_attack",$L233="aoe")</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -14424,24 +14794,24 @@
     <hyperlink ref="F20" r:id="rId57" xr:uid="{BABB0F5C-56BD-4A07-93B3-021E469232CD}"/>
     <hyperlink ref="F32" r:id="rId58" xr:uid="{61098037-76F4-4673-81EC-2C0BEA11F28D}"/>
     <hyperlink ref="F205" r:id="rId59" xr:uid="{CDB9697E-B5DD-4B05-A87F-9948E71EB15D}"/>
-    <hyperlink ref="F207" r:id="rId60" xr:uid="{1C16544A-4F4A-4C08-89CC-4F37E0986D91}"/>
-    <hyperlink ref="F208" r:id="rId61" xr:uid="{06E0FEDA-F7DA-458D-8F09-76B80DE09AB2}"/>
-    <hyperlink ref="F209" r:id="rId62" xr:uid="{08075219-10D9-404E-8E18-C232DE173646}"/>
-    <hyperlink ref="F212" r:id="rId63" xr:uid="{8346A542-3C7A-4501-8018-E883F1C014BD}"/>
-    <hyperlink ref="F213" r:id="rId64" xr:uid="{086976A0-E476-44F3-A1A7-A52FDD5C6A16}"/>
-    <hyperlink ref="F214" r:id="rId65" xr:uid="{7779F7F1-7C83-4CBB-AB2B-7D87ED427D90}"/>
-    <hyperlink ref="F244" r:id="rId66" xr:uid="{0E7F5509-4BC7-4B9D-A1EB-D898649A078B}"/>
-    <hyperlink ref="F246" r:id="rId67" xr:uid="{44F6718A-2854-42BF-B97F-E837DDE75498}"/>
-    <hyperlink ref="F265" r:id="rId68" xr:uid="{3BC7514F-0333-437E-B491-EC00925189BB}"/>
-    <hyperlink ref="F257" r:id="rId69" xr:uid="{13B89169-25A4-4FB6-A6AE-2EF0BD97D55D}"/>
-    <hyperlink ref="F250" r:id="rId70" xr:uid="{84363341-8DC7-4D5A-A434-7D3C17151FB3}"/>
+    <hyperlink ref="F214" r:id="rId60" xr:uid="{1C16544A-4F4A-4C08-89CC-4F37E0986D91}"/>
+    <hyperlink ref="F215" r:id="rId61" xr:uid="{06E0FEDA-F7DA-458D-8F09-76B80DE09AB2}"/>
+    <hyperlink ref="F216" r:id="rId62" xr:uid="{08075219-10D9-404E-8E18-C232DE173646}"/>
+    <hyperlink ref="F219" r:id="rId63" xr:uid="{8346A542-3C7A-4501-8018-E883F1C014BD}"/>
+    <hyperlink ref="F220" r:id="rId64" xr:uid="{086976A0-E476-44F3-A1A7-A52FDD5C6A16}"/>
+    <hyperlink ref="F221" r:id="rId65" xr:uid="{7779F7F1-7C83-4CBB-AB2B-7D87ED427D90}"/>
+    <hyperlink ref="F251" r:id="rId66" xr:uid="{0E7F5509-4BC7-4B9D-A1EB-D898649A078B}"/>
+    <hyperlink ref="F253" r:id="rId67" xr:uid="{44F6718A-2854-42BF-B97F-E837DDE75498}"/>
+    <hyperlink ref="F272" r:id="rId68" xr:uid="{3BC7514F-0333-437E-B491-EC00925189BB}"/>
+    <hyperlink ref="F264" r:id="rId69" xr:uid="{13B89169-25A4-4FB6-A6AE-2EF0BD97D55D}"/>
+    <hyperlink ref="F257" r:id="rId70" xr:uid="{84363341-8DC7-4D5A-A434-7D3C17151FB3}"/>
     <hyperlink ref="F124" r:id="rId71" xr:uid="{163A63BB-52A6-4D6C-B00A-1A7F1F28061D}"/>
     <hyperlink ref="F15" r:id="rId72" xr:uid="{C439613B-BEC0-48C5-814E-36E868E99B31}"/>
     <hyperlink ref="F98" r:id="rId73" xr:uid="{7E273EDB-40F6-4371-AC08-0F1FA586E40C}"/>
-    <hyperlink ref="F221" r:id="rId74" xr:uid="{4ADCEE38-28CD-43D8-9123-B30FA02F7AB5}"/>
+    <hyperlink ref="F228" r:id="rId74" xr:uid="{4ADCEE38-28CD-43D8-9123-B30FA02F7AB5}"/>
     <hyperlink ref="I99" r:id="rId75" xr:uid="{FE3AAB39-C871-4F64-AA22-E89C4CD15539}"/>
     <hyperlink ref="F94" r:id="rId76" xr:uid="{3D7B2B26-3280-40AF-A4C5-1389477FB9D2}"/>
-    <hyperlink ref="F217" r:id="rId77" xr:uid="{E1BA550E-4266-46F1-900F-62B4237C6D85}"/>
+    <hyperlink ref="F224" r:id="rId77" xr:uid="{E1BA550E-4266-46F1-900F-62B4237C6D85}"/>
     <hyperlink ref="F126" r:id="rId78" xr:uid="{F3D65CAC-0B07-443F-8FF4-96BA556BCF65}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Cambios cartas blue beetle
</commit_message>
<xml_diff>
--- a/public/resources/cartas.xlsx
+++ b/public/resources/cartas.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N346"/>
+  <dimension ref="A1:N348"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1457,7 +1457,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Blue Beetle</v>
+        <v>Blue Beetle III</v>
       </c>
       <c r="B25">
         <v>1</v>
@@ -1481,7 +1481,7 @@
         <v>Teen Titans</v>
       </c>
       <c r="I25" t="str">
-        <v/>
+        <v>https://i.ibb.co/Y7g24sDp/heroes-who-are-inside-a-robotic-suit-v0-3yxhxf07yl2g1.jpg</v>
       </c>
       <c r="J25" t="str">
         <v>Armadura escarabajo</v>
@@ -15623,9 +15623,97 @@
         <v>usar</v>
       </c>
     </row>
+    <row r="347">
+      <c r="A347" t="str">
+        <v>Nueva_carta_jv1ij</v>
+      </c>
+      <c r="B347">
+        <v>1</v>
+      </c>
+      <c r="C347">
+        <v>0</v>
+      </c>
+      <c r="D347">
+        <v>0</v>
+      </c>
+      <c r="E347" t="str">
+        <v/>
+      </c>
+      <c r="F347" t="str">
+        <v/>
+      </c>
+      <c r="G347" t="str">
+        <v/>
+      </c>
+      <c r="H347" t="str">
+        <v/>
+      </c>
+      <c r="I347" t="str">
+        <v/>
+      </c>
+      <c r="J347" t="str">
+        <v/>
+      </c>
+      <c r="K347" t="str">
+        <v/>
+      </c>
+      <c r="L347" t="str">
+        <v/>
+      </c>
+      <c r="M347" t="str">
+        <v/>
+      </c>
+      <c r="N347" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="str">
+        <v>Blue Beetle II</v>
+      </c>
+      <c r="B348">
+        <v>1</v>
+      </c>
+      <c r="C348">
+        <v>0</v>
+      </c>
+      <c r="D348">
+        <v>0</v>
+      </c>
+      <c r="E348" t="str">
+        <v>Tecnología</v>
+      </c>
+      <c r="F348" t="str">
+        <v>https://i.ibb.co/PswgLfNB/Blue-Bettle.jpg</v>
+      </c>
+      <c r="G348" t="str">
+        <v>H</v>
+      </c>
+      <c r="H348" t="str">
+        <v>JSA</v>
+      </c>
+      <c r="I348" t="str">
+        <v/>
+      </c>
+      <c r="J348" t="str">
+        <v/>
+      </c>
+      <c r="K348" t="str">
+        <v/>
+      </c>
+      <c r="L348" t="str">
+        <v/>
+      </c>
+      <c r="M348" t="str">
+        <v/>
+      </c>
+      <c r="N348" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N346"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N348"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualización cartas arrow team y enemigos
</commit_message>
<xml_diff>
--- a/public/resources/cartas.xlsx
+++ b/public/resources/cartas.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N348"/>
+  <dimension ref="A1:N356"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1698,7 +1698,7 @@
         <v>H</v>
       </c>
       <c r="H30" t="str">
-        <v/>
+        <v>The Terrifics</v>
       </c>
       <c r="I30" t="str">
         <v/>
@@ -2886,7 +2886,7 @@
         <v>H</v>
       </c>
       <c r="H57" t="str">
-        <v>JSA</v>
+        <v>JSA; The Terrifics</v>
       </c>
       <c r="I57" t="str">
         <v/>
@@ -5218,7 +5218,7 @@
         <v>H</v>
       </c>
       <c r="H110" t="str">
-        <v/>
+        <v>The Terrifics</v>
       </c>
       <c r="I110" t="str">
         <v/>
@@ -15711,9 +15711,361 @@
         <v/>
       </c>
     </row>
+    <row r="349">
+      <c r="A349" t="str">
+        <v>Phantom Girl IV</v>
+      </c>
+      <c r="B349">
+        <v>1</v>
+      </c>
+      <c r="C349">
+        <v>7200</v>
+      </c>
+      <c r="D349">
+        <v>4000</v>
+      </c>
+      <c r="E349" t="str">
+        <v>Meta</v>
+      </c>
+      <c r="F349" t="str">
+        <v>https://static.wikia.nocookie.net/marvel_dc/images/d/d9/Linnya_Wazzo_Prime_Earth_001.jpg/revision/latest?cb=20180305161820</v>
+      </c>
+      <c r="G349" t="str">
+        <v>H</v>
+      </c>
+      <c r="H349" t="str">
+        <v>The Terrifics</v>
+      </c>
+      <c r="I349" t="str">
+        <v/>
+      </c>
+      <c r="J349" t="str">
+        <v>Intangibilidad</v>
+      </c>
+      <c r="K349" t="str">
+        <v/>
+      </c>
+      <c r="L349" t="str">
+        <v>shield</v>
+      </c>
+      <c r="M349" t="str">
+        <v>Poder*0,5</v>
+      </c>
+      <c r="N349" t="str">
+        <v>usar</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="str">
+        <v>Nueva_carta_zhmo5</v>
+      </c>
+      <c r="B350">
+        <v>1</v>
+      </c>
+      <c r="C350">
+        <v>0</v>
+      </c>
+      <c r="D350">
+        <v>0</v>
+      </c>
+      <c r="E350" t="str">
+        <v/>
+      </c>
+      <c r="F350" t="str">
+        <v/>
+      </c>
+      <c r="G350" t="str">
+        <v/>
+      </c>
+      <c r="H350" t="str">
+        <v/>
+      </c>
+      <c r="I350" t="str">
+        <v/>
+      </c>
+      <c r="J350" t="str">
+        <v/>
+      </c>
+      <c r="K350" t="str">
+        <v/>
+      </c>
+      <c r="L350" t="str">
+        <v/>
+      </c>
+      <c r="M350" t="str">
+        <v/>
+      </c>
+      <c r="N350" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="str">
+        <v>Nueva_carta_zhqi6</v>
+      </c>
+      <c r="B351">
+        <v>1</v>
+      </c>
+      <c r="C351">
+        <v>0</v>
+      </c>
+      <c r="D351">
+        <v>0</v>
+      </c>
+      <c r="E351" t="str">
+        <v/>
+      </c>
+      <c r="F351" t="str">
+        <v/>
+      </c>
+      <c r="G351" t="str">
+        <v/>
+      </c>
+      <c r="H351" t="str">
+        <v/>
+      </c>
+      <c r="I351" t="str">
+        <v/>
+      </c>
+      <c r="J351" t="str">
+        <v/>
+      </c>
+      <c r="K351" t="str">
+        <v/>
+      </c>
+      <c r="L351" t="str">
+        <v/>
+      </c>
+      <c r="M351" t="str">
+        <v/>
+      </c>
+      <c r="N351" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="str">
+        <v>Merlyn</v>
+      </c>
+      <c r="B352">
+        <v>1</v>
+      </c>
+      <c r="C352">
+        <v>4500</v>
+      </c>
+      <c r="D352">
+        <v>3600</v>
+      </c>
+      <c r="E352" t="str">
+        <v>Tecnología</v>
+      </c>
+      <c r="F352" t="str">
+        <v>https://i.ibb.co/bgzN5Bjs/Meriln.jpg</v>
+      </c>
+      <c r="G352" t="str">
+        <v>V</v>
+      </c>
+      <c r="H352" t="str">
+        <v/>
+      </c>
+      <c r="I352" t="str">
+        <v/>
+      </c>
+      <c r="J352" t="str">
+        <v>Flechas oscuras</v>
+      </c>
+      <c r="K352" t="str">
+        <v/>
+      </c>
+      <c r="L352" t="str">
+        <v>stun</v>
+      </c>
+      <c r="M352" t="str">
+        <v>2</v>
+      </c>
+      <c r="N352" t="str">
+        <v>usar</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="str">
+        <v>Count Vertigo</v>
+      </c>
+      <c r="B353">
+        <v>1</v>
+      </c>
+      <c r="C353">
+        <v>4000</v>
+      </c>
+      <c r="D353">
+        <v>3800</v>
+      </c>
+      <c r="E353" t="str">
+        <v>Meta</v>
+      </c>
+      <c r="F353" t="str">
+        <v>https://i.ibb.co/b5S9cjGH/vertigo.jpg</v>
+      </c>
+      <c r="G353" t="str">
+        <v>V</v>
+      </c>
+      <c r="H353" t="str">
+        <v/>
+      </c>
+      <c r="I353" t="str">
+        <v/>
+      </c>
+      <c r="J353" t="str">
+        <v>Efecto vértigo</v>
+      </c>
+      <c r="K353" t="str">
+        <v/>
+      </c>
+      <c r="L353" t="str">
+        <v>bonus_debuff</v>
+      </c>
+      <c r="M353" t="str">
+        <v/>
+      </c>
+      <c r="N353" t="str">
+        <v>auto</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="str">
+        <v>Komodo</v>
+      </c>
+      <c r="B354">
+        <v>1</v>
+      </c>
+      <c r="C354">
+        <v>4600</v>
+      </c>
+      <c r="D354">
+        <v>3500</v>
+      </c>
+      <c r="E354" t="str">
+        <v>Tecnología</v>
+      </c>
+      <c r="F354" t="str">
+        <v>https://i.ibb.co/TypzxzD/Komodo.jpg</v>
+      </c>
+      <c r="G354" t="str">
+        <v>V</v>
+      </c>
+      <c r="H354" t="str">
+        <v/>
+      </c>
+      <c r="I354" t="str">
+        <v/>
+      </c>
+      <c r="J354" t="str">
+        <v xml:space="preserve">Traición </v>
+      </c>
+      <c r="K354" t="str">
+        <v/>
+      </c>
+      <c r="L354" t="str">
+        <v>aoe</v>
+      </c>
+      <c r="M354" t="str">
+        <v>Poder*0,5</v>
+      </c>
+      <c r="N354" t="str">
+        <v>usar</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="str">
+        <v>Brick</v>
+      </c>
+      <c r="B355">
+        <v>1</v>
+      </c>
+      <c r="C355">
+        <v>6000</v>
+      </c>
+      <c r="D355">
+        <v>4000</v>
+      </c>
+      <c r="E355" t="str">
+        <v>Meta</v>
+      </c>
+      <c r="F355" t="str">
+        <v>https://i.ibb.co/DPqRH0sh/Malo-De-Arrow.jpg</v>
+      </c>
+      <c r="G355" t="str">
+        <v>V</v>
+      </c>
+      <c r="H355" t="str">
+        <v/>
+      </c>
+      <c r="I355" t="str">
+        <v>https://i.ibb.co/jvbJPmtH/Malo-De-Arrow2.jpg</v>
+      </c>
+      <c r="J355" t="str">
+        <v>Invulnerabilidad</v>
+      </c>
+      <c r="K355" t="str">
+        <v/>
+      </c>
+      <c r="L355" t="str">
+        <v>tank</v>
+      </c>
+      <c r="M355" t="str">
+        <v>Salud*2</v>
+      </c>
+      <c r="N355" t="str">
+        <v>usar</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="str">
+        <v>Cupid</v>
+      </c>
+      <c r="B356">
+        <v>1</v>
+      </c>
+      <c r="C356">
+        <v>4000</v>
+      </c>
+      <c r="D356">
+        <v>3600</v>
+      </c>
+      <c r="E356" t="str">
+        <v>Meta</v>
+      </c>
+      <c r="F356" t="str">
+        <v>https://i.ibb.co/XxrhDG82/Quien-Sea-Esta-Pava.jpg</v>
+      </c>
+      <c r="G356" t="str">
+        <v>V</v>
+      </c>
+      <c r="H356" t="str">
+        <v/>
+      </c>
+      <c r="I356" t="str">
+        <v/>
+      </c>
+      <c r="J356" t="str">
+        <v>Amor enfermizo</v>
+      </c>
+      <c r="K356" t="str">
+        <v/>
+      </c>
+      <c r="L356" t="str">
+        <v>extra_attack</v>
+      </c>
+      <c r="M356" t="str">
+        <v>Poder*1</v>
+      </c>
+      <c r="N356" t="str">
+        <v>usar</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N348"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N356"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>